<commit_message>
annonces: 27 textes prets, rediges d'apres les intitules de facture
Fichier refait de bout en bout. Chaque annonce reprend la designation
exacte de la facture ADN — taille, modele, etat — et porte son cout
reel et sa marge.

Six sections : urgent saisonnier, boutique, Leboncoin/eBay, liquider,
prix a etablir, vendu.

Repartition de la livraison changee : 127,80 EUR / 79 articles physiques
= 1,6177 EUR par article, les lots comptant pour leur nombre de pieces.
Capital 1 875,15 EUR, CA 2 604 EUR, marge brute 897,20 EUR, net
724,13 EUR.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-stock.xlsx
+++ b/exports/maison-nsaia-stock.xlsx
@@ -140,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -189,7 +189,6 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -605,7 +604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Le coût réel inclut l'adjudication, les frais acheteur et la livraison répartie au prorata.</t>
+          <t>Coût réel = adjudication + frais acheteur + frais plateforme + livraison répartie par article.</t>
         </is>
       </c>
     </row>
@@ -731,18 +730,18 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Lot de 20 paires de sandales et tongs RELIFE / TOMMY JEANS — neuf</t>
+          <t>Lot de 2 paires ADIDAS Predator Edge P.48 2/3 — neuves</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>56.7</v>
+        <v>37.8</v>
       </c>
       <c r="C6" s="6">
-        <f>$B6*(1+Paramètres!$B$13)</f>
+        <f>$B6+$G6*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D6" s="7" t="n">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="E6" s="7">
         <f>IF($D6="","",$D6-$C6-$K6-$L6)</f>
@@ -753,7 +752,7 @@
         <v/>
       </c>
       <c r="G6" s="9" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H6" s="6">
         <f>$C6/$G6</f>
@@ -775,40 +774,40 @@
         <v>0</v>
       </c>
       <c r="M6" s="11" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>11.7</v>
+        <v>7.8</v>
       </c>
       <c r="O6" s="12" t="inlineStr">
         <is>
-          <t>ADN Lyon</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="P6" s="12" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="Q6" s="12" t="inlineStr">
         <is>
-          <t>FB2026-6354</t>
+          <t>FB2026-43716</t>
         </is>
       </c>
       <c r="R6" s="12" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>357</t>
         </is>
       </c>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin B2B</t>
+          <t>eBay + Leboncoin</t>
         </is>
       </c>
       <c r="T6" s="4" t="inlineStr"/>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>Février-mars</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="V6" s="4" t="inlineStr"/>
@@ -816,18 +815,18 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Lot de 2 paires ADIDAS Predator Edge P.48 2/3 — neuves</t>
+          <t>Lot de 20 paires de sandales et tongs RELIFE / TOMMY JEANS — neuf</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>37.8</v>
+        <v>56.7</v>
       </c>
       <c r="C7" s="6">
-        <f>$B7*(1+Paramètres!$B$13)</f>
+        <f>$B7+$G7*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D7" s="7" t="n">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="E7" s="7">
         <f>IF($D7="","",$D7-$C7-$K7-$L7)</f>
@@ -838,7 +837,7 @@
         <v/>
       </c>
       <c r="G7" s="9" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H7" s="6">
         <f>$C7/$G7</f>
@@ -860,40 +859,40 @@
         <v>0</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>7.8</v>
+        <v>11.7</v>
       </c>
       <c r="O7" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>FB2026-6354</t>
         </is>
       </c>
       <c r="R7" s="12" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>388</t>
         </is>
       </c>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t>eBay + Leboncoin</t>
+          <t>Leboncoin B2B</t>
         </is>
       </c>
       <c r="T7" s="4" t="inlineStr"/>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Février-mars</t>
         </is>
       </c>
       <c r="V7" s="4" t="inlineStr"/>
@@ -908,7 +907,7 @@
         <v>63</v>
       </c>
       <c r="C8" s="6">
-        <f>$B8*(1+Paramètres!$B$13)</f>
+        <f>$B8+$G8*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D8" s="7" t="n">
@@ -994,7 +993,7 @@
         <v>20.45</v>
       </c>
       <c r="C9" s="6">
-        <f>$B9*(1+Paramètres!$B$13)</f>
+        <f>$B9+$G9*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D9" s="7" t="n">
@@ -1073,18 +1072,18 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Pokémon MEGA Munikis Zero M3 — boîte de 30 boosters</t>
+          <t>Combinaison de pluie BMW Overall ProRain unisexe XL — neuve</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>65</v>
+        <v>68.56999999999999</v>
       </c>
       <c r="C10" s="6">
-        <f>$B10</f>
+        <f>$B10+$G10*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D10" s="7" t="n">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="E10" s="7">
         <f>IF($D10="","",$D10-$C10-$K10-$L10)</f>
@@ -1095,7 +1094,7 @@
         <v/>
       </c>
       <c r="G10" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H10" s="6">
         <f>$C10/$G10</f>
@@ -1116,31 +1115,35 @@
       <c r="L10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="M10" s="13" t="n"/>
-      <c r="N10" s="13" t="n"/>
+      <c r="M10" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="N10" s="11" t="n">
+        <v>8.57</v>
+      </c>
       <c r="O10" s="12" t="inlineStr">
         <is>
-          <t>Vendeur au Japon</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="P10" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="Q10" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FB2026-46060</t>
         </is>
       </c>
       <c r="R10" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1350</t>
         </is>
       </c>
       <c r="S10" s="4" t="inlineStr">
         <is>
-          <t>eBay + Leboncoin</t>
+          <t>Leboncoin + Vinted</t>
         </is>
       </c>
       <c r="T10" s="4" t="inlineStr"/>
@@ -1154,18 +1157,18 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Chaussures HOGAN P.36 — traces d'essayage</t>
+          <t>Pokémon MEGA Munikis Zero M3 — boîte de 30 boosters</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>12.6</v>
+        <v>65</v>
       </c>
       <c r="C11" s="6">
-        <f>$B11*(1+Paramètres!$B$13)</f>
+        <f>$B11</f>
         <v/>
       </c>
       <c r="D11" s="7" t="n">
-        <v>79</v>
+        <v>132</v>
       </c>
       <c r="E11" s="7">
         <f>IF($D11="","",$D11-$C11-$K11-$L11)</f>
@@ -1176,7 +1179,7 @@
         <v/>
       </c>
       <c r="G11" s="9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H11" s="6">
         <f>$C11/$G11</f>
@@ -1194,39 +1197,34 @@
         <f>IF($D11="","",$D11*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L11" s="6">
-        <f>IF($D11="","",$D11*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="M11" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="N11" s="11" t="n">
-        <v>2.6</v>
-      </c>
+      <c r="L11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="13" t="n"/>
+      <c r="N11" s="13" t="n"/>
       <c r="O11" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>Vendeur au Japon</t>
         </is>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Q11" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R11" s="12" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>—</t>
         </is>
       </c>
       <c r="S11" s="4" t="inlineStr">
         <is>
-          <t>Boutique</t>
+          <t>eBay + Leboncoin</t>
         </is>
       </c>
       <c r="T11" s="4" t="inlineStr"/>
@@ -1240,18 +1238,18 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Combinaison de pluie BMW Overall ProRain unisexe XL — neuve</t>
+          <t>Chaussures HOGAN P.36 — traces d'essayage</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>68.56999999999999</v>
+        <v>12.6</v>
       </c>
       <c r="C12" s="6">
-        <f>$B12*(1+Paramètres!$B$13)</f>
+        <f>$B12+$G12*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D12" s="7" t="n">
-        <v>139</v>
+        <v>79</v>
       </c>
       <c r="E12" s="7">
         <f>IF($D12="","",$D12-$C12-$K12-$L12)</f>
@@ -1280,14 +1278,15 @@
         <f>IF($D12="","",$D12*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L12" s="6" t="n">
-        <v>0</v>
+      <c r="L12" s="6">
+        <f>IF($D12="","",$D12*Paramètres!$B$7)</f>
+        <v/>
       </c>
       <c r="M12" s="11" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="N12" s="11" t="n">
-        <v>8.57</v>
+        <v>2.6</v>
       </c>
       <c r="O12" s="12" t="inlineStr">
         <is>
@@ -1296,22 +1295,22 @@
       </c>
       <c r="P12" s="12" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="Q12" s="12" t="inlineStr">
         <is>
-          <t>FB2026-46060</t>
+          <t>FB2026-43716</t>
         </is>
       </c>
       <c r="R12" s="12" t="inlineStr">
         <is>
-          <t>1350</t>
+          <t>191</t>
         </is>
       </c>
       <c r="S12" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + Vinted</t>
+          <t>Boutique</t>
         </is>
       </c>
       <c r="T12" s="4" t="inlineStr"/>
@@ -1332,7 +1331,7 @@
         <v>37.8</v>
       </c>
       <c r="C13" s="6">
-        <f>$B13*(1+Paramètres!$B$13)</f>
+        <f>$B13+$G13*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D13" s="7" t="n">
@@ -1411,18 +1410,18 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Lot de 6 vêtements femme MORGAN T.40 et L — neuf</t>
+          <t>Robe SANDRO T.40 — neuve</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
         <v>37.8</v>
       </c>
       <c r="C14" s="6">
-        <f>$B14*(1+Paramètres!$B$13)</f>
+        <f>$B14+$G14*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D14" s="7" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E14" s="7">
         <f>IF($D14="","",$D14-$C14-$K14-$L14)</f>
@@ -1433,7 +1432,7 @@
         <v/>
       </c>
       <c r="G14" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H14" s="6">
         <f>$C14/$G14</f>
@@ -1451,8 +1450,9 @@
         <f>IF($D14="","",$D14*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L14" s="6" t="n">
-        <v>0</v>
+      <c r="L14" s="6">
+        <f>IF($D14="","",$D14*Paramètres!$B$7)</f>
+        <v/>
       </c>
       <c r="M14" s="11" t="n">
         <v>30</v>
@@ -1467,22 +1467,22 @@
       </c>
       <c r="P14" s="12" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="Q14" s="12" t="inlineStr">
         <is>
-          <t>FB2026-46056</t>
+          <t>FB2026-43716</t>
         </is>
       </c>
       <c r="R14" s="12" t="inlineStr">
         <is>
-          <t>279</t>
+          <t>7</t>
         </is>
       </c>
       <c r="S14" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
+          <t>Boutique</t>
         </is>
       </c>
       <c r="T14" s="4" t="inlineStr"/>
@@ -1496,18 +1496,18 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Lot de 12 paires de tongs HAVAIANAS fuchsia 35/36 — neuf</t>
+          <t>Lot de 6 vêtements femme MORGAN T.40 et L — neuf</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>100.8</v>
+        <v>37.8</v>
       </c>
       <c r="C15" s="6">
-        <f>$B15*(1+Paramètres!$B$13)</f>
+        <f>$B15+$G15*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D15" s="7" t="n">
-        <v>159</v>
+        <v>92</v>
       </c>
       <c r="E15" s="7">
         <f>IF($D15="","",$D15-$C15-$K15-$L15)</f>
@@ -1518,7 +1518,7 @@
         <v/>
       </c>
       <c r="G15" s="9" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H15" s="6">
         <f>$C15/$G15</f>
@@ -1540,40 +1540,40 @@
         <v>0</v>
       </c>
       <c r="M15" s="11" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="N15" s="11" t="n">
-        <v>20.8</v>
+        <v>7.8</v>
       </c>
       <c r="O15" s="12" t="inlineStr">
         <is>
-          <t>ADN Lyon</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="Q15" s="12" t="inlineStr">
         <is>
-          <t>FB2026-5844</t>
+          <t>FB2026-46056</t>
         </is>
       </c>
       <c r="R15" s="12" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>279</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin, en lot</t>
+          <t>Leboncoin + eBay</t>
         </is>
       </c>
       <c r="T15" s="4" t="inlineStr"/>
       <c r="U15" s="4" t="inlineStr">
         <is>
-          <t>URGENT — saisonnier</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="V15" s="4" t="inlineStr"/>
@@ -1581,18 +1581,18 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Robe SANDRO T.40 — neuve</t>
+          <t>ADIDAS x STELLA McCARTNEY ASMC Ultraboost 21 P.36 — modèle d'exposition</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
         <v>37.8</v>
       </c>
       <c r="C16" s="6">
-        <f>$B16*(1+Paramètres!$B$13)</f>
+        <f>$B16+$G16*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D16" s="7" t="n">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="E16" s="7">
         <f>IF($D16="","",$D16-$C16-$K16-$L16)</f>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="R16" s="12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>434</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
@@ -1748,18 +1748,18 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>ADIDAS x STELLA McCARTNEY ASMC Ultraboost 21 P.36 — modèle d'exposition</t>
+          <t>Lot de 12 paires de tongs HAVAIANAS fuchsia 35/36 — neuf</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>37.8</v>
+        <v>100.8</v>
       </c>
       <c r="C18" s="6">
-        <f>$B18*(1+Paramètres!$B$13)</f>
+        <f>$B18+$G18*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D18" s="7" t="n">
-        <v>79</v>
+        <v>159</v>
       </c>
       <c r="E18" s="7">
         <f>IF($D18="","",$D18-$C18-$K18-$L18)</f>
@@ -1770,7 +1770,7 @@
         <v/>
       </c>
       <c r="G18" s="9" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H18" s="6">
         <f>$C18/$G18</f>
@@ -1788,19 +1788,18 @@
         <f>IF($D18="","",$D18*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L18" s="6">
-        <f>IF($D18="","",$D18*Paramètres!$B$7)</f>
-        <v/>
+      <c r="L18" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="M18" s="11" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="N18" s="11" t="n">
-        <v>7.8</v>
+        <v>20.8</v>
       </c>
       <c r="O18" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="P18" s="12" t="inlineStr">
@@ -1810,23 +1809,23 @@
       </c>
       <c r="Q18" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>FB2026-5844</t>
         </is>
       </c>
       <c r="R18" s="12" t="inlineStr">
         <is>
-          <t>434</t>
+          <t>120</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>Boutique</t>
+          <t>Leboncoin, en lot</t>
         </is>
       </c>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>URGENT — saisonnier</t>
         </is>
       </c>
       <c r="V18" s="4" t="inlineStr"/>
@@ -1834,18 +1833,18 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Lot de 4 gilets de flottaison MRS.ERTHA 3-6 ans — neuf</t>
+          <t>Blazer noir KARL LAGERFELD T.36 FR — neuf avec étiquette</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>37.8</v>
+        <v>50.4</v>
       </c>
       <c r="C19" s="6">
-        <f>$B19*(1+Paramètres!$B$13)</f>
+        <f>$B19+$G19*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D19" s="7" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="E19" s="7">
         <f>IF($D19="","",$D19-$C19-$K19-$L19)</f>
@@ -1856,7 +1855,7 @@
         <v/>
       </c>
       <c r="G19" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H19" s="6">
         <f>$C19/$G19</f>
@@ -1874,14 +1873,15 @@
         <f>IF($D19="","",$D19*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L19" s="6" t="n">
-        <v>0</v>
+      <c r="L19" s="6">
+        <f>IF($D19="","",$D19*Paramètres!$B$7)</f>
+        <v/>
       </c>
       <c r="M19" s="11" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="N19" s="11" t="n">
-        <v>7.8</v>
+        <v>10.4</v>
       </c>
       <c r="O19" s="12" t="inlineStr">
         <is>
@@ -1890,28 +1890,28 @@
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="Q19" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43717</t>
+          <t>FB2026-44194</t>
         </is>
       </c>
       <c r="R19" s="12" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>229</t>
         </is>
       </c>
       <c r="S19" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + Vinted</t>
+          <t>Boutique</t>
         </is>
       </c>
       <c r="T19" s="4" t="inlineStr"/>
       <c r="U19" s="4" t="inlineStr">
         <is>
-          <t>URGENT — saisonnier</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="V19" s="4" t="inlineStr"/>
@@ -1919,18 +1919,18 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Blazer noir KARL LAGERFELD T.36 FR — neuf avec étiquette</t>
+          <t>CHIARA FERRAGNI robe bustier courte T.M — neuve</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>50.4</v>
+        <v>31.95</v>
       </c>
       <c r="C20" s="6">
-        <f>$B20*(1+Paramètres!$B$13)</f>
+        <f>$B20+$G20*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D20" s="7" t="n">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="E20" s="7">
         <f>IF($D20="","",$D20-$C20-$K20-$L20)</f>
@@ -1964,14 +1964,14 @@
         <v/>
       </c>
       <c r="M20" s="11" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="N20" s="11" t="n">
-        <v>10.4</v>
+        <v>6.5</v>
       </c>
       <c r="O20" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="P20" s="12" t="inlineStr">
@@ -1981,17 +1981,17 @@
       </c>
       <c r="Q20" s="12" t="inlineStr">
         <is>
-          <t>FB2026-44194</t>
+          <t>FB2026-5996</t>
         </is>
       </c>
       <c r="R20" s="12" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>123</t>
         </is>
       </c>
       <c r="S20" s="4" t="inlineStr">
         <is>
-          <t>Boutique</t>
+          <t>Boutique + Leboncoin</t>
         </is>
       </c>
       <c r="T20" s="4" t="inlineStr"/>
@@ -2005,18 +2005,18 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>CHIARA FERRAGNI robe bustier courte T.M — neuve</t>
+          <t>Ballerines MASSIMO DUTTI P.41 — traces d'essayage</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>31.95</v>
+        <v>25.2</v>
       </c>
       <c r="C21" s="6">
-        <f>$B21*(1+Paramètres!$B$13)</f>
+        <f>$B21+$G21*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D21" s="7" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E21" s="7">
         <f>IF($D21="","",$D21-$C21-$K21-$L21)</f>
@@ -2045,39 +2045,38 @@
         <f>IF($D21="","",$D21*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L21" s="6">
-        <f>IF($D21="","",$D21*Paramètres!$B$7)</f>
-        <v/>
+      <c r="L21" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="M21" s="11" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="N21" s="11" t="n">
-        <v>6.5</v>
+        <v>5.2</v>
       </c>
       <c r="O21" s="12" t="inlineStr">
         <is>
-          <t>ADN Lyon</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="Q21" s="12" t="inlineStr">
         <is>
-          <t>FB2026-5996</t>
+          <t>FB2026-43716</t>
         </is>
       </c>
       <c r="R21" s="12" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>439</t>
         </is>
       </c>
       <c r="S21" s="4" t="inlineStr">
         <is>
-          <t>Boutique + Leboncoin</t>
+          <t>Leboncoin + eBay</t>
         </is>
       </c>
       <c r="T21" s="4" t="inlineStr"/>
@@ -2091,14 +2090,14 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Ballerines MASSIMO DUTTI P.41 — traces d'essayage</t>
+          <t>PIER ANTONIO GASPARI robe droite bleu marine T.42 — neuve</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>25.2</v>
+        <v>25.56</v>
       </c>
       <c r="C22" s="6">
-        <f>$B22*(1+Paramètres!$B$13)</f>
+        <f>$B22+$G22*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D22" s="7" t="n">
@@ -2131,8 +2130,9 @@
         <f>IF($D22="","",$D22*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L22" s="6" t="n">
-        <v>0</v>
+      <c r="L22" s="6">
+        <f>IF($D22="","",$D22*Paramètres!$B$7)</f>
+        <v/>
       </c>
       <c r="M22" s="11" t="n">
         <v>20</v>
@@ -2142,27 +2142,27 @@
       </c>
       <c r="O22" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="P22" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="Q22" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>FB2026-5996</t>
         </is>
       </c>
       <c r="R22" s="12" t="inlineStr">
         <is>
-          <t>439</t>
+          <t>29</t>
         </is>
       </c>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
+          <t>Boutique + Leboncoin</t>
         </is>
       </c>
       <c r="T22" s="4" t="inlineStr"/>
@@ -2176,18 +2176,18 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>PIER ANTONIO GASPARI robe droite bleu marine T.42 — neuve</t>
+          <t>Lot de 4 gilets de flottaison MRS.ERTHA 3-6 ans — neuf</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>25.56</v>
+        <v>37.8</v>
       </c>
       <c r="C23" s="6">
-        <f>$B23*(1+Paramètres!$B$13)</f>
+        <f>$B23+$G23*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D23" s="7" t="n">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="E23" s="7">
         <f>IF($D23="","",$D23-$C23-$K23-$L23)</f>
@@ -2198,7 +2198,7 @@
         <v/>
       </c>
       <c r="G23" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H23" s="6">
         <f>$C23/$G23</f>
@@ -2216,45 +2216,44 @@
         <f>IF($D23="","",$D23*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L23" s="6">
-        <f>IF($D23="","",$D23*Paramètres!$B$7)</f>
-        <v/>
+      <c r="L23" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="M23" s="11" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="N23" s="11" t="n">
-        <v>5.2</v>
+        <v>7.8</v>
       </c>
       <c r="O23" s="12" t="inlineStr">
         <is>
-          <t>ADN Lyon</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="Q23" s="12" t="inlineStr">
         <is>
-          <t>FB2026-5996</t>
+          <t>FB2026-43717</t>
         </is>
       </c>
       <c r="R23" s="12" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>303</t>
         </is>
       </c>
       <c r="S23" s="4" t="inlineStr">
         <is>
-          <t>Boutique + Leboncoin</t>
+          <t>Leboncoin + Vinted</t>
         </is>
       </c>
       <c r="T23" s="4" t="inlineStr"/>
       <c r="U23" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>URGENT — saisonnier</t>
         </is>
       </c>
       <c r="V23" s="4" t="inlineStr"/>
@@ -2269,7 +2268,7 @@
         <v>57.51</v>
       </c>
       <c r="C24" s="6">
-        <f>$B24*(1+Paramètres!$B$13)</f>
+        <f>$B24+$G24*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D24" s="7" t="n">
@@ -2354,7 +2353,7 @@
         <v>21.73</v>
       </c>
       <c r="C25" s="6">
-        <f>$B25*(1+Paramètres!$B$13)</f>
+        <f>$B25+$G25*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D25" s="7" t="n">
@@ -2439,7 +2438,7 @@
         <v>50.4</v>
       </c>
       <c r="C26" s="6">
-        <f>$B26*(1+Paramètres!$B$13)</f>
+        <f>$B26+$G26*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D26" s="7" t="n">
@@ -2525,7 +2524,7 @@
         <v>75.59999999999999</v>
       </c>
       <c r="C27" s="6">
-        <f>$B27*(1+Paramètres!$B$13)</f>
+        <f>$B27+$G27*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D27" s="7" t="n">
@@ -2610,7 +2609,7 @@
         <v>76.68000000000001</v>
       </c>
       <c r="C28" s="16">
-        <f>$B28*(1+Paramètres!$B$13)</f>
+        <f>$B28+$G28*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D28" s="17" t="n">
@@ -2699,7 +2698,7 @@
         <v>51.12</v>
       </c>
       <c r="C29" s="6">
-        <f>$B29*(1+Paramètres!$B$13)</f>
+        <f>$B29+$G29*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D29" s="7" t="n">
@@ -2784,7 +2783,7 @@
         <v>38.34</v>
       </c>
       <c r="C30" s="6">
-        <f>$B30*(1+Paramètres!$B$13)</f>
+        <f>$B30+$G30*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D30" s="7" t="n">
@@ -2869,7 +2868,7 @@
         <v>51.12</v>
       </c>
       <c r="C31" s="6">
-        <f>$B31*(1+Paramètres!$B$13)</f>
+        <f>$B31+$G31*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D31" s="7" t="n">
@@ -2954,7 +2953,7 @@
         <v>52.4</v>
       </c>
       <c r="C32" s="6">
-        <f>$B32*(1+Paramètres!$B$13)</f>
+        <f>$B32+$G32*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D32" s="7" t="n">
@@ -3039,7 +3038,7 @@
         <v>19.17</v>
       </c>
       <c r="C33" s="25">
-        <f>$B33*(1+Paramètres!$B$13)</f>
+        <f>$B33+$G33*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D33" s="26" t="n"/>
@@ -3122,7 +3121,7 @@
         <v>25.2</v>
       </c>
       <c r="C34" s="25">
-        <f>$B34*(1+Paramètres!$B$13)</f>
+        <f>$B34+$G34*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D34" s="26" t="n"/>
@@ -3206,7 +3205,7 @@
         <v>38.34</v>
       </c>
       <c r="C35" s="25">
-        <f>$B35*(1+Paramètres!$B$13)</f>
+        <f>$B35+$G35*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D35" s="26" t="n"/>
@@ -3289,7 +3288,7 @@
         <v>50.4</v>
       </c>
       <c r="C36" s="25">
-        <f>$B36*(1+Paramètres!$B$13)</f>
+        <f>$B36+$G36*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D36" s="26" t="n"/>
@@ -3372,7 +3371,7 @@
         <v>50.4</v>
       </c>
       <c r="C37" s="25">
-        <f>$B37*(1+Paramètres!$B$13)</f>
+        <f>$B37+$G37*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D37" s="26" t="n"/>
@@ -3456,7 +3455,7 @@
         <v>57.51</v>
       </c>
       <c r="C38" s="25">
-        <f>$B38*(1+Paramètres!$B$13)</f>
+        <f>$B38+$G38*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D38" s="26" t="n"/>
@@ -3539,7 +3538,7 @@
         <v>63</v>
       </c>
       <c r="C39" s="25">
-        <f>$B39*(1+Paramètres!$B$13)</f>
+        <f>$B39+$G39*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D39" s="26" t="n"/>
@@ -3622,7 +3621,7 @@
         <v>63</v>
       </c>
       <c r="C40" s="6">
-        <f>$B40*(1+Paramètres!$B$13)</f>
+        <f>$B40+$G40*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D40" s="13" t="n"/>
@@ -3705,7 +3704,7 @@
         <v>113.4</v>
       </c>
       <c r="C41" s="25">
-        <f>$B41*(1+Paramètres!$B$13)</f>
+        <f>$B41+$G41*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D41" s="26" t="n"/>
@@ -3876,9 +3875,8 @@
           <t>Marchandise ADN</t>
         </is>
       </c>
-      <c r="B4" s="6">
-        <f>Paramètres!B12</f>
-        <v/>
+      <c r="B4" s="6" t="n">
+        <v>1637.35</v>
       </c>
     </row>
     <row r="5">
@@ -4204,31 +4202,31 @@
     <row r="12">
       <c r="A12" s="39" t="inlineStr">
         <is>
-          <t>Total marchandise ADN</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>1637.35</v>
+          <t>Nombre d'articles physiques reçus d'ADN</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>79</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>34 lots</t>
+          <t>les lots comptent pour leur nombre de pièces</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="39" t="inlineStr">
         <is>
-          <t>Taux de livraison appliqué</t>
-        </is>
-      </c>
-      <c r="B13" s="46">
+          <t>Livraison par article</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
         <f>B11/B12</f>
         <v/>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Réparti au prorata du prix d'achat</t>
+          <t>réparti au nombre d'articles, pas au prix</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4290,7 @@
           <t>Nombre d'annonces prévues</t>
         </is>
       </c>
-      <c r="B21" s="47" t="n">
+      <c r="B21" s="46" t="n">
         <v>40</v>
       </c>
     </row>
@@ -5920,32 +5918,32 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="48" t="inlineStr">
+      <c r="A42" s="47" t="inlineStr">
         <is>
           <t>Facture</t>
         </is>
       </c>
-      <c r="B42" s="48" t="inlineStr">
+      <c r="B42" s="47" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C42" s="48" t="inlineStr">
+      <c r="C42" s="47" t="inlineStr">
         <is>
           <t>Maison</t>
         </is>
       </c>
-      <c r="D42" s="48" t="inlineStr">
+      <c r="D42" s="47" t="inlineStr">
         <is>
           <t>Commande</t>
         </is>
       </c>
-      <c r="E42" s="48" t="inlineStr">
+      <c r="E42" s="47" t="inlineStr">
         <is>
           <t>Désignation</t>
         </is>
       </c>
-      <c r="F42" s="48" t="inlineStr">
+      <c r="F42" s="47" t="inlineStr">
         <is>
           <t>Total TTC</t>
         </is>

</xml_diff>

<commit_message>
stock: livraison repartie par unite de vente et non par article
Un lot vendu en bloc compte pour un colis, pas pour son nombre de
pieces : les 12 Havaianas et les 20 sandales comptent chacun pour 1,
les 4 gilets Mrs.Ertha pour 4 et les 2 Predator pour 2 puisqu'ils
partent separement.

127,80 EUR / 43 unites de vente = 2,9721 EUR par unite.

Le lot de sandales passe de 85,27 a 114,65 EUR de marge, les Havaianas
de 19,07 a 35,51 EUR. Marge brute 899,68 EUR, net 719,87 EUR.

Colonne 'Unites de vente' ajoutee au tableau ; annonces.md mis a jour
avec les nouveaux couts et marges.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-stock.xlsx
+++ b/exports/maison-nsaia-stock.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Factures" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stock complet'!$A$5:$V$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stock complet'!$A$5:$W$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V42"/>
+  <dimension ref="A1:W42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -592,6 +592,7 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="20" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -604,7 +605,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Coût réel = adjudication + frais acheteur + frais plateforme + livraison répartie par article.</t>
+          <t>Coût réel = adjudication + frais acheteur + frais plateforme + livraison répartie par unité de vente.</t>
         </is>
       </c>
     </row>
@@ -726,22 +727,27 @@
           <t>Vendu le</t>
         </is>
       </c>
+      <c r="W5" s="3" t="inlineStr">
+        <is>
+          <t>Unités de vente</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Lot de 2 paires ADIDAS Predator Edge P.48 2/3 — neuves</t>
+          <t>Lot de 20 paires de sandales et tongs RELIFE / TOMMY JEANS — neuf</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>37.8</v>
+        <v>56.7</v>
       </c>
       <c r="C6" s="6">
-        <f>$B6+$G6*Paramètres!$B$13</f>
+        <f>$B6+$W6*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D6" s="7" t="n">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="E6" s="7">
         <f>IF($D6="","",$D6-$C6-$K6-$L6)</f>
@@ -752,7 +758,7 @@
         <v/>
       </c>
       <c r="G6" s="9" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="H6" s="6">
         <f>$C6/$G6</f>
@@ -774,59 +780,62 @@
         <v>0</v>
       </c>
       <c r="M6" s="11" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="N6" s="11" t="n">
-        <v>7.8</v>
+        <v>11.7</v>
       </c>
       <c r="O6" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="P6" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>11/08/2026</t>
         </is>
       </c>
       <c r="Q6" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>FB2026-6354</t>
         </is>
       </c>
       <c r="R6" s="12" t="inlineStr">
         <is>
-          <t>357</t>
+          <t>388</t>
         </is>
       </c>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>eBay + Leboncoin</t>
+          <t>Leboncoin B2B</t>
         </is>
       </c>
       <c r="T6" s="4" t="inlineStr"/>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Février-mars</t>
         </is>
       </c>
       <c r="V6" s="4" t="inlineStr"/>
+      <c r="W6" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Lot de 20 paires de sandales et tongs RELIFE / TOMMY JEANS — neuf</t>
+          <t>Lot de 2 paires ADIDAS Predator Edge P.48 2/3 — neuves</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>56.7</v>
+        <v>37.8</v>
       </c>
       <c r="C7" s="6">
-        <f>$B7+$G7*Paramètres!$B$13</f>
+        <f>$B7+$W7*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D7" s="7" t="n">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="E7" s="7">
         <f>IF($D7="","",$D7-$C7-$K7-$L7)</f>
@@ -837,7 +846,7 @@
         <v/>
       </c>
       <c r="G7" s="9" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H7" s="6">
         <f>$C7/$G7</f>
@@ -859,43 +868,46 @@
         <v>0</v>
       </c>
       <c r="M7" s="11" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="N7" s="11" t="n">
-        <v>11.7</v>
+        <v>7.8</v>
       </c>
       <c r="O7" s="12" t="inlineStr">
         <is>
-          <t>ADN Lyon</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
-          <t>11/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr">
         <is>
-          <t>FB2026-6354</t>
+          <t>FB2026-43716</t>
         </is>
       </c>
       <c r="R7" s="12" t="inlineStr">
         <is>
-          <t>388</t>
+          <t>357</t>
         </is>
       </c>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin B2B</t>
+          <t>eBay + Leboncoin</t>
         </is>
       </c>
       <c r="T7" s="4" t="inlineStr"/>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>Février-mars</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="V7" s="4" t="inlineStr"/>
+      <c r="W7" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -907,7 +919,7 @@
         <v>63</v>
       </c>
       <c r="C8" s="6">
-        <f>$B8+$G8*Paramètres!$B$13</f>
+        <f>$B8+$W8*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D8" s="7" t="n">
@@ -982,6 +994,9 @@
         </is>
       </c>
       <c r="V8" s="4" t="inlineStr"/>
+      <c r="W8" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -993,7 +1008,7 @@
         <v>20.45</v>
       </c>
       <c r="C9" s="6">
-        <f>$B9+$G9*Paramètres!$B$13</f>
+        <f>$B9+$W9*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D9" s="7" t="n">
@@ -1068,6 +1083,9 @@
         </is>
       </c>
       <c r="V9" s="4" t="inlineStr"/>
+      <c r="W9" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1079,7 +1097,7 @@
         <v>68.56999999999999</v>
       </c>
       <c r="C10" s="6">
-        <f>$B10+$G10*Paramètres!$B$13</f>
+        <f>$B10+$W10*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D10" s="7" t="n">
@@ -1153,6 +1171,9 @@
         </is>
       </c>
       <c r="V10" s="4" t="inlineStr"/>
+      <c r="W10" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1234,6 +1255,9 @@
         </is>
       </c>
       <c r="V11" s="4" t="inlineStr"/>
+      <c r="W11" s="4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1245,7 +1269,7 @@
         <v>12.6</v>
       </c>
       <c r="C12" s="6">
-        <f>$B12+$G12*Paramètres!$B$13</f>
+        <f>$B12+$W12*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D12" s="7" t="n">
@@ -1320,6 +1344,9 @@
         </is>
       </c>
       <c r="V12" s="4" t="inlineStr"/>
+      <c r="W12" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1331,7 +1358,7 @@
         <v>37.8</v>
       </c>
       <c r="C13" s="6">
-        <f>$B13+$G13*Paramètres!$B$13</f>
+        <f>$B13+$W13*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D13" s="7" t="n">
@@ -1406,22 +1433,25 @@
         </is>
       </c>
       <c r="V13" s="4" t="inlineStr"/>
+      <c r="W13" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Robe SANDRO T.40 — neuve</t>
+          <t>Lot de 12 paires de tongs HAVAIANAS fuchsia 35/36 — neuf</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>37.8</v>
+        <v>100.8</v>
       </c>
       <c r="C14" s="6">
-        <f>$B14+$G14*Paramètres!$B$13</f>
+        <f>$B14+$W14*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D14" s="7" t="n">
-        <v>89</v>
+        <v>159</v>
       </c>
       <c r="E14" s="7">
         <f>IF($D14="","",$D14-$C14-$K14-$L14)</f>
@@ -1432,7 +1462,7 @@
         <v/>
       </c>
       <c r="G14" s="9" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H14" s="6">
         <f>$C14/$G14</f>
@@ -1450,19 +1480,18 @@
         <f>IF($D14="","",$D14*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L14" s="6">
-        <f>IF($D14="","",$D14*Paramètres!$B$7)</f>
-        <v/>
+      <c r="L14" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="M14" s="11" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="N14" s="11" t="n">
-        <v>7.8</v>
+        <v>20.8</v>
       </c>
       <c r="O14" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="P14" s="12" t="inlineStr">
@@ -1472,42 +1501,45 @@
       </c>
       <c r="Q14" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>FB2026-5844</t>
         </is>
       </c>
       <c r="R14" s="12" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>120</t>
         </is>
       </c>
       <c r="S14" s="4" t="inlineStr">
         <is>
-          <t>Boutique</t>
+          <t>Leboncoin, en lot</t>
         </is>
       </c>
       <c r="T14" s="4" t="inlineStr"/>
       <c r="U14" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>URGENT — saisonnier</t>
         </is>
       </c>
       <c r="V14" s="4" t="inlineStr"/>
+      <c r="W14" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Lot de 6 vêtements femme MORGAN T.40 et L — neuf</t>
+          <t>Robe SANDRO T.40 — neuve</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
         <v>37.8</v>
       </c>
       <c r="C15" s="6">
-        <f>$B15+$G15*Paramètres!$B$13</f>
+        <f>$B15+$W15*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D15" s="7" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E15" s="7">
         <f>IF($D15="","",$D15-$C15-$K15-$L15)</f>
@@ -1518,7 +1550,7 @@
         <v/>
       </c>
       <c r="G15" s="9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H15" s="6">
         <f>$C15/$G15</f>
@@ -1536,8 +1568,9 @@
         <f>IF($D15="","",$D15*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L15" s="6" t="n">
-        <v>0</v>
+      <c r="L15" s="6">
+        <f>IF($D15="","",$D15*Paramètres!$B$7)</f>
+        <v/>
       </c>
       <c r="M15" s="11" t="n">
         <v>30</v>
@@ -1552,22 +1585,22 @@
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="Q15" s="12" t="inlineStr">
         <is>
-          <t>FB2026-46056</t>
+          <t>FB2026-43716</t>
         </is>
       </c>
       <c r="R15" s="12" t="inlineStr">
         <is>
-          <t>279</t>
+          <t>7</t>
         </is>
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
+          <t>Boutique</t>
         </is>
       </c>
       <c r="T15" s="4" t="inlineStr"/>
@@ -1577,22 +1610,25 @@
         </is>
       </c>
       <c r="V15" s="4" t="inlineStr"/>
+      <c r="W15" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>ADIDAS x STELLA McCARTNEY ASMC Ultraboost 21 P.36 — modèle d'exposition</t>
+          <t>Lot de 2 pompes immergées ROBBY VP550W</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>37.8</v>
+        <v>45</v>
       </c>
       <c r="C16" s="6">
-        <f>$B16+$G16*Paramètres!$B$13</f>
+        <f>$B16</f>
         <v/>
       </c>
       <c r="D16" s="7" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E16" s="7">
         <f>IF($D16="","",$D16-$C16-$K16-$L16)</f>
@@ -1603,7 +1639,7 @@
         <v/>
       </c>
       <c r="G16" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H16" s="6">
         <f>$C16/$G16</f>
@@ -1621,39 +1657,34 @@
         <f>IF($D16="","",$D16*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L16" s="6">
-        <f>IF($D16="","",$D16*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="M16" s="11" t="n">
-        <v>30</v>
-      </c>
-      <c r="N16" s="11" t="n">
-        <v>7.8</v>
-      </c>
+      <c r="L16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="13" t="n"/>
+      <c r="N16" s="13" t="n"/>
       <c r="O16" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN (facture à retrouver)</t>
         </is>
       </c>
       <c r="P16" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Q16" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R16" s="12" t="inlineStr">
         <is>
-          <t>434</t>
+          <t>84</t>
         </is>
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>Boutique</t>
+          <t>Leboncoin, main propre</t>
         </is>
       </c>
       <c r="T16" s="4" t="inlineStr"/>
@@ -1663,22 +1694,25 @@
         </is>
       </c>
       <c r="V16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Lot de 2 pompes immergées ROBBY VP550W</t>
+          <t>ADIDAS x STELLA McCARTNEY ASMC Ultraboost 21 P.36 — modèle d'exposition</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>45</v>
+        <v>37.8</v>
       </c>
       <c r="C17" s="6">
-        <f>$B17</f>
+        <f>$B17+$W17*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D17" s="7" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E17" s="7">
         <f>IF($D17="","",$D17-$C17-$K17-$L17)</f>
@@ -1689,7 +1723,7 @@
         <v/>
       </c>
       <c r="G17" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H17" s="6">
         <f>$C17/$G17</f>
@@ -1707,34 +1741,39 @@
         <f>IF($D17="","",$D17*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="L17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="13" t="n"/>
-      <c r="N17" s="13" t="n"/>
+      <c r="L17" s="6">
+        <f>IF($D17="","",$D17*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="M17" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="N17" s="11" t="n">
+        <v>7.8</v>
+      </c>
       <c r="O17" s="12" t="inlineStr">
         <is>
-          <t>ADN (facture à retrouver)</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="Q17" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>FB2026-43716</t>
         </is>
       </c>
       <c r="R17" s="12" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>434</t>
         </is>
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin, main propre</t>
+          <t>Boutique</t>
         </is>
       </c>
       <c r="T17" s="4" t="inlineStr"/>
@@ -1744,22 +1783,25 @@
         </is>
       </c>
       <c r="V17" s="4" t="inlineStr"/>
+      <c r="W17" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Lot de 12 paires de tongs HAVAIANAS fuchsia 35/36 — neuf</t>
+          <t>Lot de 6 vêtements femme MORGAN T.40 et L — neuf</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>100.8</v>
+        <v>37.8</v>
       </c>
       <c r="C18" s="6">
-        <f>$B18+$G18*Paramètres!$B$13</f>
+        <f>$B18+$W18*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D18" s="7" t="n">
-        <v>159</v>
+        <v>92</v>
       </c>
       <c r="E18" s="7">
         <f>IF($D18="","",$D18-$C18-$K18-$L18)</f>
@@ -1770,7 +1812,7 @@
         <v/>
       </c>
       <c r="G18" s="9" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H18" s="6">
         <f>$C18/$G18</f>
@@ -1792,43 +1834,46 @@
         <v>0</v>
       </c>
       <c r="M18" s="11" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="N18" s="11" t="n">
-        <v>20.8</v>
+        <v>7.8</v>
       </c>
       <c r="O18" s="12" t="inlineStr">
         <is>
-          <t>ADN Lyon</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="P18" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="Q18" s="12" t="inlineStr">
         <is>
-          <t>FB2026-5844</t>
+          <t>FB2026-46056</t>
         </is>
       </c>
       <c r="R18" s="12" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>279</t>
         </is>
       </c>
       <c r="S18" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin, en lot</t>
+          <t>Leboncoin + eBay</t>
         </is>
       </c>
       <c r="T18" s="4" t="inlineStr"/>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>URGENT — saisonnier</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="V18" s="4" t="inlineStr"/>
+      <c r="W18" s="4" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1840,7 +1885,7 @@
         <v>50.4</v>
       </c>
       <c r="C19" s="6">
-        <f>$B19+$G19*Paramètres!$B$13</f>
+        <f>$B19+$W19*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D19" s="7" t="n">
@@ -1915,6 +1960,9 @@
         </is>
       </c>
       <c r="V19" s="4" t="inlineStr"/>
+      <c r="W19" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1926,7 +1974,7 @@
         <v>31.95</v>
       </c>
       <c r="C20" s="6">
-        <f>$B20+$G20*Paramètres!$B$13</f>
+        <f>$B20+$W20*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D20" s="7" t="n">
@@ -2001,6 +2049,9 @@
         </is>
       </c>
       <c r="V20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -2012,7 +2063,7 @@
         <v>25.2</v>
       </c>
       <c r="C21" s="6">
-        <f>$B21+$G21*Paramètres!$B$13</f>
+        <f>$B21+$W21*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D21" s="7" t="n">
@@ -2086,6 +2137,9 @@
         </is>
       </c>
       <c r="V21" s="4" t="inlineStr"/>
+      <c r="W21" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2097,7 +2151,7 @@
         <v>25.56</v>
       </c>
       <c r="C22" s="6">
-        <f>$B22+$G22*Paramètres!$B$13</f>
+        <f>$B22+$W22*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D22" s="7" t="n">
@@ -2172,22 +2226,25 @@
         </is>
       </c>
       <c r="V22" s="4" t="inlineStr"/>
+      <c r="W22" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Lot de 4 gilets de flottaison MRS.ERTHA 3-6 ans — neuf</t>
+          <t>PHILIPP PLEIN SPORT baskets montantes P.40 — neuves</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>37.8</v>
+        <v>57.51</v>
       </c>
       <c r="C23" s="6">
-        <f>$B23+$G23*Paramètres!$B$13</f>
+        <f>$B23+$W23*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D23" s="7" t="n">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="E23" s="7">
         <f>IF($D23="","",$D23-$C23-$K23-$L23)</f>
@@ -2198,7 +2255,7 @@
         <v/>
       </c>
       <c r="G23" s="9" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H23" s="6">
         <f>$C23/$G23</f>
@@ -2220,59 +2277,62 @@
         <v>0</v>
       </c>
       <c r="M23" s="11" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="N23" s="11" t="n">
-        <v>7.8</v>
+        <v>11.7</v>
       </c>
       <c r="O23" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="Q23" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43717</t>
+          <t>FB2026-6023</t>
         </is>
       </c>
       <c r="R23" s="12" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>159</t>
         </is>
       </c>
       <c r="S23" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + Vinted</t>
+          <t>Leboncoin + eBay</t>
         </is>
       </c>
       <c r="T23" s="4" t="inlineStr"/>
       <c r="U23" s="4" t="inlineStr">
         <is>
-          <t>URGENT — saisonnier</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="V23" s="4" t="inlineStr"/>
+      <c r="W23" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>PHILIPP PLEIN SPORT baskets montantes P.40 — neuves</t>
+          <t>Lot de 4 gilets de flottaison MRS.ERTHA 3-6 ans — neuf</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>57.51</v>
+        <v>37.8</v>
       </c>
       <c r="C24" s="6">
-        <f>$B24+$G24*Paramètres!$B$13</f>
+        <f>$B24+$W24*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D24" s="7" t="n">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="E24" s="7">
         <f>IF($D24="","",$D24-$C24-$K24-$L24)</f>
@@ -2283,7 +2343,7 @@
         <v/>
       </c>
       <c r="G24" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H24" s="6">
         <f>$C24/$G24</f>
@@ -2305,43 +2365,46 @@
         <v>0</v>
       </c>
       <c r="M24" s="11" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="N24" s="11" t="n">
-        <v>11.7</v>
+        <v>7.8</v>
       </c>
       <c r="O24" s="12" t="inlineStr">
         <is>
-          <t>ADN Lyon</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="Q24" s="12" t="inlineStr">
         <is>
-          <t>FB2026-6023</t>
+          <t>FB2026-43717</t>
         </is>
       </c>
       <c r="R24" s="12" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>303</t>
         </is>
       </c>
       <c r="S24" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
+          <t>Leboncoin + Vinted</t>
         </is>
       </c>
       <c r="T24" s="4" t="inlineStr"/>
       <c r="U24" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>URGENT — saisonnier</t>
         </is>
       </c>
       <c r="V24" s="4" t="inlineStr"/>
+      <c r="W24" s="4" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2353,7 +2416,7 @@
         <v>21.73</v>
       </c>
       <c r="C25" s="6">
-        <f>$B25+$G25*Paramètres!$B$13</f>
+        <f>$B25+$W25*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D25" s="7" t="n">
@@ -2427,6 +2490,9 @@
         </is>
       </c>
       <c r="V25" s="4" t="inlineStr"/>
+      <c r="W25" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2438,7 +2504,7 @@
         <v>50.4</v>
       </c>
       <c r="C26" s="6">
-        <f>$B26+$G26*Paramètres!$B$13</f>
+        <f>$B26+$W26*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D26" s="7" t="n">
@@ -2513,6 +2579,9 @@
         </is>
       </c>
       <c r="V26" s="4" t="inlineStr"/>
+      <c r="W26" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2524,7 +2593,7 @@
         <v>75.59999999999999</v>
       </c>
       <c r="C27" s="6">
-        <f>$B27+$G27*Paramètres!$B$13</f>
+        <f>$B27+$W27*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D27" s="7" t="n">
@@ -2598,6 +2667,9 @@
         </is>
       </c>
       <c r="V27" s="4" t="inlineStr"/>
+      <c r="W27" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
@@ -2609,7 +2681,7 @@
         <v>76.68000000000001</v>
       </c>
       <c r="C28" s="16">
-        <f>$B28+$G28*Paramètres!$B$13</f>
+        <f>$B28+$W28*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D28" s="17" t="n">
@@ -2687,6 +2759,9 @@
           <t>12/08/2026</t>
         </is>
       </c>
+      <c r="W28" s="14" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2698,7 +2773,7 @@
         <v>51.12</v>
       </c>
       <c r="C29" s="6">
-        <f>$B29+$G29*Paramètres!$B$13</f>
+        <f>$B29+$W29*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D29" s="7" t="n">
@@ -2772,6 +2847,9 @@
         </is>
       </c>
       <c r="V29" s="4" t="inlineStr"/>
+      <c r="W29" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2783,7 +2861,7 @@
         <v>38.34</v>
       </c>
       <c r="C30" s="6">
-        <f>$B30+$G30*Paramètres!$B$13</f>
+        <f>$B30+$W30*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D30" s="7" t="n">
@@ -2857,6 +2935,9 @@
         </is>
       </c>
       <c r="V30" s="4" t="inlineStr"/>
+      <c r="W30" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2868,7 +2949,7 @@
         <v>51.12</v>
       </c>
       <c r="C31" s="6">
-        <f>$B31+$G31*Paramètres!$B$13</f>
+        <f>$B31+$W31*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D31" s="7" t="n">
@@ -2942,6 +3023,9 @@
         </is>
       </c>
       <c r="V31" s="4" t="inlineStr"/>
+      <c r="W31" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2953,7 +3037,7 @@
         <v>52.4</v>
       </c>
       <c r="C32" s="6">
-        <f>$B32+$G32*Paramètres!$B$13</f>
+        <f>$B32+$W32*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D32" s="7" t="n">
@@ -3027,6 +3111,9 @@
         </is>
       </c>
       <c r="V32" s="4" t="inlineStr"/>
+      <c r="W32" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="23" t="inlineStr">
@@ -3038,7 +3125,7 @@
         <v>19.17</v>
       </c>
       <c r="C33" s="25">
-        <f>$B33+$G33*Paramètres!$B$13</f>
+        <f>$B33+$W33*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D33" s="26" t="n"/>
@@ -3110,6 +3197,9 @@
         </is>
       </c>
       <c r="V33" s="23" t="inlineStr"/>
+      <c r="W33" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="23" t="inlineStr">
@@ -3121,7 +3211,7 @@
         <v>25.2</v>
       </c>
       <c r="C34" s="25">
-        <f>$B34+$G34*Paramètres!$B$13</f>
+        <f>$B34+$W34*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D34" s="26" t="n"/>
@@ -3194,6 +3284,9 @@
         </is>
       </c>
       <c r="V34" s="23" t="inlineStr"/>
+      <c r="W34" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="23" t="inlineStr">
@@ -3205,7 +3298,7 @@
         <v>38.34</v>
       </c>
       <c r="C35" s="25">
-        <f>$B35+$G35*Paramètres!$B$13</f>
+        <f>$B35+$W35*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D35" s="26" t="n"/>
@@ -3277,6 +3370,9 @@
         </is>
       </c>
       <c r="V35" s="23" t="inlineStr"/>
+      <c r="W35" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="23" t="inlineStr">
@@ -3288,7 +3384,7 @@
         <v>50.4</v>
       </c>
       <c r="C36" s="25">
-        <f>$B36+$G36*Paramètres!$B$13</f>
+        <f>$B36+$W36*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D36" s="26" t="n"/>
@@ -3360,6 +3456,9 @@
         </is>
       </c>
       <c r="V36" s="23" t="inlineStr"/>
+      <c r="W36" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="23" t="inlineStr">
@@ -3371,7 +3470,7 @@
         <v>50.4</v>
       </c>
       <c r="C37" s="25">
-        <f>$B37+$G37*Paramètres!$B$13</f>
+        <f>$B37+$W37*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D37" s="26" t="n"/>
@@ -3444,6 +3543,9 @@
         </is>
       </c>
       <c r="V37" s="23" t="inlineStr"/>
+      <c r="W37" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="23" t="inlineStr">
@@ -3455,7 +3557,7 @@
         <v>57.51</v>
       </c>
       <c r="C38" s="25">
-        <f>$B38+$G38*Paramètres!$B$13</f>
+        <f>$B38+$W38*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D38" s="26" t="n"/>
@@ -3527,6 +3629,9 @@
         </is>
       </c>
       <c r="V38" s="23" t="inlineStr"/>
+      <c r="W38" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
@@ -3538,7 +3643,7 @@
         <v>63</v>
       </c>
       <c r="C39" s="25">
-        <f>$B39+$G39*Paramètres!$B$13</f>
+        <f>$B39+$W39*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D39" s="26" t="n"/>
@@ -3610,6 +3715,9 @@
         </is>
       </c>
       <c r="V39" s="23" t="inlineStr"/>
+      <c r="W39" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -3621,7 +3729,7 @@
         <v>63</v>
       </c>
       <c r="C40" s="6">
-        <f>$B40+$G40*Paramètres!$B$13</f>
+        <f>$B40+$W40*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D40" s="13" t="n"/>
@@ -3693,6 +3801,9 @@
         </is>
       </c>
       <c r="V40" s="4" t="inlineStr"/>
+      <c r="W40" s="4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="23" t="inlineStr">
@@ -3704,7 +3815,7 @@
         <v>113.4</v>
       </c>
       <c r="C41" s="25">
-        <f>$B41+$G41*Paramètres!$B$13</f>
+        <f>$B41+$W41*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D41" s="26" t="n"/>
@@ -3777,6 +3888,9 @@
         </is>
       </c>
       <c r="V41" s="23" t="inlineStr"/>
+      <c r="W41" s="23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="33" t="inlineStr">
@@ -3829,9 +3943,10 @@
       <c r="T42" s="37" t="n"/>
       <c r="U42" s="37" t="n"/>
       <c r="V42" s="37" t="n"/>
+      <c r="W42" s="37" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:V41"/>
+  <autoFilter ref="A5:W41"/>
   <conditionalFormatting sqref="E6:E41">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>10</formula>
@@ -4202,22 +4317,22 @@
     <row r="12">
       <c r="A12" s="39" t="inlineStr">
         <is>
-          <t>Nombre d'articles physiques reçus d'ADN</t>
+          <t>Unités de vente reçues d'ADN</t>
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>79</v>
+        <v>43</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>les lots comptent pour leur nombre de pièces</t>
+          <t>un lot vendu en bloc compte pour 1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="39" t="inlineStr">
         <is>
-          <t>Livraison par article</t>
+          <t>Livraison par unité de vente</t>
         </is>
       </c>
       <c r="B13" s="6">
@@ -4226,7 +4341,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>réparti au nombre d'articles, pas au prix</t>
+          <t>réparti au nombre de colis à expédier</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
stock: colonne prix plancher pour la negociation et la famille
Prix plancher = seuil d'equilibre x 1,15, arrondi a l'euro superieur.
C'est le prix le plus bas acceptable, y compris pour la famille.
Coefficient reglable dans Parametres.

Cinq lots ont un plancher SUPERIEUR a leur prix de marche : NB GS 1906
(103 contre 99), Tommy Jeans (72 contre 65), NB montantes P.44 (71
contre 65), Emporio Armani (71 contre 69), NB P.38 (54 contre 54). Ils
ne peuvent pas etre vendus a 15 % de marge au prix du marche — c'est la
preuve definitive que le probleme est a l'achat, pas au prix.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-stock.xlsx
+++ b/exports/maison-nsaia-stock.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Factures" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stock complet'!$A$5:$X$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stock complet'!$A$5:$Y$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -140,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -191,6 +191,7 @@
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -568,33 +569,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X42"/>
+  <dimension ref="A1:Y42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="7" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="22" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
-    <col width="9" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="7" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="9" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -641,100 +643,105 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
+          <t>Prix plancher</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
           <t>PRIX DE VENTE</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Marge nette</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Rendement</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Nb</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Coût / art.</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Prix / art.</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Marge / art.</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>URSSAF</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>Carte</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="O5" s="3" t="inlineStr">
         <is>
           <t>Adjugé</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>Frais acheteur</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>Maison</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr">
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="R5" s="3" t="inlineStr">
+      <c r="S5" s="3" t="inlineStr">
         <is>
           <t>Facture</t>
         </is>
       </c>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="T5" s="3" t="inlineStr">
         <is>
           <t>Lot</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr">
+      <c r="U5" s="3" t="inlineStr">
         <is>
           <t>Canal</t>
         </is>
       </c>
-      <c r="U5" s="3" t="inlineStr">
+      <c r="V5" s="3" t="inlineStr">
         <is>
           <t>Statut</t>
         </is>
       </c>
-      <c r="V5" s="3" t="inlineStr">
+      <c r="W5" s="3" t="inlineStr">
         <is>
           <t>Priorité</t>
         </is>
       </c>
-      <c r="W5" s="3" t="inlineStr">
+      <c r="X5" s="3" t="inlineStr">
         <is>
           <t>Vendu le</t>
         </is>
       </c>
-      <c r="X5" s="3" t="inlineStr">
+      <c r="Y5" s="3" t="inlineStr">
         <is>
           <t>Unités de vente</t>
         </is>
@@ -750,85 +757,89 @@
         <v>56.7</v>
       </c>
       <c r="C6" s="6">
-        <f>$B6+$X6*Paramètres!$B$13</f>
+        <f>$B6+$Y6*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D6" s="7">
         <f>$C6/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="6">
+        <f>CEILING($D6*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F6" s="8" t="n">
         <v>199</v>
       </c>
-      <c r="F6" s="8">
-        <f>IF($E6="","",$E6-$C6-$L6-$M6)</f>
-        <v/>
-      </c>
-      <c r="G6" s="9">
-        <f>IF($F6="","",$F6/$C6)</f>
-        <v/>
-      </c>
-      <c r="H6" s="10" t="n">
+      <c r="G6" s="8">
+        <f>IF($F6="","",$F6-$C6-$M6-$N6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="9">
+        <f>IF($G6="","",$G6/$C6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="I6" s="6">
-        <f>$C6/$H6</f>
-        <v/>
-      </c>
       <c r="J6" s="6">
-        <f>IF($E6="","",$E6/$H6)</f>
+        <f>$C6/$I6</f>
         <v/>
       </c>
       <c r="K6" s="6">
-        <f>IF($F6="","",$F6/$H6)</f>
-        <v/>
-      </c>
-      <c r="L6" s="7">
-        <f>IF($E6="","",$E6*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M6" s="6" t="n">
+        <f>IF($F6="","",$F6/$I6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="6">
+        <f>IF($G6="","",$G6/$I6)</f>
+        <v/>
+      </c>
+      <c r="M6" s="7">
+        <f>IF($F6="","",$F6*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="11" t="n">
+      <c r="O6" s="11" t="n">
         <v>45</v>
       </c>
-      <c r="O6" s="11" t="n">
+      <c r="P6" s="11" t="n">
         <v>11.7</v>
       </c>
-      <c r="P6" s="12" t="inlineStr">
+      <c r="Q6" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q6" s="12" t="inlineStr">
+      <c r="R6" s="12" t="inlineStr">
         <is>
           <t>11/08/2026</t>
         </is>
       </c>
-      <c r="R6" s="12" t="inlineStr">
+      <c r="S6" s="12" t="inlineStr">
         <is>
           <t>FB2026-6354</t>
         </is>
       </c>
-      <c r="S6" s="12" t="inlineStr">
+      <c r="T6" s="12" t="inlineStr">
         <is>
           <t>388</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
+      <c r="U6" s="4" t="inlineStr">
         <is>
           <t>Leboncoin B2B</t>
         </is>
       </c>
-      <c r="U6" s="4" t="inlineStr"/>
-      <c r="V6" s="4" t="inlineStr">
+      <c r="V6" s="4" t="inlineStr"/>
+      <c r="W6" s="4" t="inlineStr">
         <is>
           <t>Février-mars</t>
         </is>
       </c>
-      <c r="W6" s="4" t="inlineStr"/>
-      <c r="X6" s="4" t="n">
+      <c r="X6" s="4" t="inlineStr"/>
+      <c r="Y6" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -842,85 +853,89 @@
         <v>37.8</v>
       </c>
       <c r="C7" s="6">
-        <f>$B7+$X7*Paramètres!$B$13</f>
+        <f>$B7+$Y7*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D7" s="7">
         <f>$C7/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="6">
+        <f>CEILING($D7*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F7" s="8" t="n">
         <v>178</v>
       </c>
-      <c r="F7" s="8">
-        <f>IF($E7="","",$E7-$C7-$L7-$M7)</f>
-        <v/>
-      </c>
-      <c r="G7" s="9">
-        <f>IF($F7="","",$F7/$C7)</f>
-        <v/>
-      </c>
-      <c r="H7" s="10" t="n">
+      <c r="G7" s="8">
+        <f>IF($F7="","",$F7-$C7-$M7-$N7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="9">
+        <f>IF($G7="","",$G7/$C7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="6">
-        <f>$C7/$H7</f>
-        <v/>
-      </c>
       <c r="J7" s="6">
-        <f>IF($E7="","",$E7/$H7)</f>
+        <f>$C7/$I7</f>
         <v/>
       </c>
       <c r="K7" s="6">
-        <f>IF($F7="","",$F7/$H7)</f>
-        <v/>
-      </c>
-      <c r="L7" s="7">
-        <f>IF($E7="","",$E7*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M7" s="6" t="n">
+        <f>IF($F7="","",$F7/$I7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="6">
+        <f>IF($G7="","",$G7/$I7)</f>
+        <v/>
+      </c>
+      <c r="M7" s="7">
+        <f>IF($F7="","",$F7*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N7" s="11" t="n">
+      <c r="O7" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="O7" s="11" t="n">
+      <c r="P7" s="11" t="n">
         <v>7.8</v>
       </c>
-      <c r="P7" s="12" t="inlineStr">
+      <c r="Q7" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q7" s="12" t="inlineStr">
+      <c r="R7" s="12" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R7" s="12" t="inlineStr">
+      <c r="S7" s="12" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S7" s="12" t="inlineStr">
+      <c r="T7" s="12" t="inlineStr">
         <is>
           <t>357</t>
         </is>
       </c>
-      <c r="T7" s="4" t="inlineStr">
+      <c r="U7" s="4" t="inlineStr">
         <is>
           <t>eBay + Leboncoin</t>
         </is>
       </c>
-      <c r="U7" s="4" t="inlineStr"/>
-      <c r="V7" s="4" t="inlineStr">
+      <c r="V7" s="4" t="inlineStr"/>
+      <c r="W7" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W7" s="4" t="inlineStr"/>
-      <c r="X7" s="4" t="n">
+      <c r="X7" s="4" t="inlineStr"/>
+      <c r="Y7" s="4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -934,86 +949,90 @@
         <v>63</v>
       </c>
       <c r="C8" s="6">
-        <f>$B8+$X8*Paramètres!$B$13</f>
+        <f>$B8+$Y8*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D8" s="7">
         <f>$C8/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="6">
+        <f>CEILING($D8*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F8" s="8" t="n">
         <v>159</v>
       </c>
-      <c r="F8" s="8">
-        <f>IF($E8="","",$E8-$C8-$L8-$M8)</f>
-        <v/>
-      </c>
-      <c r="G8" s="9">
-        <f>IF($F8="","",$F8/$C8)</f>
-        <v/>
-      </c>
-      <c r="H8" s="10" t="n">
+      <c r="G8" s="8">
+        <f>IF($F8="","",$F8-$C8-$M8-$N8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="9">
+        <f>IF($G8="","",$G8/$C8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="6">
-        <f>$C8/$H8</f>
-        <v/>
-      </c>
       <c r="J8" s="6">
-        <f>IF($E8="","",$E8/$H8)</f>
+        <f>$C8/$I8</f>
         <v/>
       </c>
       <c r="K8" s="6">
-        <f>IF($F8="","",$F8/$H8)</f>
-        <v/>
-      </c>
-      <c r="L8" s="7">
-        <f>IF($E8="","",$E8*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M8" s="6">
-        <f>IF($E8="","",$E8*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N8" s="11" t="n">
+        <f>IF($F8="","",$F8/$I8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="6">
+        <f>IF($G8="","",$G8/$I8)</f>
+        <v/>
+      </c>
+      <c r="M8" s="7">
+        <f>IF($F8="","",$F8*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N8" s="6">
+        <f>IF($F8="","",$F8*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O8" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="O8" s="11" t="n">
+      <c r="P8" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="P8" s="12" t="inlineStr">
+      <c r="Q8" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q8" s="12" t="inlineStr">
+      <c r="R8" s="12" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
-      <c r="R8" s="12" t="inlineStr">
+      <c r="S8" s="12" t="inlineStr">
         <is>
           <t>FB2026-46058</t>
         </is>
       </c>
-      <c r="S8" s="12" t="inlineStr">
+      <c r="T8" s="12" t="inlineStr">
         <is>
           <t>162</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
+      <c r="U8" s="4" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="U8" s="4" t="inlineStr"/>
-      <c r="V8" s="4" t="inlineStr">
+      <c r="V8" s="4" t="inlineStr"/>
+      <c r="W8" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W8" s="4" t="inlineStr"/>
-      <c r="X8" s="4" t="n">
+      <c r="X8" s="4" t="inlineStr"/>
+      <c r="Y8" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1027,86 +1046,90 @@
         <v>20.45</v>
       </c>
       <c r="C9" s="6">
-        <f>$B9+$X9*Paramètres!$B$13</f>
+        <f>$B9+$Y9*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D9" s="7">
         <f>$C9/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="6">
+        <f>CEILING($D9*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F9" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="F9" s="8">
-        <f>IF($E9="","",$E9-$C9-$L9-$M9)</f>
-        <v/>
-      </c>
-      <c r="G9" s="9">
-        <f>IF($F9="","",$F9/$C9)</f>
-        <v/>
-      </c>
-      <c r="H9" s="10" t="n">
+      <c r="G9" s="8">
+        <f>IF($F9="","",$F9-$C9-$M9-$N9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="9">
+        <f>IF($G9="","",$G9/$C9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="6">
-        <f>$C9/$H9</f>
-        <v/>
-      </c>
       <c r="J9" s="6">
-        <f>IF($E9="","",$E9/$H9)</f>
+        <f>$C9/$I9</f>
         <v/>
       </c>
       <c r="K9" s="6">
-        <f>IF($F9="","",$F9/$H9)</f>
-        <v/>
-      </c>
-      <c r="L9" s="7">
-        <f>IF($E9="","",$E9*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M9" s="6">
-        <f>IF($E9="","",$E9*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N9" s="11" t="n">
+        <f>IF($F9="","",$F9/$I9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="6">
+        <f>IF($G9="","",$G9/$I9)</f>
+        <v/>
+      </c>
+      <c r="M9" s="7">
+        <f>IF($F9="","",$F9*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N9" s="6">
+        <f>IF($F9="","",$F9*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O9" s="11" t="n">
         <v>16</v>
       </c>
-      <c r="O9" s="11" t="n">
+      <c r="P9" s="11" t="n">
         <v>4.16</v>
       </c>
-      <c r="P9" s="12" t="inlineStr">
+      <c r="Q9" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q9" s="12" t="inlineStr">
+      <c r="R9" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R9" s="12" t="inlineStr">
+      <c r="S9" s="12" t="inlineStr">
         <is>
           <t>FB2026-5996</t>
         </is>
       </c>
-      <c r="S9" s="12" t="inlineStr">
+      <c r="T9" s="12" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="T9" s="4" t="inlineStr">
+      <c r="U9" s="4" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="U9" s="4" t="inlineStr"/>
-      <c r="V9" s="4" t="inlineStr">
+      <c r="V9" s="4" t="inlineStr"/>
+      <c r="W9" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W9" s="4" t="inlineStr"/>
-      <c r="X9" s="4" t="n">
+      <c r="X9" s="4" t="inlineStr"/>
+      <c r="Y9" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1120,85 +1143,89 @@
         <v>68.56999999999999</v>
       </c>
       <c r="C10" s="6">
-        <f>$B10+$X10*Paramètres!$B$13</f>
+        <f>$B10+$Y10*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D10" s="7">
         <f>$C10/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="6">
+        <f>CEILING($D10*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F10" s="8" t="n">
         <v>139</v>
       </c>
-      <c r="F10" s="8">
-        <f>IF($E10="","",$E10-$C10-$L10-$M10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="9">
-        <f>IF($F10="","",$F10/$C10)</f>
-        <v/>
-      </c>
-      <c r="H10" s="10" t="n">
+      <c r="G10" s="8">
+        <f>IF($F10="","",$F10-$C10-$M10-$N10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="9">
+        <f>IF($G10="","",$G10/$C10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="6">
-        <f>$C10/$H10</f>
-        <v/>
-      </c>
       <c r="J10" s="6">
-        <f>IF($E10="","",$E10/$H10)</f>
+        <f>$C10/$I10</f>
         <v/>
       </c>
       <c r="K10" s="6">
-        <f>IF($F10="","",$F10/$H10)</f>
-        <v/>
-      </c>
-      <c r="L10" s="7">
-        <f>IF($E10="","",$E10*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M10" s="6" t="n">
+        <f>IF($F10="","",$F10/$I10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="6">
+        <f>IF($G10="","",$G10/$I10)</f>
+        <v/>
+      </c>
+      <c r="M10" s="7">
+        <f>IF($F10="","",$F10*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N10" s="11" t="n">
+      <c r="O10" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="O10" s="11" t="n">
+      <c r="P10" s="11" t="n">
         <v>8.57</v>
       </c>
-      <c r="P10" s="12" t="inlineStr">
+      <c r="Q10" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr">
+      <c r="R10" s="12" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
-      <c r="R10" s="12" t="inlineStr">
+      <c r="S10" s="12" t="inlineStr">
         <is>
           <t>FB2026-46060</t>
         </is>
       </c>
-      <c r="S10" s="12" t="inlineStr">
+      <c r="T10" s="12" t="inlineStr">
         <is>
           <t>1350</t>
         </is>
       </c>
-      <c r="T10" s="4" t="inlineStr">
+      <c r="U10" s="4" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="U10" s="4" t="inlineStr"/>
-      <c r="V10" s="4" t="inlineStr">
+      <c r="V10" s="4" t="inlineStr"/>
+      <c r="W10" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W10" s="4" t="inlineStr"/>
-      <c r="X10" s="4" t="n">
+      <c r="X10" s="4" t="inlineStr"/>
+      <c r="Y10" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1219,74 +1246,78 @@
         <f>$C11/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="6">
+        <f>CEILING($D11*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F11" s="8" t="n">
         <v>132</v>
       </c>
-      <c r="F11" s="8">
-        <f>IF($E11="","",$E11-$C11-$L11-$M11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="9">
-        <f>IF($F11="","",$F11/$C11)</f>
-        <v/>
-      </c>
-      <c r="H11" s="10" t="n">
+      <c r="G11" s="8">
+        <f>IF($F11="","",$F11-$C11-$M11-$N11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="9">
+        <f>IF($G11="","",$G11/$C11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="I11" s="6">
-        <f>$C11/$H11</f>
-        <v/>
-      </c>
       <c r="J11" s="6">
-        <f>IF($E11="","",$E11/$H11)</f>
+        <f>$C11/$I11</f>
         <v/>
       </c>
       <c r="K11" s="6">
-        <f>IF($F11="","",$F11/$H11)</f>
-        <v/>
-      </c>
-      <c r="L11" s="7">
-        <f>IF($E11="","",$E11*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M11" s="6" t="n">
+        <f>IF($F11="","",$F11/$I11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="6">
+        <f>IF($G11="","",$G11/$I11)</f>
+        <v/>
+      </c>
+      <c r="M11" s="7">
+        <f>IF($F11="","",$F11*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N11" s="13" t="n"/>
       <c r="O11" s="13" t="n"/>
-      <c r="P11" s="12" t="inlineStr">
+      <c r="P11" s="13" t="n"/>
+      <c r="Q11" s="12" t="inlineStr">
         <is>
           <t>Vendeur au Japon</t>
         </is>
       </c>
-      <c r="Q11" s="12" t="inlineStr">
+      <c r="R11" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="R11" s="12" t="inlineStr">
+      <c r="S11" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="S11" s="12" t="inlineStr">
+      <c r="T11" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="T11" s="4" t="inlineStr">
+      <c r="U11" s="4" t="inlineStr">
         <is>
           <t>eBay + Leboncoin</t>
         </is>
       </c>
-      <c r="U11" s="4" t="inlineStr"/>
-      <c r="V11" s="4" t="inlineStr">
+      <c r="V11" s="4" t="inlineStr"/>
+      <c r="W11" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W11" s="4" t="inlineStr"/>
-      <c r="X11" s="4" t="n">
+      <c r="X11" s="4" t="inlineStr"/>
+      <c r="Y11" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1300,86 +1331,90 @@
         <v>12.6</v>
       </c>
       <c r="C12" s="6">
-        <f>$B12+$X12*Paramètres!$B$13</f>
+        <f>$B12+$Y12*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D12" s="7">
         <f>$C12/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="6">
+        <f>CEILING($D12*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F12" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="F12" s="8">
-        <f>IF($E12="","",$E12-$C12-$L12-$M12)</f>
-        <v/>
-      </c>
-      <c r="G12" s="9">
-        <f>IF($F12="","",$F12/$C12)</f>
-        <v/>
-      </c>
-      <c r="H12" s="10" t="n">
+      <c r="G12" s="8">
+        <f>IF($F12="","",$F12-$C12-$M12-$N12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="9">
+        <f>IF($G12="","",$G12/$C12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="6">
-        <f>$C12/$H12</f>
-        <v/>
-      </c>
       <c r="J12" s="6">
-        <f>IF($E12="","",$E12/$H12)</f>
+        <f>$C12/$I12</f>
         <v/>
       </c>
       <c r="K12" s="6">
-        <f>IF($F12="","",$F12/$H12)</f>
-        <v/>
-      </c>
-      <c r="L12" s="7">
-        <f>IF($E12="","",$E12*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M12" s="6">
-        <f>IF($E12="","",$E12*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N12" s="11" t="n">
+        <f>IF($F12="","",$F12/$I12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="6">
+        <f>IF($G12="","",$G12/$I12)</f>
+        <v/>
+      </c>
+      <c r="M12" s="7">
+        <f>IF($F12="","",$F12*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N12" s="6">
+        <f>IF($F12="","",$F12*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O12" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="O12" s="11" t="n">
+      <c r="P12" s="11" t="n">
         <v>2.6</v>
       </c>
-      <c r="P12" s="12" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr">
+      <c r="R12" s="12" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R12" s="12" t="inlineStr">
+      <c r="S12" s="12" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S12" s="12" t="inlineStr">
+      <c r="T12" s="12" t="inlineStr">
         <is>
           <t>191</t>
         </is>
       </c>
-      <c r="T12" s="4" t="inlineStr">
+      <c r="U12" s="4" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="U12" s="4" t="inlineStr"/>
-      <c r="V12" s="4" t="inlineStr">
+      <c r="V12" s="4" t="inlineStr"/>
+      <c r="W12" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W12" s="4" t="inlineStr"/>
-      <c r="X12" s="4" t="n">
+      <c r="X12" s="4" t="inlineStr"/>
+      <c r="Y12" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1393,86 +1428,90 @@
         <v>37.8</v>
       </c>
       <c r="C13" s="6">
-        <f>$B13+$X13*Paramètres!$B$13</f>
+        <f>$B13+$Y13*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D13" s="7">
         <f>$C13/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="6">
+        <f>CEILING($D13*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F13" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="F13" s="8">
-        <f>IF($E13="","",$E13-$C13-$L13-$M13)</f>
-        <v/>
-      </c>
-      <c r="G13" s="9">
-        <f>IF($F13="","",$F13/$C13)</f>
-        <v/>
-      </c>
-      <c r="H13" s="10" t="n">
+      <c r="G13" s="8">
+        <f>IF($F13="","",$F13-$C13-$M13-$N13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="9">
+        <f>IF($G13="","",$G13/$C13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I13" s="6">
-        <f>$C13/$H13</f>
-        <v/>
-      </c>
       <c r="J13" s="6">
-        <f>IF($E13="","",$E13/$H13)</f>
+        <f>$C13/$I13</f>
         <v/>
       </c>
       <c r="K13" s="6">
-        <f>IF($F13="","",$F13/$H13)</f>
-        <v/>
-      </c>
-      <c r="L13" s="7">
-        <f>IF($E13="","",$E13*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M13" s="6">
-        <f>IF($E13="","",$E13*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N13" s="11" t="n">
+        <f>IF($F13="","",$F13/$I13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>IF($G13="","",$G13/$I13)</f>
+        <v/>
+      </c>
+      <c r="M13" s="7">
+        <f>IF($F13="","",$F13*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N13" s="6">
+        <f>IF($F13="","",$F13*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O13" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="O13" s="11" t="n">
+      <c r="P13" s="11" t="n">
         <v>7.8</v>
       </c>
-      <c r="P13" s="12" t="inlineStr">
+      <c r="Q13" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q13" s="12" t="inlineStr">
+      <c r="R13" s="12" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R13" s="12" t="inlineStr">
+      <c r="S13" s="12" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S13" s="12" t="inlineStr">
+      <c r="T13" s="12" t="inlineStr">
         <is>
           <t>417</t>
         </is>
       </c>
-      <c r="T13" s="4" t="inlineStr">
+      <c r="U13" s="4" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="U13" s="4" t="inlineStr"/>
-      <c r="V13" s="4" t="inlineStr">
+      <c r="V13" s="4" t="inlineStr"/>
+      <c r="W13" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W13" s="4" t="inlineStr"/>
-      <c r="X13" s="4" t="n">
+      <c r="X13" s="4" t="inlineStr"/>
+      <c r="Y13" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1486,86 +1525,90 @@
         <v>37.8</v>
       </c>
       <c r="C14" s="6">
-        <f>$B14+$X14*Paramètres!$B$13</f>
+        <f>$B14+$Y14*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D14" s="7">
         <f>$C14/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E14" s="8" t="n">
+      <c r="E14" s="6">
+        <f>CEILING($D14*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F14" s="8" t="n">
         <v>89</v>
       </c>
-      <c r="F14" s="8">
-        <f>IF($E14="","",$E14-$C14-$L14-$M14)</f>
-        <v/>
-      </c>
-      <c r="G14" s="9">
-        <f>IF($F14="","",$F14/$C14)</f>
-        <v/>
-      </c>
-      <c r="H14" s="10" t="n">
+      <c r="G14" s="8">
+        <f>IF($F14="","",$F14-$C14-$M14-$N14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="9">
+        <f>IF($G14="","",$G14/$C14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="6">
-        <f>$C14/$H14</f>
-        <v/>
-      </c>
       <c r="J14" s="6">
-        <f>IF($E14="","",$E14/$H14)</f>
+        <f>$C14/$I14</f>
         <v/>
       </c>
       <c r="K14" s="6">
-        <f>IF($F14="","",$F14/$H14)</f>
-        <v/>
-      </c>
-      <c r="L14" s="7">
-        <f>IF($E14="","",$E14*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M14" s="6">
-        <f>IF($E14="","",$E14*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N14" s="11" t="n">
+        <f>IF($F14="","",$F14/$I14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="6">
+        <f>IF($G14="","",$G14/$I14)</f>
+        <v/>
+      </c>
+      <c r="M14" s="7">
+        <f>IF($F14="","",$F14*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N14" s="6">
+        <f>IF($F14="","",$F14*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O14" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="O14" s="11" t="n">
+      <c r="P14" s="11" t="n">
         <v>7.8</v>
       </c>
-      <c r="P14" s="12" t="inlineStr">
+      <c r="Q14" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
+      <c r="R14" s="12" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R14" s="12" t="inlineStr">
+      <c r="S14" s="12" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S14" s="12" t="inlineStr">
+      <c r="T14" s="12" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="T14" s="4" t="inlineStr">
+      <c r="U14" s="4" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="U14" s="4" t="inlineStr"/>
-      <c r="V14" s="4" t="inlineStr">
+      <c r="V14" s="4" t="inlineStr"/>
+      <c r="W14" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W14" s="4" t="inlineStr"/>
-      <c r="X14" s="4" t="n">
+      <c r="X14" s="4" t="inlineStr"/>
+      <c r="Y14" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1579,85 +1622,89 @@
         <v>37.8</v>
       </c>
       <c r="C15" s="6">
-        <f>$B15+$X15*Paramètres!$B$13</f>
+        <f>$B15+$Y15*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D15" s="7">
         <f>$C15/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E15" s="8" t="n">
+      <c r="E15" s="6">
+        <f>CEILING($D15*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F15" s="8" t="n">
         <v>92</v>
       </c>
-      <c r="F15" s="8">
-        <f>IF($E15="","",$E15-$C15-$L15-$M15)</f>
-        <v/>
-      </c>
-      <c r="G15" s="9">
-        <f>IF($F15="","",$F15/$C15)</f>
-        <v/>
-      </c>
-      <c r="H15" s="10" t="n">
+      <c r="G15" s="8">
+        <f>IF($F15="","",$F15-$C15-$M15-$N15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="9">
+        <f>IF($G15="","",$G15/$C15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="I15" s="6">
-        <f>$C15/$H15</f>
-        <v/>
-      </c>
       <c r="J15" s="6">
-        <f>IF($E15="","",$E15/$H15)</f>
+        <f>$C15/$I15</f>
         <v/>
       </c>
       <c r="K15" s="6">
-        <f>IF($F15="","",$F15/$H15)</f>
-        <v/>
-      </c>
-      <c r="L15" s="7">
-        <f>IF($E15="","",$E15*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M15" s="6" t="n">
+        <f>IF($F15="","",$F15/$I15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="6">
+        <f>IF($G15="","",$G15/$I15)</f>
+        <v/>
+      </c>
+      <c r="M15" s="7">
+        <f>IF($F15="","",$F15*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N15" s="11" t="n">
+      <c r="O15" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="O15" s="11" t="n">
+      <c r="P15" s="11" t="n">
         <v>7.8</v>
       </c>
-      <c r="P15" s="12" t="inlineStr">
+      <c r="Q15" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q15" s="12" t="inlineStr">
+      <c r="R15" s="12" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
-      <c r="R15" s="12" t="inlineStr">
+      <c r="S15" s="12" t="inlineStr">
         <is>
           <t>FB2026-46056</t>
         </is>
       </c>
-      <c r="S15" s="12" t="inlineStr">
+      <c r="T15" s="12" t="inlineStr">
         <is>
           <t>279</t>
         </is>
       </c>
-      <c r="T15" s="4" t="inlineStr">
+      <c r="U15" s="4" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="U15" s="4" t="inlineStr"/>
-      <c r="V15" s="4" t="inlineStr">
+      <c r="V15" s="4" t="inlineStr"/>
+      <c r="W15" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W15" s="4" t="inlineStr"/>
-      <c r="X15" s="4" t="n">
+      <c r="X15" s="4" t="inlineStr"/>
+      <c r="Y15" s="4" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1678,74 +1725,78 @@
         <f>$C16/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="6">
+        <f>CEILING($D16*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F16" s="8" t="n">
         <v>84</v>
       </c>
-      <c r="F16" s="8">
-        <f>IF($E16="","",$E16-$C16-$L16-$M16)</f>
-        <v/>
-      </c>
-      <c r="G16" s="9">
-        <f>IF($F16="","",$F16/$C16)</f>
-        <v/>
-      </c>
-      <c r="H16" s="10" t="n">
+      <c r="G16" s="8">
+        <f>IF($F16="","",$F16-$C16-$M16-$N16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="9">
+        <f>IF($G16="","",$G16/$C16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="I16" s="6">
-        <f>$C16/$H16</f>
-        <v/>
-      </c>
       <c r="J16" s="6">
-        <f>IF($E16="","",$E16/$H16)</f>
+        <f>$C16/$I16</f>
         <v/>
       </c>
       <c r="K16" s="6">
-        <f>IF($F16="","",$F16/$H16)</f>
-        <v/>
-      </c>
-      <c r="L16" s="7">
-        <f>IF($E16="","",$E16*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M16" s="6" t="n">
+        <f>IF($F16="","",$F16/$I16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="6">
+        <f>IF($G16="","",$G16/$I16)</f>
+        <v/>
+      </c>
+      <c r="M16" s="7">
+        <f>IF($F16="","",$F16*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N16" s="13" t="n"/>
       <c r="O16" s="13" t="n"/>
-      <c r="P16" s="12" t="inlineStr">
+      <c r="P16" s="13" t="n"/>
+      <c r="Q16" s="12" t="inlineStr">
         <is>
           <t>ADN (facture à retrouver)</t>
         </is>
       </c>
-      <c r="Q16" s="12" t="inlineStr">
+      <c r="R16" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="R16" s="12" t="inlineStr">
+      <c r="S16" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="S16" s="12" t="inlineStr">
+      <c r="T16" s="12" t="inlineStr">
         <is>
           <t>84</t>
         </is>
       </c>
-      <c r="T16" s="4" t="inlineStr">
+      <c r="U16" s="4" t="inlineStr">
         <is>
           <t>Leboncoin, main propre</t>
         </is>
       </c>
-      <c r="U16" s="4" t="inlineStr"/>
-      <c r="V16" s="4" t="inlineStr">
+      <c r="V16" s="4" t="inlineStr"/>
+      <c r="W16" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W16" s="4" t="inlineStr"/>
-      <c r="X16" s="4" t="n">
+      <c r="X16" s="4" t="inlineStr"/>
+      <c r="Y16" s="4" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1759,86 +1810,90 @@
         <v>37.8</v>
       </c>
       <c r="C17" s="6">
-        <f>$B17+$X17*Paramètres!$B$13</f>
+        <f>$B17+$Y17*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D17" s="7">
         <f>$C17/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E17" s="8" t="n">
+      <c r="E17" s="6">
+        <f>CEILING($D17*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F17" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="F17" s="8">
-        <f>IF($E17="","",$E17-$C17-$L17-$M17)</f>
-        <v/>
-      </c>
-      <c r="G17" s="9">
-        <f>IF($F17="","",$F17/$C17)</f>
-        <v/>
-      </c>
-      <c r="H17" s="10" t="n">
+      <c r="G17" s="8">
+        <f>IF($F17="","",$F17-$C17-$M17-$N17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="9">
+        <f>IF($G17="","",$G17/$C17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="6">
-        <f>$C17/$H17</f>
-        <v/>
-      </c>
       <c r="J17" s="6">
-        <f>IF($E17="","",$E17/$H17)</f>
+        <f>$C17/$I17</f>
         <v/>
       </c>
       <c r="K17" s="6">
-        <f>IF($F17="","",$F17/$H17)</f>
-        <v/>
-      </c>
-      <c r="L17" s="7">
-        <f>IF($E17="","",$E17*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M17" s="6">
-        <f>IF($E17="","",$E17*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N17" s="11" t="n">
+        <f>IF($F17="","",$F17/$I17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="6">
+        <f>IF($G17="","",$G17/$I17)</f>
+        <v/>
+      </c>
+      <c r="M17" s="7">
+        <f>IF($F17="","",$F17*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N17" s="6">
+        <f>IF($F17="","",$F17*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O17" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="O17" s="11" t="n">
+      <c r="P17" s="11" t="n">
         <v>7.8</v>
       </c>
-      <c r="P17" s="12" t="inlineStr">
+      <c r="Q17" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q17" s="12" t="inlineStr">
+      <c r="R17" s="12" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R17" s="12" t="inlineStr">
+      <c r="S17" s="12" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S17" s="12" t="inlineStr">
+      <c r="T17" s="12" t="inlineStr">
         <is>
           <t>434</t>
         </is>
       </c>
-      <c r="T17" s="4" t="inlineStr">
+      <c r="U17" s="4" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="U17" s="4" t="inlineStr"/>
-      <c r="V17" s="4" t="inlineStr">
+      <c r="V17" s="4" t="inlineStr"/>
+      <c r="W17" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W17" s="4" t="inlineStr"/>
-      <c r="X17" s="4" t="n">
+      <c r="X17" s="4" t="inlineStr"/>
+      <c r="Y17" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1852,89 +1907,93 @@
         <v>100.8</v>
       </c>
       <c r="C18" s="16">
-        <f>$B18+$X18*Paramètres!$B$13</f>
+        <f>$B18+$Y18*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D18" s="17">
         <f>$C18/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="16">
+        <f>CEILING($D18*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F18" s="18" t="n">
         <v>168</v>
       </c>
-      <c r="F18" s="18">
-        <f>IF($E18="","",$E18-$C18-$L18-$M18)</f>
-        <v/>
-      </c>
-      <c r="G18" s="19">
-        <f>IF($F18="","",$F18/$C18)</f>
-        <v/>
-      </c>
-      <c r="H18" s="20" t="n">
+      <c r="G18" s="18">
+        <f>IF($F18="","",$F18-$C18-$M18-$N18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="19">
+        <f>IF($G18="","",$G18/$C18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="I18" s="16">
-        <f>$C18/$H18</f>
-        <v/>
-      </c>
       <c r="J18" s="16">
-        <f>IF($E18="","",$E18/$H18)</f>
+        <f>$C18/$I18</f>
         <v/>
       </c>
       <c r="K18" s="16">
-        <f>IF($F18="","",$F18/$H18)</f>
-        <v/>
-      </c>
-      <c r="L18" s="17">
-        <f>IF($E18="","",$E18*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M18" s="16" t="n">
+        <f>IF($F18="","",$F18/$I18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="16">
+        <f>IF($G18="","",$G18/$I18)</f>
+        <v/>
+      </c>
+      <c r="M18" s="17">
+        <f>IF($F18="","",$F18*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N18" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="N18" s="21" t="n">
+      <c r="O18" s="21" t="n">
         <v>80</v>
       </c>
-      <c r="O18" s="21" t="n">
+      <c r="P18" s="21" t="n">
         <v>20.8</v>
       </c>
-      <c r="P18" s="22" t="inlineStr">
+      <c r="Q18" s="22" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q18" s="22" t="inlineStr">
+      <c r="R18" s="22" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R18" s="22" t="inlineStr">
+      <c r="S18" s="22" t="inlineStr">
         <is>
           <t>FB2026-5844</t>
         </is>
       </c>
-      <c r="S18" s="22" t="inlineStr">
+      <c r="T18" s="22" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
-      <c r="T18" s="14" t="inlineStr">
+      <c r="U18" s="14" t="inlineStr">
         <is>
           <t>Leboncoin, à l'unité</t>
         </is>
       </c>
-      <c r="U18" s="14" t="inlineStr"/>
-      <c r="V18" s="14" t="inlineStr">
+      <c r="V18" s="14" t="inlineStr"/>
+      <c r="W18" s="14" t="inlineStr">
         <is>
           <t>URGENT — 2 sur 12 vendues</t>
         </is>
       </c>
-      <c r="W18" s="14" t="inlineStr">
+      <c r="X18" s="14" t="inlineStr">
         <is>
           <t>2 vendues</t>
         </is>
       </c>
-      <c r="X18" s="14" t="n">
+      <c r="Y18" s="14" t="n">
         <v>12</v>
       </c>
     </row>
@@ -1948,86 +2007,90 @@
         <v>50.4</v>
       </c>
       <c r="C19" s="6">
-        <f>$B19+$X19*Paramètres!$B$13</f>
+        <f>$B19+$Y19*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D19" s="7">
         <f>$C19/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E19" s="8" t="n">
+      <c r="E19" s="6">
+        <f>CEILING($D19*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F19" s="8" t="n">
         <v>89</v>
       </c>
-      <c r="F19" s="8">
-        <f>IF($E19="","",$E19-$C19-$L19-$M19)</f>
-        <v/>
-      </c>
-      <c r="G19" s="9">
-        <f>IF($F19="","",$F19/$C19)</f>
-        <v/>
-      </c>
-      <c r="H19" s="10" t="n">
+      <c r="G19" s="8">
+        <f>IF($F19="","",$F19-$C19-$M19-$N19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="9">
+        <f>IF($G19="","",$G19/$C19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I19" s="6">
-        <f>$C19/$H19</f>
-        <v/>
-      </c>
       <c r="J19" s="6">
-        <f>IF($E19="","",$E19/$H19)</f>
+        <f>$C19/$I19</f>
         <v/>
       </c>
       <c r="K19" s="6">
-        <f>IF($F19="","",$F19/$H19)</f>
-        <v/>
-      </c>
-      <c r="L19" s="7">
-        <f>IF($E19="","",$E19*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M19" s="6">
-        <f>IF($E19="","",$E19*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N19" s="11" t="n">
+        <f>IF($F19="","",$F19/$I19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="6">
+        <f>IF($G19="","",$G19/$I19)</f>
+        <v/>
+      </c>
+      <c r="M19" s="7">
+        <f>IF($F19="","",$F19*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N19" s="6">
+        <f>IF($F19="","",$F19*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O19" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="O19" s="11" t="n">
+      <c r="P19" s="11" t="n">
         <v>10.4</v>
       </c>
-      <c r="P19" s="12" t="inlineStr">
+      <c r="Q19" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
+      <c r="R19" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R19" s="12" t="inlineStr">
+      <c r="S19" s="12" t="inlineStr">
         <is>
           <t>FB2026-44194</t>
         </is>
       </c>
-      <c r="S19" s="12" t="inlineStr">
+      <c r="T19" s="12" t="inlineStr">
         <is>
           <t>229</t>
         </is>
       </c>
-      <c r="T19" s="4" t="inlineStr">
+      <c r="U19" s="4" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="U19" s="4" t="inlineStr"/>
-      <c r="V19" s="4" t="inlineStr">
+      <c r="V19" s="4" t="inlineStr"/>
+      <c r="W19" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W19" s="4" t="inlineStr"/>
-      <c r="X19" s="4" t="n">
+      <c r="X19" s="4" t="inlineStr"/>
+      <c r="Y19" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2041,86 +2104,90 @@
         <v>31.95</v>
       </c>
       <c r="C20" s="6">
-        <f>$B20+$X20*Paramètres!$B$13</f>
+        <f>$B20+$Y20*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D20" s="7">
         <f>$C20/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E20" s="8" t="n">
+      <c r="E20" s="6">
+        <f>CEILING($D20*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F20" s="8" t="n">
         <v>69</v>
       </c>
-      <c r="F20" s="8">
-        <f>IF($E20="","",$E20-$C20-$L20-$M20)</f>
-        <v/>
-      </c>
-      <c r="G20" s="9">
-        <f>IF($F20="","",$F20/$C20)</f>
-        <v/>
-      </c>
-      <c r="H20" s="10" t="n">
+      <c r="G20" s="8">
+        <f>IF($F20="","",$F20-$C20-$M20-$N20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="9">
+        <f>IF($G20="","",$G20/$C20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="6">
-        <f>$C20/$H20</f>
-        <v/>
-      </c>
       <c r="J20" s="6">
-        <f>IF($E20="","",$E20/$H20)</f>
+        <f>$C20/$I20</f>
         <v/>
       </c>
       <c r="K20" s="6">
-        <f>IF($F20="","",$F20/$H20)</f>
-        <v/>
-      </c>
-      <c r="L20" s="7">
-        <f>IF($E20="","",$E20*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M20" s="6">
-        <f>IF($E20="","",$E20*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N20" s="11" t="n">
+        <f>IF($F20="","",$F20/$I20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="6">
+        <f>IF($G20="","",$G20/$I20)</f>
+        <v/>
+      </c>
+      <c r="M20" s="7">
+        <f>IF($F20="","",$F20*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N20" s="6">
+        <f>IF($F20="","",$F20*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O20" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="O20" s="11" t="n">
+      <c r="P20" s="11" t="n">
         <v>6.5</v>
       </c>
-      <c r="P20" s="12" t="inlineStr">
+      <c r="Q20" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q20" s="12" t="inlineStr">
+      <c r="R20" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R20" s="12" t="inlineStr">
+      <c r="S20" s="12" t="inlineStr">
         <is>
           <t>FB2026-5996</t>
         </is>
       </c>
-      <c r="S20" s="12" t="inlineStr">
+      <c r="T20" s="12" t="inlineStr">
         <is>
           <t>123</t>
         </is>
       </c>
-      <c r="T20" s="4" t="inlineStr">
+      <c r="U20" s="4" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="U20" s="4" t="inlineStr"/>
-      <c r="V20" s="4" t="inlineStr">
+      <c r="V20" s="4" t="inlineStr"/>
+      <c r="W20" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W20" s="4" t="inlineStr"/>
-      <c r="X20" s="4" t="n">
+      <c r="X20" s="4" t="inlineStr"/>
+      <c r="Y20" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2134,85 +2201,89 @@
         <v>25.2</v>
       </c>
       <c r="C21" s="6">
-        <f>$B21+$X21*Paramètres!$B$13</f>
+        <f>$B21+$Y21*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D21" s="7">
         <f>$C21/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E21" s="6">
+        <f>CEILING($D21*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F21" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="F21" s="8">
-        <f>IF($E21="","",$E21-$C21-$L21-$M21)</f>
-        <v/>
-      </c>
-      <c r="G21" s="9">
-        <f>IF($F21="","",$F21/$C21)</f>
-        <v/>
-      </c>
-      <c r="H21" s="10" t="n">
+      <c r="G21" s="8">
+        <f>IF($F21="","",$F21-$C21-$M21-$N21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="9">
+        <f>IF($G21="","",$G21/$C21)</f>
+        <v/>
+      </c>
+      <c r="I21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I21" s="6">
-        <f>$C21/$H21</f>
-        <v/>
-      </c>
       <c r="J21" s="6">
-        <f>IF($E21="","",$E21/$H21)</f>
+        <f>$C21/$I21</f>
         <v/>
       </c>
       <c r="K21" s="6">
-        <f>IF($F21="","",$F21/$H21)</f>
-        <v/>
-      </c>
-      <c r="L21" s="7">
-        <f>IF($E21="","",$E21*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M21" s="6" t="n">
+        <f>IF($F21="","",$F21/$I21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="6">
+        <f>IF($G21="","",$G21/$I21)</f>
+        <v/>
+      </c>
+      <c r="M21" s="7">
+        <f>IF($F21="","",$F21*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N21" s="11" t="n">
+      <c r="O21" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="O21" s="11" t="n">
+      <c r="P21" s="11" t="n">
         <v>5.2</v>
       </c>
-      <c r="P21" s="12" t="inlineStr">
+      <c r="Q21" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q21" s="12" t="inlineStr">
+      <c r="R21" s="12" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R21" s="12" t="inlineStr">
+      <c r="S21" s="12" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S21" s="12" t="inlineStr">
+      <c r="T21" s="12" t="inlineStr">
         <is>
           <t>439</t>
         </is>
       </c>
-      <c r="T21" s="4" t="inlineStr">
+      <c r="U21" s="4" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="U21" s="4" t="inlineStr"/>
-      <c r="V21" s="4" t="inlineStr">
+      <c r="V21" s="4" t="inlineStr"/>
+      <c r="W21" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W21" s="4" t="inlineStr"/>
-      <c r="X21" s="4" t="n">
+      <c r="X21" s="4" t="inlineStr"/>
+      <c r="Y21" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2226,86 +2297,90 @@
         <v>25.56</v>
       </c>
       <c r="C22" s="6">
-        <f>$B22+$X22*Paramètres!$B$13</f>
+        <f>$B22+$Y22*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D22" s="7">
         <f>$C22/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E22" s="8" t="n">
+      <c r="E22" s="6">
+        <f>CEILING($D22*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F22" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="F22" s="8">
-        <f>IF($E22="","",$E22-$C22-$L22-$M22)</f>
-        <v/>
-      </c>
-      <c r="G22" s="9">
-        <f>IF($F22="","",$F22/$C22)</f>
-        <v/>
-      </c>
-      <c r="H22" s="10" t="n">
+      <c r="G22" s="8">
+        <f>IF($F22="","",$F22-$C22-$M22-$N22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="9">
+        <f>IF($G22="","",$G22/$C22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I22" s="6">
-        <f>$C22/$H22</f>
-        <v/>
-      </c>
       <c r="J22" s="6">
-        <f>IF($E22="","",$E22/$H22)</f>
+        <f>$C22/$I22</f>
         <v/>
       </c>
       <c r="K22" s="6">
-        <f>IF($F22="","",$F22/$H22)</f>
-        <v/>
-      </c>
-      <c r="L22" s="7">
-        <f>IF($E22="","",$E22*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M22" s="6">
-        <f>IF($E22="","",$E22*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N22" s="11" t="n">
+        <f>IF($F22="","",$F22/$I22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="6">
+        <f>IF($G22="","",$G22/$I22)</f>
+        <v/>
+      </c>
+      <c r="M22" s="7">
+        <f>IF($F22="","",$F22*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N22" s="6">
+        <f>IF($F22="","",$F22*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O22" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="O22" s="11" t="n">
+      <c r="P22" s="11" t="n">
         <v>5.2</v>
       </c>
-      <c r="P22" s="12" t="inlineStr">
+      <c r="Q22" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q22" s="12" t="inlineStr">
+      <c r="R22" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R22" s="12" t="inlineStr">
+      <c r="S22" s="12" t="inlineStr">
         <is>
           <t>FB2026-5996</t>
         </is>
       </c>
-      <c r="S22" s="12" t="inlineStr">
+      <c r="T22" s="12" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="T22" s="4" t="inlineStr">
+      <c r="U22" s="4" t="inlineStr">
         <is>
           <t>Boutique + Leboncoin</t>
         </is>
       </c>
-      <c r="U22" s="4" t="inlineStr"/>
-      <c r="V22" s="4" t="inlineStr">
+      <c r="V22" s="4" t="inlineStr"/>
+      <c r="W22" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W22" s="4" t="inlineStr"/>
-      <c r="X22" s="4" t="n">
+      <c r="X22" s="4" t="inlineStr"/>
+      <c r="Y22" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2319,85 +2394,89 @@
         <v>57.51</v>
       </c>
       <c r="C23" s="6">
-        <f>$B23+$X23*Paramètres!$B$13</f>
+        <f>$B23+$Y23*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D23" s="7">
         <f>$C23/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E23" s="8" t="n">
+      <c r="E23" s="6">
+        <f>CEILING($D23*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F23" s="8" t="n">
         <v>89</v>
       </c>
-      <c r="F23" s="8">
-        <f>IF($E23="","",$E23-$C23-$L23-$M23)</f>
-        <v/>
-      </c>
-      <c r="G23" s="9">
-        <f>IF($F23="","",$F23/$C23)</f>
-        <v/>
-      </c>
-      <c r="H23" s="10" t="n">
+      <c r="G23" s="8">
+        <f>IF($F23="","",$F23-$C23-$M23-$N23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="9">
+        <f>IF($G23="","",$G23/$C23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I23" s="6">
-        <f>$C23/$H23</f>
-        <v/>
-      </c>
       <c r="J23" s="6">
-        <f>IF($E23="","",$E23/$H23)</f>
+        <f>$C23/$I23</f>
         <v/>
       </c>
       <c r="K23" s="6">
-        <f>IF($F23="","",$F23/$H23)</f>
-        <v/>
-      </c>
-      <c r="L23" s="7">
-        <f>IF($E23="","",$E23*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M23" s="6" t="n">
+        <f>IF($F23="","",$F23/$I23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="6">
+        <f>IF($G23="","",$G23/$I23)</f>
+        <v/>
+      </c>
+      <c r="M23" s="7">
+        <f>IF($F23="","",$F23*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N23" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N23" s="11" t="n">
+      <c r="O23" s="11" t="n">
         <v>45</v>
       </c>
-      <c r="O23" s="11" t="n">
+      <c r="P23" s="11" t="n">
         <v>11.7</v>
       </c>
-      <c r="P23" s="12" t="inlineStr">
+      <c r="Q23" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q23" s="12" t="inlineStr">
+      <c r="R23" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R23" s="12" t="inlineStr">
+      <c r="S23" s="12" t="inlineStr">
         <is>
           <t>FB2026-6023</t>
         </is>
       </c>
-      <c r="S23" s="12" t="inlineStr">
+      <c r="T23" s="12" t="inlineStr">
         <is>
           <t>159</t>
         </is>
       </c>
-      <c r="T23" s="4" t="inlineStr">
+      <c r="U23" s="4" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="U23" s="4" t="inlineStr"/>
-      <c r="V23" s="4" t="inlineStr">
+      <c r="V23" s="4" t="inlineStr"/>
+      <c r="W23" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W23" s="4" t="inlineStr"/>
-      <c r="X23" s="4" t="n">
+      <c r="X23" s="4" t="inlineStr"/>
+      <c r="Y23" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2411,85 +2490,89 @@
         <v>37.8</v>
       </c>
       <c r="C24" s="6">
-        <f>$B24+$X24*Paramètres!$B$13</f>
+        <f>$B24+$Y24*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D24" s="7">
         <f>$C24/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E24" s="8" t="n">
+      <c r="E24" s="6">
+        <f>CEILING($D24*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F24" s="8" t="n">
         <v>76</v>
       </c>
-      <c r="F24" s="8">
-        <f>IF($E24="","",$E24-$C24-$L24-$M24)</f>
-        <v/>
-      </c>
-      <c r="G24" s="9">
-        <f>IF($F24="","",$F24/$C24)</f>
-        <v/>
-      </c>
-      <c r="H24" s="10" t="n">
+      <c r="G24" s="8">
+        <f>IF($F24="","",$F24-$C24-$M24-$N24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="9">
+        <f>IF($G24="","",$G24/$C24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="I24" s="6">
-        <f>$C24/$H24</f>
-        <v/>
-      </c>
       <c r="J24" s="6">
-        <f>IF($E24="","",$E24/$H24)</f>
+        <f>$C24/$I24</f>
         <v/>
       </c>
       <c r="K24" s="6">
-        <f>IF($F24="","",$F24/$H24)</f>
-        <v/>
-      </c>
-      <c r="L24" s="7">
-        <f>IF($E24="","",$E24*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M24" s="6" t="n">
+        <f>IF($F24="","",$F24/$I24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="6">
+        <f>IF($G24="","",$G24/$I24)</f>
+        <v/>
+      </c>
+      <c r="M24" s="7">
+        <f>IF($F24="","",$F24*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N24" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N24" s="11" t="n">
+      <c r="O24" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="O24" s="11" t="n">
+      <c r="P24" s="11" t="n">
         <v>7.8</v>
       </c>
-      <c r="P24" s="12" t="inlineStr">
+      <c r="Q24" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q24" s="12" t="inlineStr">
+      <c r="R24" s="12" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R24" s="12" t="inlineStr">
+      <c r="S24" s="12" t="inlineStr">
         <is>
           <t>FB2026-43717</t>
         </is>
       </c>
-      <c r="S24" s="12" t="inlineStr">
+      <c r="T24" s="12" t="inlineStr">
         <is>
           <t>303</t>
         </is>
       </c>
-      <c r="T24" s="4" t="inlineStr">
+      <c r="U24" s="4" t="inlineStr">
         <is>
           <t>Leboncoin + Vinted</t>
         </is>
       </c>
-      <c r="U24" s="4" t="inlineStr"/>
-      <c r="V24" s="4" t="inlineStr">
+      <c r="V24" s="4" t="inlineStr"/>
+      <c r="W24" s="4" t="inlineStr">
         <is>
           <t>URGENT — saisonnier</t>
         </is>
       </c>
-      <c r="W24" s="4" t="inlineStr"/>
-      <c r="X24" s="4" t="n">
+      <c r="X24" s="4" t="inlineStr"/>
+      <c r="Y24" s="4" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2503,85 +2586,89 @@
         <v>21.73</v>
       </c>
       <c r="C25" s="6">
-        <f>$B25+$X25*Paramètres!$B$13</f>
+        <f>$B25+$Y25*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D25" s="7">
         <f>$C25/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E25" s="8" t="n">
+      <c r="E25" s="6">
+        <f>CEILING($D25*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F25" s="8" t="n">
         <v>49</v>
       </c>
-      <c r="F25" s="8">
-        <f>IF($E25="","",$E25-$C25-$L25-$M25)</f>
-        <v/>
-      </c>
-      <c r="G25" s="9">
-        <f>IF($F25="","",$F25/$C25)</f>
-        <v/>
-      </c>
-      <c r="H25" s="10" t="n">
+      <c r="G25" s="8">
+        <f>IF($F25="","",$F25-$C25-$M25-$N25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="9">
+        <f>IF($G25="","",$G25/$C25)</f>
+        <v/>
+      </c>
+      <c r="I25" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I25" s="6">
-        <f>$C25/$H25</f>
-        <v/>
-      </c>
       <c r="J25" s="6">
-        <f>IF($E25="","",$E25/$H25)</f>
+        <f>$C25/$I25</f>
         <v/>
       </c>
       <c r="K25" s="6">
-        <f>IF($F25="","",$F25/$H25)</f>
-        <v/>
-      </c>
-      <c r="L25" s="7">
-        <f>IF($E25="","",$E25*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M25" s="6" t="n">
+        <f>IF($F25="","",$F25/$I25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="6">
+        <f>IF($G25="","",$G25/$I25)</f>
+        <v/>
+      </c>
+      <c r="M25" s="7">
+        <f>IF($F25="","",$F25*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N25" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N25" s="11" t="n">
+      <c r="O25" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="O25" s="11" t="n">
+      <c r="P25" s="11" t="n">
         <v>4.42</v>
       </c>
-      <c r="P25" s="12" t="inlineStr">
+      <c r="Q25" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q25" s="12" t="inlineStr">
+      <c r="R25" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R25" s="12" t="inlineStr">
+      <c r="S25" s="12" t="inlineStr">
         <is>
           <t>FB2026-6023</t>
         </is>
       </c>
-      <c r="S25" s="12" t="inlineStr">
+      <c r="T25" s="12" t="inlineStr">
         <is>
           <t>155</t>
         </is>
       </c>
-      <c r="T25" s="4" t="inlineStr">
+      <c r="U25" s="4" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="U25" s="4" t="inlineStr"/>
-      <c r="V25" s="4" t="inlineStr">
+      <c r="V25" s="4" t="inlineStr"/>
+      <c r="W25" s="4" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="W25" s="4" t="inlineStr"/>
-      <c r="X25" s="4" t="n">
+      <c r="X25" s="4" t="inlineStr"/>
+      <c r="Y25" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2595,86 +2682,90 @@
         <v>50.4</v>
       </c>
       <c r="C26" s="6">
-        <f>$B26+$X26*Paramètres!$B$13</f>
+        <f>$B26+$Y26*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D26" s="7">
         <f>$C26/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
-      <c r="E26" s="8" t="n">
+      <c r="E26" s="6">
+        <f>CEILING($D26*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F26" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="F26" s="8">
-        <f>IF($E26="","",$E26-$C26-$L26-$M26)</f>
-        <v/>
-      </c>
-      <c r="G26" s="9">
-        <f>IF($F26="","",$F26/$C26)</f>
-        <v/>
-      </c>
-      <c r="H26" s="10" t="n">
+      <c r="G26" s="8">
+        <f>IF($F26="","",$F26-$C26-$M26-$N26)</f>
+        <v/>
+      </c>
+      <c r="H26" s="9">
+        <f>IF($G26="","",$G26/$C26)</f>
+        <v/>
+      </c>
+      <c r="I26" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I26" s="6">
-        <f>$C26/$H26</f>
-        <v/>
-      </c>
       <c r="J26" s="6">
-        <f>IF($E26="","",$E26/$H26)</f>
+        <f>$C26/$I26</f>
         <v/>
       </c>
       <c r="K26" s="6">
-        <f>IF($F26="","",$F26/$H26)</f>
-        <v/>
-      </c>
-      <c r="L26" s="7">
-        <f>IF($E26="","",$E26*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M26" s="6">
-        <f>IF($E26="","",$E26*Paramètres!$B$7)</f>
-        <v/>
-      </c>
-      <c r="N26" s="11" t="n">
+        <f>IF($F26="","",$F26/$I26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="6">
+        <f>IF($G26="","",$G26/$I26)</f>
+        <v/>
+      </c>
+      <c r="M26" s="7">
+        <f>IF($F26="","",$F26*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N26" s="6">
+        <f>IF($F26="","",$F26*Paramètres!$B$7)</f>
+        <v/>
+      </c>
+      <c r="O26" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="O26" s="11" t="n">
+      <c r="P26" s="11" t="n">
         <v>10.4</v>
       </c>
-      <c r="P26" s="12" t="inlineStr">
+      <c r="Q26" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q26" s="12" t="inlineStr">
+      <c r="R26" s="12" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R26" s="12" t="inlineStr">
+      <c r="S26" s="12" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S26" s="12" t="inlineStr">
+      <c r="T26" s="12" t="inlineStr">
         <is>
           <t>408</t>
         </is>
       </c>
-      <c r="T26" s="4" t="inlineStr">
+      <c r="U26" s="4" t="inlineStr">
         <is>
           <t>Boutique</t>
         </is>
       </c>
-      <c r="U26" s="4" t="inlineStr"/>
-      <c r="V26" s="4" t="inlineStr">
+      <c r="V26" s="4" t="inlineStr"/>
+      <c r="W26" s="4" t="inlineStr">
         <is>
           <t>URGENT — saisonnier</t>
         </is>
       </c>
-      <c r="W26" s="4" t="inlineStr"/>
-      <c r="X26" s="4" t="n">
+      <c r="X26" s="4" t="inlineStr"/>
+      <c r="Y26" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2688,85 +2779,89 @@
         <v>75.59999999999999</v>
       </c>
       <c r="C27" s="6">
-        <f>$B27+$X27*Paramètres!$B$13</f>
+        <f>$B27+$Y27*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D27" s="7">
         <f>$C27/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E27" s="8" t="n">
+      <c r="E27" s="6">
+        <f>CEILING($D27*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F27" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="F27" s="8">
-        <f>IF($E27="","",$E27-$C27-$L27-$M27)</f>
-        <v/>
-      </c>
-      <c r="G27" s="9">
-        <f>IF($F27="","",$F27/$C27)</f>
-        <v/>
-      </c>
-      <c r="H27" s="10" t="n">
+      <c r="G27" s="8">
+        <f>IF($F27="","",$F27-$C27-$M27-$N27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="9">
+        <f>IF($G27="","",$G27/$C27)</f>
+        <v/>
+      </c>
+      <c r="I27" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I27" s="6">
-        <f>$C27/$H27</f>
-        <v/>
-      </c>
       <c r="J27" s="6">
-        <f>IF($E27="","",$E27/$H27)</f>
+        <f>$C27/$I27</f>
         <v/>
       </c>
       <c r="K27" s="6">
-        <f>IF($F27="","",$F27/$H27)</f>
-        <v/>
-      </c>
-      <c r="L27" s="7">
-        <f>IF($E27="","",$E27*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M27" s="6" t="n">
+        <f>IF($F27="","",$F27/$I27)</f>
+        <v/>
+      </c>
+      <c r="L27" s="6">
+        <f>IF($G27="","",$G27/$I27)</f>
+        <v/>
+      </c>
+      <c r="M27" s="7">
+        <f>IF($F27="","",$F27*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N27" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N27" s="11" t="n">
+      <c r="O27" s="11" t="n">
         <v>60</v>
       </c>
-      <c r="O27" s="11" t="n">
+      <c r="P27" s="11" t="n">
         <v>15.6</v>
       </c>
-      <c r="P27" s="12" t="inlineStr">
+      <c r="Q27" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q27" s="12" t="inlineStr">
+      <c r="R27" s="12" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R27" s="12" t="inlineStr">
+      <c r="S27" s="12" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S27" s="12" t="inlineStr">
+      <c r="T27" s="12" t="inlineStr">
         <is>
           <t>199</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr">
+      <c r="U27" s="4" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="U27" s="4" t="inlineStr"/>
-      <c r="V27" s="4" t="inlineStr">
+      <c r="V27" s="4" t="inlineStr"/>
+      <c r="W27" s="4" t="inlineStr">
         <is>
           <t>Liquider</t>
         </is>
       </c>
-      <c r="W27" s="4" t="inlineStr"/>
-      <c r="X27" s="4" t="n">
+      <c r="X27" s="4" t="inlineStr"/>
+      <c r="Y27" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2780,89 +2875,93 @@
         <v>76.68000000000001</v>
       </c>
       <c r="C28" s="16">
-        <f>$B28+$X28*Paramètres!$B$13</f>
+        <f>$B28+$Y28*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D28" s="17">
         <f>$C28/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E28" s="18" t="n">
+      <c r="E28" s="16">
+        <f>CEILING($D28*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F28" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="F28" s="18">
-        <f>IF($E28="","",$E28-$C28-$L28-$M28)</f>
-        <v/>
-      </c>
-      <c r="G28" s="19">
-        <f>IF($F28="","",$F28/$C28)</f>
-        <v/>
-      </c>
-      <c r="H28" s="20" t="n">
+      <c r="G28" s="18">
+        <f>IF($F28="","",$F28-$C28-$M28-$N28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="19">
+        <f>IF($G28="","",$G28/$C28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I28" s="16">
-        <f>$C28/$H28</f>
-        <v/>
-      </c>
       <c r="J28" s="16">
-        <f>IF($E28="","",$E28/$H28)</f>
+        <f>$C28/$I28</f>
         <v/>
       </c>
       <c r="K28" s="16">
-        <f>IF($F28="","",$F28/$H28)</f>
-        <v/>
-      </c>
-      <c r="L28" s="17">
-        <f>IF($E28="","",$E28*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M28" s="16" t="n">
+        <f>IF($F28="","",$F28/$I28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="16">
+        <f>IF($G28="","",$G28/$I28)</f>
+        <v/>
+      </c>
+      <c r="M28" s="17">
+        <f>IF($F28="","",$F28*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N28" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="N28" s="21" t="n">
+      <c r="O28" s="21" t="n">
         <v>60</v>
       </c>
-      <c r="O28" s="21" t="n">
+      <c r="P28" s="21" t="n">
         <v>15.6</v>
       </c>
-      <c r="P28" s="22" t="inlineStr">
+      <c r="Q28" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q28" s="22" t="inlineStr">
+      <c r="R28" s="22" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R28" s="22" t="inlineStr">
+      <c r="S28" s="22" t="inlineStr">
         <is>
           <t>FB2026-44192</t>
         </is>
       </c>
-      <c r="S28" s="22" t="inlineStr">
+      <c r="T28" s="22" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="T28" s="14" t="inlineStr">
+      <c r="U28" s="14" t="inlineStr">
         <is>
           <t>Vinted, acheteur en Italie</t>
         </is>
       </c>
-      <c r="U28" s="14" t="inlineStr"/>
-      <c r="V28" s="14" t="inlineStr">
+      <c r="V28" s="14" t="inlineStr"/>
+      <c r="W28" s="14" t="inlineStr">
         <is>
           <t>VENDUE</t>
         </is>
       </c>
-      <c r="W28" s="14" t="inlineStr">
+      <c r="X28" s="14" t="inlineStr">
         <is>
           <t>12/08/2026</t>
         </is>
       </c>
-      <c r="X28" s="14" t="n">
+      <c r="Y28" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2876,85 +2975,89 @@
         <v>51.12</v>
       </c>
       <c r="C29" s="6">
-        <f>$B29+$X29*Paramètres!$B$13</f>
+        <f>$B29+$Y29*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D29" s="7">
         <f>$C29/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E29" s="8" t="n">
+      <c r="E29" s="6">
+        <f>CEILING($D29*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F29" s="8" t="n">
         <v>69</v>
       </c>
-      <c r="F29" s="8">
-        <f>IF($E29="","",$E29-$C29-$L29-$M29)</f>
-        <v/>
-      </c>
-      <c r="G29" s="9">
-        <f>IF($F29="","",$F29/$C29)</f>
-        <v/>
-      </c>
-      <c r="H29" s="10" t="n">
+      <c r="G29" s="8">
+        <f>IF($F29="","",$F29-$C29-$M29-$N29)</f>
+        <v/>
+      </c>
+      <c r="H29" s="9">
+        <f>IF($G29="","",$G29/$C29)</f>
+        <v/>
+      </c>
+      <c r="I29" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I29" s="6">
-        <f>$C29/$H29</f>
-        <v/>
-      </c>
       <c r="J29" s="6">
-        <f>IF($E29="","",$E29/$H29)</f>
+        <f>$C29/$I29</f>
         <v/>
       </c>
       <c r="K29" s="6">
-        <f>IF($F29="","",$F29/$H29)</f>
-        <v/>
-      </c>
-      <c r="L29" s="7">
-        <f>IF($E29="","",$E29*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M29" s="6" t="n">
+        <f>IF($F29="","",$F29/$I29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="6">
+        <f>IF($G29="","",$G29/$I29)</f>
+        <v/>
+      </c>
+      <c r="M29" s="7">
+        <f>IF($F29="","",$F29*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N29" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N29" s="11" t="n">
+      <c r="O29" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="O29" s="11" t="n">
+      <c r="P29" s="11" t="n">
         <v>10.4</v>
       </c>
-      <c r="P29" s="12" t="inlineStr">
+      <c r="Q29" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q29" s="12" t="inlineStr">
+      <c r="R29" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R29" s="12" t="inlineStr">
+      <c r="S29" s="12" t="inlineStr">
         <is>
           <t>FB2026-6023</t>
         </is>
       </c>
-      <c r="S29" s="12" t="inlineStr">
+      <c r="T29" s="12" t="inlineStr">
         <is>
           <t>150</t>
         </is>
       </c>
-      <c r="T29" s="4" t="inlineStr">
+      <c r="U29" s="4" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="U29" s="4" t="inlineStr"/>
-      <c r="V29" s="4" t="inlineStr">
+      <c r="V29" s="4" t="inlineStr"/>
+      <c r="W29" s="4" t="inlineStr">
         <is>
           <t>Liquider</t>
         </is>
       </c>
-      <c r="W29" s="4" t="inlineStr"/>
-      <c r="X29" s="4" t="n">
+      <c r="X29" s="4" t="inlineStr"/>
+      <c r="Y29" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2968,85 +3071,89 @@
         <v>38.34</v>
       </c>
       <c r="C30" s="6">
-        <f>$B30+$X30*Paramètres!$B$13</f>
+        <f>$B30+$Y30*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D30" s="7">
         <f>$C30/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E30" s="8" t="n">
+      <c r="E30" s="6">
+        <f>CEILING($D30*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F30" s="8" t="n">
         <v>54</v>
       </c>
-      <c r="F30" s="8">
-        <f>IF($E30="","",$E30-$C30-$L30-$M30)</f>
-        <v/>
-      </c>
-      <c r="G30" s="9">
-        <f>IF($F30="","",$F30/$C30)</f>
-        <v/>
-      </c>
-      <c r="H30" s="10" t="n">
+      <c r="G30" s="8">
+        <f>IF($F30="","",$F30-$C30-$M30-$N30)</f>
+        <v/>
+      </c>
+      <c r="H30" s="9">
+        <f>IF($G30="","",$G30/$C30)</f>
+        <v/>
+      </c>
+      <c r="I30" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I30" s="6">
-        <f>$C30/$H30</f>
-        <v/>
-      </c>
       <c r="J30" s="6">
-        <f>IF($E30="","",$E30/$H30)</f>
+        <f>$C30/$I30</f>
         <v/>
       </c>
       <c r="K30" s="6">
-        <f>IF($F30="","",$F30/$H30)</f>
-        <v/>
-      </c>
-      <c r="L30" s="7">
-        <f>IF($E30="","",$E30*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M30" s="6" t="n">
+        <f>IF($F30="","",$F30/$I30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>IF($G30="","",$G30/$I30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="7">
+        <f>IF($F30="","",$F30*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N30" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N30" s="11" t="n">
+      <c r="O30" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="O30" s="11" t="n">
+      <c r="P30" s="11" t="n">
         <v>7.8</v>
       </c>
-      <c r="P30" s="12" t="inlineStr">
+      <c r="Q30" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q30" s="12" t="inlineStr">
+      <c r="R30" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R30" s="12" t="inlineStr">
+      <c r="S30" s="12" t="inlineStr">
         <is>
           <t>FB2026-6023</t>
         </is>
       </c>
-      <c r="S30" s="12" t="inlineStr">
+      <c r="T30" s="12" t="inlineStr">
         <is>
           <t>114</t>
         </is>
       </c>
-      <c r="T30" s="4" t="inlineStr">
+      <c r="U30" s="4" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="U30" s="4" t="inlineStr"/>
-      <c r="V30" s="4" t="inlineStr">
+      <c r="V30" s="4" t="inlineStr"/>
+      <c r="W30" s="4" t="inlineStr">
         <is>
           <t>Liquider</t>
         </is>
       </c>
-      <c r="W30" s="4" t="inlineStr"/>
-      <c r="X30" s="4" t="n">
+      <c r="X30" s="4" t="inlineStr"/>
+      <c r="Y30" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3060,85 +3167,89 @@
         <v>51.12</v>
       </c>
       <c r="C31" s="6">
-        <f>$B31+$X31*Paramètres!$B$13</f>
+        <f>$B31+$Y31*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D31" s="7">
         <f>$C31/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E31" s="8" t="n">
+      <c r="E31" s="6">
+        <f>CEILING($D31*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F31" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="F31" s="8">
-        <f>IF($E31="","",$E31-$C31-$L31-$M31)</f>
-        <v/>
-      </c>
-      <c r="G31" s="9">
-        <f>IF($F31="","",$F31/$C31)</f>
-        <v/>
-      </c>
-      <c r="H31" s="10" t="n">
+      <c r="G31" s="8">
+        <f>IF($F31="","",$F31-$C31-$M31-$N31)</f>
+        <v/>
+      </c>
+      <c r="H31" s="9">
+        <f>IF($G31="","",$G31/$C31)</f>
+        <v/>
+      </c>
+      <c r="I31" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I31" s="6">
-        <f>$C31/$H31</f>
-        <v/>
-      </c>
       <c r="J31" s="6">
-        <f>IF($E31="","",$E31/$H31)</f>
+        <f>$C31/$I31</f>
         <v/>
       </c>
       <c r="K31" s="6">
-        <f>IF($F31="","",$F31/$H31)</f>
-        <v/>
-      </c>
-      <c r="L31" s="7">
-        <f>IF($E31="","",$E31*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M31" s="6" t="n">
+        <f>IF($F31="","",$F31/$I31)</f>
+        <v/>
+      </c>
+      <c r="L31" s="6">
+        <f>IF($G31="","",$G31/$I31)</f>
+        <v/>
+      </c>
+      <c r="M31" s="7">
+        <f>IF($F31="","",$F31*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N31" s="11" t="n">
+      <c r="O31" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="O31" s="11" t="n">
+      <c r="P31" s="11" t="n">
         <v>10.4</v>
       </c>
-      <c r="P31" s="12" t="inlineStr">
+      <c r="Q31" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q31" s="12" t="inlineStr">
+      <c r="R31" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R31" s="12" t="inlineStr">
+      <c r="S31" s="12" t="inlineStr">
         <is>
           <t>FB2026-6023</t>
         </is>
       </c>
-      <c r="S31" s="12" t="inlineStr">
+      <c r="T31" s="12" t="inlineStr">
         <is>
           <t>156</t>
         </is>
       </c>
-      <c r="T31" s="4" t="inlineStr">
+      <c r="U31" s="4" t="inlineStr">
         <is>
           <t>Leboncoin</t>
         </is>
       </c>
-      <c r="U31" s="4" t="inlineStr"/>
-      <c r="V31" s="4" t="inlineStr">
+      <c r="V31" s="4" t="inlineStr"/>
+      <c r="W31" s="4" t="inlineStr">
         <is>
           <t>Liquider</t>
         </is>
       </c>
-      <c r="W31" s="4" t="inlineStr"/>
-      <c r="X31" s="4" t="n">
+      <c r="X31" s="4" t="inlineStr"/>
+      <c r="Y31" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3152,85 +3263,89 @@
         <v>52.4</v>
       </c>
       <c r="C32" s="6">
-        <f>$B32+$X32*Paramètres!$B$13</f>
+        <f>$B32+$Y32*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D32" s="7">
         <f>$C32/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E32" s="8" t="n">
+      <c r="E32" s="6">
+        <f>CEILING($D32*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F32" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="F32" s="8">
-        <f>IF($E32="","",$E32-$C32-$L32-$M32)</f>
-        <v/>
-      </c>
-      <c r="G32" s="9">
-        <f>IF($F32="","",$F32/$C32)</f>
-        <v/>
-      </c>
-      <c r="H32" s="10" t="n">
+      <c r="G32" s="8">
+        <f>IF($F32="","",$F32-$C32-$M32-$N32)</f>
+        <v/>
+      </c>
+      <c r="H32" s="9">
+        <f>IF($G32="","",$G32/$C32)</f>
+        <v/>
+      </c>
+      <c r="I32" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I32" s="6">
-        <f>$C32/$H32</f>
-        <v/>
-      </c>
       <c r="J32" s="6">
-        <f>IF($E32="","",$E32/$H32)</f>
+        <f>$C32/$I32</f>
         <v/>
       </c>
       <c r="K32" s="6">
-        <f>IF($F32="","",$F32/$H32)</f>
-        <v/>
-      </c>
-      <c r="L32" s="7">
-        <f>IF($E32="","",$E32*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M32" s="6" t="n">
+        <f>IF($F32="","",$F32/$I32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="6">
+        <f>IF($G32="","",$G32/$I32)</f>
+        <v/>
+      </c>
+      <c r="M32" s="7">
+        <f>IF($F32="","",$F32*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N32" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N32" s="11" t="n">
+      <c r="O32" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="O32" s="11" t="n">
+      <c r="P32" s="11" t="n">
         <v>10.66</v>
       </c>
-      <c r="P32" s="12" t="inlineStr">
+      <c r="Q32" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q32" s="12" t="inlineStr">
+      <c r="R32" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R32" s="12" t="inlineStr">
+      <c r="S32" s="12" t="inlineStr">
         <is>
           <t>FB2026-6023</t>
         </is>
       </c>
-      <c r="S32" s="12" t="inlineStr">
+      <c r="T32" s="12" t="inlineStr">
         <is>
           <t>158</t>
         </is>
       </c>
-      <c r="T32" s="4" t="inlineStr">
+      <c r="U32" s="4" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="U32" s="4" t="inlineStr"/>
-      <c r="V32" s="4" t="inlineStr">
+      <c r="V32" s="4" t="inlineStr"/>
+      <c r="W32" s="4" t="inlineStr">
         <is>
           <t>Liquider</t>
         </is>
       </c>
-      <c r="W32" s="4" t="inlineStr"/>
-      <c r="X32" s="4" t="n">
+      <c r="X32" s="4" t="inlineStr"/>
+      <c r="Y32" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3244,89 +3359,93 @@
         <v>57.51</v>
       </c>
       <c r="C33" s="16">
-        <f>$B33+$X33*Paramètres!$B$13</f>
+        <f>$B33+$Y33*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D33" s="17">
         <f>$C33/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E33" s="18" t="n">
+      <c r="E33" s="16">
+        <f>CEILING($D33*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F33" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="F33" s="18">
-        <f>IF($E33="","",$E33-$C33-$L33-$M33)</f>
-        <v/>
-      </c>
-      <c r="G33" s="19">
-        <f>IF($F33="","",$F33/$C33)</f>
-        <v/>
-      </c>
-      <c r="H33" s="20" t="n">
+      <c r="G33" s="18">
+        <f>IF($F33="","",$F33-$C33-$M33-$N33)</f>
+        <v/>
+      </c>
+      <c r="H33" s="19">
+        <f>IF($G33="","",$G33/$C33)</f>
+        <v/>
+      </c>
+      <c r="I33" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I33" s="16">
-        <f>$C33/$H33</f>
-        <v/>
-      </c>
       <c r="J33" s="16">
-        <f>IF($E33="","",$E33/$H33)</f>
+        <f>$C33/$I33</f>
         <v/>
       </c>
       <c r="K33" s="16">
-        <f>IF($F33="","",$F33/$H33)</f>
-        <v/>
-      </c>
-      <c r="L33" s="17">
-        <f>IF($E33="","",$E33*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M33" s="16" t="n">
+        <f>IF($F33="","",$F33/$I33)</f>
+        <v/>
+      </c>
+      <c r="L33" s="16">
+        <f>IF($G33="","",$G33/$I33)</f>
+        <v/>
+      </c>
+      <c r="M33" s="17">
+        <f>IF($F33="","",$F33*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N33" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="N33" s="21" t="n">
+      <c r="O33" s="21" t="n">
         <v>45</v>
       </c>
-      <c r="O33" s="21" t="n">
+      <c r="P33" s="21" t="n">
         <v>11.7</v>
       </c>
-      <c r="P33" s="22" t="inlineStr">
+      <c r="Q33" s="22" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="Q33" s="22" t="inlineStr">
+      <c r="R33" s="22" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R33" s="22" t="inlineStr">
+      <c r="S33" s="22" t="inlineStr">
         <is>
           <t>FB2026-6023</t>
         </is>
       </c>
-      <c r="S33" s="22" t="inlineStr">
+      <c r="T33" s="22" t="inlineStr">
         <is>
           <t>141</t>
         </is>
       </c>
-      <c r="T33" s="14" t="inlineStr">
+      <c r="U33" s="14" t="inlineStr">
         <is>
           <t>date à compléter</t>
         </is>
       </c>
-      <c r="U33" s="14" t="inlineStr"/>
-      <c r="V33" s="14" t="inlineStr">
+      <c r="V33" s="14" t="inlineStr"/>
+      <c r="W33" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="W33" s="14" t="inlineStr">
+      <c r="X33" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="X33" s="14" t="n">
+      <c r="Y33" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3340,89 +3459,93 @@
         <v>113.4</v>
       </c>
       <c r="C34" s="16">
-        <f>$B34+$X34*Paramètres!$B$13</f>
+        <f>$B34+$Y34*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D34" s="17">
         <f>$C34/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E34" s="18" t="n">
+      <c r="E34" s="16">
+        <f>CEILING($D34*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F34" s="18" t="n">
         <v>125</v>
       </c>
-      <c r="F34" s="18">
-        <f>IF($E34="","",$E34-$C34-$L34-$M34)</f>
-        <v/>
-      </c>
-      <c r="G34" s="19">
-        <f>IF($F34="","",$F34/$C34)</f>
-        <v/>
-      </c>
-      <c r="H34" s="20" t="n">
+      <c r="G34" s="18">
+        <f>IF($F34="","",$F34-$C34-$M34-$N34)</f>
+        <v/>
+      </c>
+      <c r="H34" s="19">
+        <f>IF($G34="","",$G34/$C34)</f>
+        <v/>
+      </c>
+      <c r="I34" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I34" s="16">
-        <f>$C34/$H34</f>
-        <v/>
-      </c>
       <c r="J34" s="16">
-        <f>IF($E34="","",$E34/$H34)</f>
+        <f>$C34/$I34</f>
         <v/>
       </c>
       <c r="K34" s="16">
-        <f>IF($F34="","",$F34/$H34)</f>
-        <v/>
-      </c>
-      <c r="L34" s="17">
-        <f>IF($E34="","",$E34*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M34" s="16" t="n">
+        <f>IF($F34="","",$F34/$I34)</f>
+        <v/>
+      </c>
+      <c r="L34" s="16">
+        <f>IF($G34="","",$G34/$I34)</f>
+        <v/>
+      </c>
+      <c r="M34" s="17">
+        <f>IF($F34="","",$F34*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N34" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="N34" s="21" t="n">
+      <c r="O34" s="21" t="n">
         <v>90</v>
       </c>
-      <c r="O34" s="21" t="n">
+      <c r="P34" s="21" t="n">
         <v>23.4</v>
       </c>
-      <c r="P34" s="22" t="inlineStr">
+      <c r="Q34" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q34" s="22" t="inlineStr">
+      <c r="R34" s="22" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R34" s="22" t="inlineStr">
+      <c r="S34" s="22" t="inlineStr">
         <is>
           <t>FB2026-44194</t>
         </is>
       </c>
-      <c r="S34" s="22" t="inlineStr">
+      <c r="T34" s="22" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="T34" s="14" t="inlineStr">
+      <c r="U34" s="14" t="inlineStr">
         <is>
           <t>date à compléter</t>
         </is>
       </c>
-      <c r="U34" s="14" t="inlineStr"/>
-      <c r="V34" s="14" t="inlineStr">
+      <c r="V34" s="14" t="inlineStr"/>
+      <c r="W34" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="W34" s="14" t="inlineStr">
+      <c r="X34" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="X34" s="14" t="n">
+      <c r="Y34" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3436,89 +3559,93 @@
         <v>25.2</v>
       </c>
       <c r="C35" s="16">
-        <f>$B35+$X35*Paramètres!$B$13</f>
+        <f>$B35+$Y35*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D35" s="17">
         <f>$C35/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E35" s="18" t="n">
+      <c r="E35" s="16">
+        <f>CEILING($D35*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F35" s="18" t="n">
         <v>35</v>
       </c>
-      <c r="F35" s="18">
-        <f>IF($E35="","",$E35-$C35-$L35-$M35)</f>
-        <v/>
-      </c>
-      <c r="G35" s="19">
-        <f>IF($F35="","",$F35/$C35)</f>
-        <v/>
-      </c>
-      <c r="H35" s="20" t="n">
+      <c r="G35" s="18">
+        <f>IF($F35="","",$F35-$C35-$M35-$N35)</f>
+        <v/>
+      </c>
+      <c r="H35" s="19">
+        <f>IF($G35="","",$G35/$C35)</f>
+        <v/>
+      </c>
+      <c r="I35" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I35" s="16">
-        <f>$C35/$H35</f>
-        <v/>
-      </c>
       <c r="J35" s="16">
-        <f>IF($E35="","",$E35/$H35)</f>
+        <f>$C35/$I35</f>
         <v/>
       </c>
       <c r="K35" s="16">
-        <f>IF($F35="","",$F35/$H35)</f>
-        <v/>
-      </c>
-      <c r="L35" s="17">
-        <f>IF($E35="","",$E35*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M35" s="16" t="n">
+        <f>IF($F35="","",$F35/$I35)</f>
+        <v/>
+      </c>
+      <c r="L35" s="16">
+        <f>IF($G35="","",$G35/$I35)</f>
+        <v/>
+      </c>
+      <c r="M35" s="17">
+        <f>IF($F35="","",$F35*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N35" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="N35" s="21" t="n">
+      <c r="O35" s="21" t="n">
         <v>20</v>
       </c>
-      <c r="O35" s="21" t="n">
+      <c r="P35" s="21" t="n">
         <v>5.2</v>
       </c>
-      <c r="P35" s="22" t="inlineStr">
+      <c r="Q35" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q35" s="22" t="inlineStr">
+      <c r="R35" s="22" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R35" s="22" t="inlineStr">
+      <c r="S35" s="22" t="inlineStr">
         <is>
           <t>FB2026-43717</t>
         </is>
       </c>
-      <c r="S35" s="22" t="inlineStr">
+      <c r="T35" s="22" t="inlineStr">
         <is>
           <t>168</t>
         </is>
       </c>
-      <c r="T35" s="14" t="inlineStr">
+      <c r="U35" s="14" t="inlineStr">
         <is>
           <t>date à compléter</t>
         </is>
       </c>
-      <c r="U35" s="14" t="inlineStr"/>
-      <c r="V35" s="14" t="inlineStr">
+      <c r="V35" s="14" t="inlineStr"/>
+      <c r="W35" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="W35" s="14" t="inlineStr">
+      <c r="X35" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="X35" s="14" t="n">
+      <c r="Y35" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3532,89 +3659,93 @@
         <v>50.4</v>
       </c>
       <c r="C36" s="16">
-        <f>$B36+$X36*Paramètres!$B$13</f>
+        <f>$B36+$Y36*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D36" s="17">
         <f>$C36/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E36" s="18" t="n">
+      <c r="E36" s="16">
+        <f>CEILING($D36*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F36" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="F36" s="18">
-        <f>IF($E36="","",$E36-$C36-$L36-$M36)</f>
-        <v/>
-      </c>
-      <c r="G36" s="19">
-        <f>IF($F36="","",$F36/$C36)</f>
-        <v/>
-      </c>
-      <c r="H36" s="20" t="n">
+      <c r="G36" s="18">
+        <f>IF($F36="","",$F36-$C36-$M36-$N36)</f>
+        <v/>
+      </c>
+      <c r="H36" s="19">
+        <f>IF($G36="","",$G36/$C36)</f>
+        <v/>
+      </c>
+      <c r="I36" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I36" s="16">
-        <f>$C36/$H36</f>
-        <v/>
-      </c>
       <c r="J36" s="16">
-        <f>IF($E36="","",$E36/$H36)</f>
+        <f>$C36/$I36</f>
         <v/>
       </c>
       <c r="K36" s="16">
-        <f>IF($F36="","",$F36/$H36)</f>
-        <v/>
-      </c>
-      <c r="L36" s="17">
-        <f>IF($E36="","",$E36*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M36" s="16" t="n">
+        <f>IF($F36="","",$F36/$I36)</f>
+        <v/>
+      </c>
+      <c r="L36" s="16">
+        <f>IF($G36="","",$G36/$I36)</f>
+        <v/>
+      </c>
+      <c r="M36" s="17">
+        <f>IF($F36="","",$F36*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N36" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="N36" s="21" t="n">
+      <c r="O36" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="O36" s="21" t="n">
+      <c r="P36" s="21" t="n">
         <v>10.4</v>
       </c>
-      <c r="P36" s="22" t="inlineStr">
+      <c r="Q36" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q36" s="22" t="inlineStr">
+      <c r="R36" s="22" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R36" s="22" t="inlineStr">
+      <c r="S36" s="22" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S36" s="22" t="inlineStr">
+      <c r="T36" s="22" t="inlineStr">
         <is>
           <t>170</t>
         </is>
       </c>
-      <c r="T36" s="14" t="inlineStr">
+      <c r="U36" s="14" t="inlineStr">
         <is>
           <t>date à compléter</t>
         </is>
       </c>
-      <c r="U36" s="14" t="inlineStr"/>
-      <c r="V36" s="14" t="inlineStr">
+      <c r="V36" s="14" t="inlineStr"/>
+      <c r="W36" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="W36" s="14" t="inlineStr">
+      <c r="X36" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="X36" s="14" t="n">
+      <c r="Y36" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3628,89 +3759,93 @@
         <v>50.4</v>
       </c>
       <c r="C37" s="16">
-        <f>$B37+$X37*Paramètres!$B$13</f>
+        <f>$B37+$Y37*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D37" s="17">
         <f>$C37/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E37" s="18" t="n">
+      <c r="E37" s="16">
+        <f>CEILING($D37*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F37" s="18" t="n">
         <v>60</v>
       </c>
-      <c r="F37" s="18">
-        <f>IF($E37="","",$E37-$C37-$L37-$M37)</f>
-        <v/>
-      </c>
-      <c r="G37" s="19">
-        <f>IF($F37="","",$F37/$C37)</f>
-        <v/>
-      </c>
-      <c r="H37" s="20" t="n">
+      <c r="G37" s="18">
+        <f>IF($F37="","",$F37-$C37-$M37-$N37)</f>
+        <v/>
+      </c>
+      <c r="H37" s="19">
+        <f>IF($G37="","",$G37/$C37)</f>
+        <v/>
+      </c>
+      <c r="I37" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I37" s="16">
-        <f>$C37/$H37</f>
-        <v/>
-      </c>
       <c r="J37" s="16">
-        <f>IF($E37="","",$E37/$H37)</f>
+        <f>$C37/$I37</f>
         <v/>
       </c>
       <c r="K37" s="16">
-        <f>IF($F37="","",$F37/$H37)</f>
-        <v/>
-      </c>
-      <c r="L37" s="17">
-        <f>IF($E37="","",$E37*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M37" s="16" t="n">
+        <f>IF($F37="","",$F37/$I37)</f>
+        <v/>
+      </c>
+      <c r="L37" s="16">
+        <f>IF($G37="","",$G37/$I37)</f>
+        <v/>
+      </c>
+      <c r="M37" s="17">
+        <f>IF($F37="","",$F37*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N37" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="N37" s="21" t="n">
+      <c r="O37" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="O37" s="21" t="n">
+      <c r="P37" s="21" t="n">
         <v>10.4</v>
       </c>
-      <c r="P37" s="22" t="inlineStr">
+      <c r="Q37" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q37" s="22" t="inlineStr">
+      <c r="R37" s="22" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R37" s="22" t="inlineStr">
+      <c r="S37" s="22" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S37" s="22" t="inlineStr">
+      <c r="T37" s="22" t="inlineStr">
         <is>
           <t>431</t>
         </is>
       </c>
-      <c r="T37" s="14" t="inlineStr">
+      <c r="U37" s="14" t="inlineStr">
         <is>
           <t>date à compléter</t>
         </is>
       </c>
-      <c r="U37" s="14" t="inlineStr"/>
-      <c r="V37" s="14" t="inlineStr">
+      <c r="V37" s="14" t="inlineStr"/>
+      <c r="W37" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="W37" s="14" t="inlineStr">
+      <c r="X37" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="X37" s="14" t="n">
+      <c r="Y37" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3724,89 +3859,93 @@
         <v>63</v>
       </c>
       <c r="C38" s="16">
-        <f>$B38+$X38*Paramètres!$B$13</f>
+        <f>$B38+$Y38*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D38" s="17">
         <f>$C38/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E38" s="18" t="n">
+      <c r="E38" s="16">
+        <f>CEILING($D38*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F38" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="F38" s="18">
-        <f>IF($E38="","",$E38-$C38-$L38-$M38)</f>
-        <v/>
-      </c>
-      <c r="G38" s="19">
-        <f>IF($F38="","",$F38/$C38)</f>
-        <v/>
-      </c>
-      <c r="H38" s="20" t="n">
+      <c r="G38" s="18">
+        <f>IF($F38="","",$F38-$C38-$M38-$N38)</f>
+        <v/>
+      </c>
+      <c r="H38" s="19">
+        <f>IF($G38="","",$G38/$C38)</f>
+        <v/>
+      </c>
+      <c r="I38" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I38" s="16">
-        <f>$C38/$H38</f>
-        <v/>
-      </c>
       <c r="J38" s="16">
-        <f>IF($E38="","",$E38/$H38)</f>
+        <f>$C38/$I38</f>
         <v/>
       </c>
       <c r="K38" s="16">
-        <f>IF($F38="","",$F38/$H38)</f>
-        <v/>
-      </c>
-      <c r="L38" s="17">
-        <f>IF($E38="","",$E38*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M38" s="16" t="n">
+        <f>IF($F38="","",$F38/$I38)</f>
+        <v/>
+      </c>
+      <c r="L38" s="16">
+        <f>IF($G38="","",$G38/$I38)</f>
+        <v/>
+      </c>
+      <c r="M38" s="17">
+        <f>IF($F38="","",$F38*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N38" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="N38" s="21" t="n">
+      <c r="O38" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="O38" s="21" t="n">
+      <c r="P38" s="21" t="n">
         <v>13</v>
       </c>
-      <c r="P38" s="22" t="inlineStr">
+      <c r="Q38" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q38" s="22" t="inlineStr">
+      <c r="R38" s="22" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="R38" s="22" t="inlineStr">
+      <c r="S38" s="22" t="inlineStr">
         <is>
           <t>FB2026-43716</t>
         </is>
       </c>
-      <c r="S38" s="22" t="inlineStr">
+      <c r="T38" s="22" t="inlineStr">
         <is>
           <t>103</t>
         </is>
       </c>
-      <c r="T38" s="14" t="inlineStr">
+      <c r="U38" s="14" t="inlineStr">
         <is>
           <t>date à compléter</t>
         </is>
       </c>
-      <c r="U38" s="14" t="inlineStr"/>
-      <c r="V38" s="14" t="inlineStr">
+      <c r="V38" s="14" t="inlineStr"/>
+      <c r="W38" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="W38" s="14" t="inlineStr">
+      <c r="X38" s="14" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="X38" s="14" t="n">
+      <c r="Y38" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3820,83 +3959,87 @@
         <v>19.17</v>
       </c>
       <c r="C39" s="25">
-        <f>$B39+$X39*Paramètres!$B$13</f>
+        <f>$B39+$Y39*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D39" s="26">
         <f>$C39/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E39" s="27" t="n"/>
-      <c r="F39" s="28">
-        <f>IF($E39="","",$E39-$C39-$L39-$M39)</f>
-        <v/>
-      </c>
-      <c r="G39" s="29">
-        <f>IF($F39="","",$F39/$C39)</f>
-        <v/>
-      </c>
-      <c r="H39" s="30" t="n">
+      <c r="E39" s="25">
+        <f>CEILING($D39*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F39" s="27" t="n"/>
+      <c r="G39" s="28">
+        <f>IF($F39="","",$F39-$C39-$M39-$N39)</f>
+        <v/>
+      </c>
+      <c r="H39" s="29">
+        <f>IF($G39="","",$G39/$C39)</f>
+        <v/>
+      </c>
+      <c r="I39" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="I39" s="25">
-        <f>$C39/$H39</f>
-        <v/>
-      </c>
       <c r="J39" s="25">
-        <f>IF($E39="","",$E39/$H39)</f>
+        <f>$C39/$I39</f>
         <v/>
       </c>
       <c r="K39" s="25">
-        <f>IF($F39="","",$F39/$H39)</f>
-        <v/>
-      </c>
-      <c r="L39" s="26">
-        <f>IF($E39="","",$E39*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M39" s="25" t="n">
+        <f>IF($F39="","",$F39/$I39)</f>
+        <v/>
+      </c>
+      <c r="L39" s="25">
+        <f>IF($G39="","",$G39/$I39)</f>
+        <v/>
+      </c>
+      <c r="M39" s="26">
+        <f>IF($F39="","",$F39*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N39" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="N39" s="31" t="n">
+      <c r="O39" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="O39" s="31" t="n">
+      <c r="P39" s="31" t="n">
         <v>3.9</v>
       </c>
-      <c r="P39" s="32" t="inlineStr">
+      <c r="Q39" s="32" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q39" s="32" t="inlineStr">
+      <c r="R39" s="32" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R39" s="32" t="inlineStr">
+      <c r="S39" s="32" t="inlineStr">
         <is>
           <t>FB2026-44192</t>
         </is>
       </c>
-      <c r="S39" s="32" t="inlineStr">
+      <c r="T39" s="32" t="inlineStr">
         <is>
           <t>159</t>
         </is>
       </c>
-      <c r="T39" s="23" t="inlineStr">
+      <c r="U39" s="23" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="U39" s="23" t="inlineStr"/>
-      <c r="V39" s="23" t="inlineStr">
+      <c r="V39" s="23" t="inlineStr"/>
+      <c r="W39" s="23" t="inlineStr">
         <is>
           <t>PRIX À ÉTABLIR</t>
         </is>
       </c>
-      <c r="W39" s="23" t="inlineStr"/>
-      <c r="X39" s="23" t="n">
+      <c r="X39" s="23" t="inlineStr"/>
+      <c r="Y39" s="23" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3910,83 +4053,87 @@
         <v>38.34</v>
       </c>
       <c r="C40" s="25">
-        <f>$B40+$X40*Paramètres!$B$13</f>
+        <f>$B40+$Y40*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D40" s="26">
         <f>$C40/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E40" s="27" t="n"/>
-      <c r="F40" s="28">
-        <f>IF($E40="","",$E40-$C40-$L40-$M40)</f>
-        <v/>
-      </c>
-      <c r="G40" s="29">
-        <f>IF($F40="","",$F40/$C40)</f>
-        <v/>
-      </c>
-      <c r="H40" s="30" t="n">
+      <c r="E40" s="25">
+        <f>CEILING($D40*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F40" s="27" t="n"/>
+      <c r="G40" s="28">
+        <f>IF($F40="","",$F40-$C40-$M40-$N40)</f>
+        <v/>
+      </c>
+      <c r="H40" s="29">
+        <f>IF($G40="","",$G40/$C40)</f>
+        <v/>
+      </c>
+      <c r="I40" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="I40" s="25">
-        <f>$C40/$H40</f>
-        <v/>
-      </c>
       <c r="J40" s="25">
-        <f>IF($E40="","",$E40/$H40)</f>
+        <f>$C40/$I40</f>
         <v/>
       </c>
       <c r="K40" s="25">
-        <f>IF($F40="","",$F40/$H40)</f>
-        <v/>
-      </c>
-      <c r="L40" s="26">
-        <f>IF($E40="","",$E40*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M40" s="25" t="n">
+        <f>IF($F40="","",$F40/$I40)</f>
+        <v/>
+      </c>
+      <c r="L40" s="25">
+        <f>IF($G40="","",$G40/$I40)</f>
+        <v/>
+      </c>
+      <c r="M40" s="26">
+        <f>IF($F40="","",$F40*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N40" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="N40" s="31" t="n">
+      <c r="O40" s="31" t="n">
         <v>30</v>
       </c>
-      <c r="O40" s="31" t="n">
+      <c r="P40" s="31" t="n">
         <v>7.8</v>
       </c>
-      <c r="P40" s="32" t="inlineStr">
+      <c r="Q40" s="32" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q40" s="32" t="inlineStr">
+      <c r="R40" s="32" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="R40" s="32" t="inlineStr">
+      <c r="S40" s="32" t="inlineStr">
         <is>
           <t>FB2026-44192</t>
         </is>
       </c>
-      <c r="S40" s="32" t="inlineStr">
+      <c r="T40" s="32" t="inlineStr">
         <is>
           <t>299</t>
         </is>
       </c>
-      <c r="T40" s="23" t="inlineStr">
+      <c r="U40" s="23" t="inlineStr">
         <is>
           <t>Leboncoin + eBay</t>
         </is>
       </c>
-      <c r="U40" s="23" t="inlineStr"/>
-      <c r="V40" s="23" t="inlineStr">
+      <c r="V40" s="23" t="inlineStr"/>
+      <c r="W40" s="23" t="inlineStr">
         <is>
           <t>PRIX À ÉTABLIR</t>
         </is>
       </c>
-      <c r="W40" s="23" t="inlineStr"/>
-      <c r="X40" s="23" t="n">
+      <c r="X40" s="23" t="inlineStr"/>
+      <c r="Y40" s="23" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4000,83 +4147,87 @@
         <v>63</v>
       </c>
       <c r="C41" s="6">
-        <f>$B41+$X41*Paramètres!$B$13</f>
+        <f>$B41+$Y41*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D41" s="7">
         <f>$C41/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E41" s="13" t="n"/>
-      <c r="F41" s="8">
-        <f>IF($E41="","",$E41-$C41-$L41-$M41)</f>
-        <v/>
-      </c>
-      <c r="G41" s="9">
-        <f>IF($F41="","",$F41/$C41)</f>
-        <v/>
-      </c>
-      <c r="H41" s="10" t="n">
+      <c r="E41" s="6">
+        <f>CEILING($D41*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F41" s="13" t="n"/>
+      <c r="G41" s="8">
+        <f>IF($F41="","",$F41-$C41-$M41-$N41)</f>
+        <v/>
+      </c>
+      <c r="H41" s="9">
+        <f>IF($G41="","",$G41/$C41)</f>
+        <v/>
+      </c>
+      <c r="I41" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="I41" s="6">
-        <f>$C41/$H41</f>
-        <v/>
-      </c>
       <c r="J41" s="6">
-        <f>IF($E41="","",$E41/$H41)</f>
+        <f>$C41/$I41</f>
         <v/>
       </c>
       <c r="K41" s="6">
-        <f>IF($F41="","",$F41/$H41)</f>
-        <v/>
-      </c>
-      <c r="L41" s="7">
-        <f>IF($E41="","",$E41*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="M41" s="6" t="n">
+        <f>IF($F41="","",$F41/$I41)</f>
+        <v/>
+      </c>
+      <c r="L41" s="6">
+        <f>IF($G41="","",$G41/$I41)</f>
+        <v/>
+      </c>
+      <c r="M41" s="7">
+        <f>IF($F41="","",$F41*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N41" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N41" s="11" t="n">
+      <c r="O41" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="O41" s="11" t="n">
+      <c r="P41" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="P41" s="12" t="inlineStr">
+      <c r="Q41" s="12" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="Q41" s="12" t="inlineStr">
+      <c r="R41" s="12" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
-      <c r="R41" s="12" t="inlineStr">
+      <c r="S41" s="12" t="inlineStr">
         <is>
           <t>FB2026-46056</t>
         </is>
       </c>
-      <c r="S41" s="12" t="inlineStr">
+      <c r="T41" s="12" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="T41" s="4" t="inlineStr">
+      <c r="U41" s="4" t="inlineStr">
         <is>
           <t>Vinted, authentification</t>
         </is>
       </c>
-      <c r="U41" s="4" t="inlineStr"/>
-      <c r="V41" s="4" t="inlineStr">
+      <c r="V41" s="4" t="inlineStr"/>
+      <c r="W41" s="4" t="inlineStr">
         <is>
           <t>PRIX À ÉTABLIR</t>
         </is>
       </c>
-      <c r="W41" s="4" t="inlineStr"/>
-      <c r="X41" s="4" t="n">
+      <c r="X41" s="4" t="inlineStr"/>
+      <c r="Y41" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4095,34 +4246,34 @@
         <v/>
       </c>
       <c r="D42" s="35" t="n"/>
-      <c r="E42" s="34">
-        <f>SUM(E6:E41)</f>
-        <v/>
-      </c>
+      <c r="E42" s="35" t="n"/>
       <c r="F42" s="34">
         <f>SUM(F6:F41)</f>
         <v/>
       </c>
-      <c r="G42" s="36">
-        <f>F42/C42</f>
-        <v/>
-      </c>
-      <c r="H42" s="37">
-        <f>SUM(H6:H41)</f>
-        <v/>
-      </c>
-      <c r="I42" s="35" t="n"/>
+      <c r="G42" s="34">
+        <f>SUM(G6:G41)</f>
+        <v/>
+      </c>
+      <c r="H42" s="36">
+        <f>G42/C42</f>
+        <v/>
+      </c>
+      <c r="I42" s="37">
+        <f>SUM(I6:I41)</f>
+        <v/>
+      </c>
       <c r="J42" s="35" t="n"/>
       <c r="K42" s="35" t="n"/>
-      <c r="L42" s="34">
-        <f>SUM(L6:L41)</f>
-        <v/>
-      </c>
+      <c r="L42" s="35" t="n"/>
       <c r="M42" s="34">
         <f>SUM(M6:M41)</f>
         <v/>
       </c>
-      <c r="N42" s="35" t="n"/>
+      <c r="N42" s="34">
+        <f>SUM(N6:N41)</f>
+        <v/>
+      </c>
       <c r="O42" s="35" t="n"/>
       <c r="P42" s="35" t="n"/>
       <c r="Q42" s="35" t="n"/>
@@ -4133,10 +4284,11 @@
       <c r="V42" s="35" t="n"/>
       <c r="W42" s="35" t="n"/>
       <c r="X42" s="35" t="n"/>
+      <c r="Y42" s="35" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:X41"/>
-  <conditionalFormatting sqref="F6:F41">
+  <autoFilter ref="A5:Y41"/>
+  <conditionalFormatting sqref="G6:G41">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>10</formula>
     </cfRule>
@@ -4151,7 +4303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -4229,7 +4381,7 @@
         </is>
       </c>
       <c r="B10" s="8">
-        <f>'Stock complet'!E42</f>
+        <f>'Stock complet'!F42</f>
         <v/>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -4245,7 +4397,7 @@
         </is>
       </c>
       <c r="B11" s="7">
-        <f>-'Stock complet'!L42</f>
+        <f>-'Stock complet'!M42</f>
         <v/>
       </c>
     </row>
@@ -4256,7 +4408,7 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <f>-'Stock complet'!M42</f>
+        <f>-'Stock complet'!N42</f>
         <v/>
       </c>
     </row>
@@ -4266,7 +4418,7 @@
         <v/>
       </c>
       <c r="B13" s="34">
-        <f>'Stock complet'!F42</f>
+        <f>'Stock complet'!G42</f>
         <v/>
       </c>
     </row>
@@ -4359,7 +4511,7 @@
         </is>
       </c>
       <c r="B23" s="43">
-        <f>'Stock complet'!H42</f>
+        <f>'Stock complet'!I42</f>
         <v/>
       </c>
     </row>
@@ -4394,7 +4546,14 @@
     <row r="29">
       <c r="A29" s="44" t="inlineStr">
         <is>
-          <t>COLONNE SEUIL D'ÉQUILIBRE : ne jamais vendre en dessous. En dessous, la vente coûte de l'argent.</t>
+          <t>SEUIL D'ÉQUILIBRE : ne jamais vendre en dessous, la vente coûterait de l'argent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="39" t="inlineStr">
+        <is>
+          <t>PRIX PLANCHER : le plus bas acceptable, y compris pour la famille. 15 % au-dessus du seuil.</t>
         </is>
       </c>
     </row>
@@ -4409,7 +4568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4603,6 +4762,28 @@
       </c>
       <c r="B21" s="47" t="n">
         <v>40</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="38" t="inlineStr">
+        <is>
+          <t>PLANCHER DE NÉGOCIATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>Coefficient appliqué au seuil d'équilibre</t>
+        </is>
+      </c>
+      <c r="B24" s="48" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>prix plancher = seuil × ce coefficient</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -6229,32 +6410,32 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="48" t="inlineStr">
+      <c r="A42" s="49" t="inlineStr">
         <is>
           <t>Facture</t>
         </is>
       </c>
-      <c r="B42" s="48" t="inlineStr">
+      <c r="B42" s="49" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C42" s="48" t="inlineStr">
+      <c r="C42" s="49" t="inlineStr">
         <is>
           <t>Maison</t>
         </is>
       </c>
-      <c r="D42" s="48" t="inlineStr">
+      <c r="D42" s="49" t="inlineStr">
         <is>
           <t>Commande</t>
         </is>
       </c>
-      <c r="E42" s="48" t="inlineStr">
+      <c r="E42" s="49" t="inlineStr">
         <is>
           <t>Désignation</t>
         </is>
       </c>
-      <c r="F42" s="48" t="inlineStr">
+      <c r="F42" s="49" t="inlineStr">
         <is>
           <t>Total TTC</t>
         </is>

</xml_diff>

<commit_message>
stock: plancher de negociation a 30 % au-dessus du seuil
Retour a un coefficient seul apres essai d'une condition combinee avec
25 EUR de marge minimale : celle-ci classait 12 lots sur 28 comme
invendables, dont huit qui rapportent reellement 18 a 24 EUR. Refuser
cet argent sur du stock deja paye n'a pas de sens.

Distinction posee dans la checklist : le seuil de 25 EUR sert a decider
d'ACHETER, le prix plancher a decider de VENDRE. Sur du stock deja paye,
seul le second compte.

A 1,30, six lots restent sous leur plancher — exactement les mauvais
achats de sport et le short ba&sh.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-stock.xlsx
+++ b/exports/maison-nsaia-stock.xlsx
@@ -4303,7 +4303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -4553,7 +4553,14 @@
     <row r="30">
       <c r="A30" s="39" t="inlineStr">
         <is>
-          <t>PRIX PLANCHER : le plus bas acceptable, y compris pour la famille. 15 % au-dessus du seuil.</t>
+          <t>PRIX PLANCHER : 30 % au-dessus du seuil. Le plus bas acceptable, famille comprise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Ne pas confondre avec le seuil de sourcing de 25 € : celui-là sert à decider d'ACHETER, pas de vendre.</t>
         </is>
       </c>
     </row>
@@ -4774,15 +4781,15 @@
     <row r="24">
       <c r="A24" s="39" t="inlineStr">
         <is>
-          <t>Coefficient appliqué au seuil d'équilibre</t>
+          <t>Coefficient sur le seuil d'équilibre</t>
         </is>
       </c>
       <c r="B24" s="48" t="n">
-        <v>1.15</v>
+        <v>1.3</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>prix plancher = seuil × ce coefficient</t>
+          <t>plancher = seuil × ce coefficient</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
stock: toupies Beyblade a 49 EUR le lot de quatre
Marche releve : QuadDrive Starter Pack autour de 15 EUR piece neuve,
soit ~60 EUR les quatre. A 49 EUR l'acheteur economise 18 %.

Lot n°159 : marge 21,38 EUR. Lot n°299 : 2,21 EUR — il a ete paye le
double pour un contenu identique.

Regle ajoutee a la checklist : dans une meme vacation, deux lots
identiques peuvent partir du simple au double. Parcourir le catalogue a
la recherche d'un lot jumeau avant d'encherir.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-stock.xlsx
+++ b/exports/maison-nsaia-stock.xlsx
@@ -140,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -170,7 +170,6 @@
     <xf numFmtId="165" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2577,116 +2576,116 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>GEOX baskets P.35 — neuves</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="n">
-        <v>21.73</v>
-      </c>
-      <c r="C25" s="6">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>Lot de 4 toupies BEYBLADE HASBRO</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="n">
+        <v>19.17</v>
+      </c>
+      <c r="C25" s="25">
         <f>$B25+$Y25*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="26">
         <f>$C25/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="25">
         <f>CEILING($D25*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F25" s="8" t="n">
+      <c r="F25" s="27" t="n">
         <v>49</v>
       </c>
-      <c r="G25" s="8">
+      <c r="G25" s="27">
         <f>IF($F25="","",$F25-$C25-$M25-$N25)</f>
         <v/>
       </c>
-      <c r="H25" s="9">
+      <c r="H25" s="28">
         <f>IF($G25="","",$G25/$C25)</f>
         <v/>
       </c>
-      <c r="I25" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" s="6">
+      <c r="I25" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="J25" s="25">
         <f>$C25/$I25</f>
         <v/>
       </c>
-      <c r="K25" s="6">
+      <c r="K25" s="25">
         <f>IF($F25="","",$F25/$I25)</f>
         <v/>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="25">
         <f>IF($G25="","",$G25/$I25)</f>
         <v/>
       </c>
-      <c r="M25" s="7">
+      <c r="M25" s="26">
         <f>IF($F25="","",$F25*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N25" s="6" t="n">
+      <c r="N25" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="O25" s="11" t="n">
-        <v>17</v>
-      </c>
-      <c r="P25" s="11" t="n">
-        <v>4.42</v>
-      </c>
-      <c r="Q25" s="12" t="inlineStr">
-        <is>
-          <t>ADN Lyon</t>
-        </is>
-      </c>
-      <c r="R25" s="12" t="inlineStr">
+      <c r="O25" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="P25" s="30" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="Q25" s="31" t="inlineStr">
+        <is>
+          <t>ADN Le Mans</t>
+        </is>
+      </c>
+      <c r="R25" s="31" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="S25" s="12" t="inlineStr">
-        <is>
-          <t>FB2026-6023</t>
-        </is>
-      </c>
-      <c r="T25" s="12" t="inlineStr">
-        <is>
-          <t>155</t>
-        </is>
-      </c>
-      <c r="U25" s="4" t="inlineStr">
-        <is>
-          <t>Leboncoin + eBay</t>
-        </is>
-      </c>
-      <c r="V25" s="4" t="inlineStr"/>
-      <c r="W25" s="4" t="inlineStr">
+      <c r="S25" s="31" t="inlineStr">
+        <is>
+          <t>FB2026-44192</t>
+        </is>
+      </c>
+      <c r="T25" s="31" t="inlineStr">
+        <is>
+          <t>159</t>
+        </is>
+      </c>
+      <c r="U25" s="23" t="inlineStr">
+        <is>
+          <t>Leboncoin + eBay, en lot</t>
+        </is>
+      </c>
+      <c r="V25" s="23" t="inlineStr"/>
+      <c r="W25" s="23" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="X25" s="4" t="inlineStr"/>
-      <c r="Y25" s="4" t="n">
+      <c r="X25" s="23" t="inlineStr"/>
+      <c r="Y25" s="23" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Short BA&amp;SH Fegor T.34 — neuf</t>
+          <t>GEOX baskets P.35 — neuves</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>50.4</v>
+        <v>21.73</v>
       </c>
       <c r="C26" s="6">
         <f>$B26+$Y26*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D26" s="7">
-        <f>$C26/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
+        <f>$C26/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
       <c r="E26" s="6">
@@ -2694,7 +2693,7 @@
         <v/>
       </c>
       <c r="F26" s="8" t="n">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="G26" s="8">
         <f>IF($F26="","",$F26-$C26-$M26-$N26)</f>
@@ -2723,45 +2722,44 @@
         <f>IF($F26="","",$F26*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N26" s="6">
-        <f>IF($F26="","",$F26*Paramètres!$B$7)</f>
-        <v/>
+      <c r="N26" s="6" t="n">
+        <v>0</v>
       </c>
       <c r="O26" s="11" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="P26" s="11" t="n">
-        <v>10.4</v>
+        <v>4.42</v>
       </c>
       <c r="Q26" s="12" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="R26" s="12" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="S26" s="12" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>FB2026-6023</t>
         </is>
       </c>
       <c r="T26" s="12" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>155</t>
         </is>
       </c>
       <c r="U26" s="4" t="inlineStr">
         <is>
-          <t>Boutique</t>
+          <t>Leboncoin + eBay</t>
         </is>
       </c>
       <c r="V26" s="4" t="inlineStr"/>
       <c r="W26" s="4" t="inlineStr">
         <is>
-          <t>URGENT — saisonnier</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="X26" s="4" t="inlineStr"/>
@@ -2772,18 +2770,18 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>NEW BALANCE G19064IK Alkaline Green P.38½ — neuves avec boîte</t>
+          <t>Short BA&amp;SH Fegor T.34 — neuf</t>
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>75.59999999999999</v>
+        <v>50.4</v>
       </c>
       <c r="C27" s="6">
         <f>$B27+$Y27*Paramètres!$B$13</f>
         <v/>
       </c>
       <c r="D27" s="7">
-        <f>$C27/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
+        <f>$C27/(1-Paramètres!$B$5-Paramètres!$B$6-Paramètres!$B$7)</f>
         <v/>
       </c>
       <c r="E27" s="6">
@@ -2791,7 +2789,7 @@
         <v/>
       </c>
       <c r="F27" s="8" t="n">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="G27" s="8">
         <f>IF($F27="","",$F27-$C27-$M27-$N27)</f>
@@ -2820,14 +2818,15 @@
         <f>IF($F27="","",$F27*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N27" s="6" t="n">
-        <v>0</v>
+      <c r="N27" s="6">
+        <f>IF($F27="","",$F27*Paramètres!$B$7)</f>
+        <v/>
       </c>
       <c r="O27" s="11" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="P27" s="11" t="n">
-        <v>15.6</v>
+        <v>10.4</v>
       </c>
       <c r="Q27" s="12" t="inlineStr">
         <is>
@@ -2846,18 +2845,18 @@
       </c>
       <c r="T27" s="12" t="inlineStr">
         <is>
-          <t>199</t>
+          <t>408</t>
         </is>
       </c>
       <c r="U27" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin</t>
+          <t>Boutique</t>
         </is>
       </c>
       <c r="V27" s="4" t="inlineStr"/>
       <c r="W27" s="4" t="inlineStr">
         <is>
-          <t>Liquider</t>
+          <t>URGENT — saisonnier</t>
         </is>
       </c>
       <c r="X27" s="4" t="inlineStr"/>
@@ -2866,209 +2865,209 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>NEW BALANCE G19064IK Alkaline Green P.38½ — neuves avec boîte</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>75.59999999999999</v>
+      </c>
+      <c r="C28" s="6">
+        <f>$B28+$Y28*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D28" s="7">
+        <f>$C28/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
+        <v/>
+      </c>
+      <c r="E28" s="6">
+        <f>CEILING($D28*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F28" s="8" t="n">
+        <v>99</v>
+      </c>
+      <c r="G28" s="8">
+        <f>IF($F28="","",$F28-$C28-$M28-$N28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="9">
+        <f>IF($G28="","",$G28/$C28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" s="6">
+        <f>$C28/$I28</f>
+        <v/>
+      </c>
+      <c r="K28" s="6">
+        <f>IF($F28="","",$F28/$I28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="6">
+        <f>IF($G28="","",$G28/$I28)</f>
+        <v/>
+      </c>
+      <c r="M28" s="7">
+        <f>IF($F28="","",$F28*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="P28" s="11" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="Q28" s="12" t="inlineStr">
+        <is>
+          <t>ADN Le Mans</t>
+        </is>
+      </c>
+      <c r="R28" s="12" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="S28" s="12" t="inlineStr">
+        <is>
+          <t>FB2026-43716</t>
+        </is>
+      </c>
+      <c r="T28" s="12" t="inlineStr">
+        <is>
+          <t>199</t>
+        </is>
+      </c>
+      <c r="U28" s="4" t="inlineStr">
+        <is>
+          <t>Leboncoin</t>
+        </is>
+      </c>
+      <c r="V28" s="4" t="inlineStr"/>
+      <c r="W28" s="4" t="inlineStr">
+        <is>
+          <t>Liquider</t>
+        </is>
+      </c>
+      <c r="X28" s="4" t="inlineStr"/>
+      <c r="Y28" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>SALOMON X Ultra 5 Mid GTX P.44 — neuves</t>
         </is>
       </c>
-      <c r="B28" s="15" t="n">
+      <c r="B29" s="15" t="n">
         <v>76.68000000000001</v>
       </c>
-      <c r="C28" s="16">
-        <f>$B28+$Y28*Paramètres!$B$13</f>
-        <v/>
-      </c>
-      <c r="D28" s="17">
-        <f>$C28/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
-        <v/>
-      </c>
-      <c r="E28" s="16">
-        <f>CEILING($D28*Paramètres!$B$24,1)</f>
-        <v/>
-      </c>
-      <c r="F28" s="18" t="n">
+      <c r="C29" s="16">
+        <f>$B29+$Y29*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D29" s="17">
+        <f>$C29/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
+        <v/>
+      </c>
+      <c r="E29" s="16">
+        <f>CEILING($D29*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F29" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="G28" s="18">
-        <f>IF($F28="","",$F28-$C28-$M28-$N28)</f>
-        <v/>
-      </c>
-      <c r="H28" s="19">
-        <f>IF($G28="","",$G28/$C28)</f>
-        <v/>
-      </c>
-      <c r="I28" s="20" t="n">
+      <c r="G29" s="18">
+        <f>IF($F29="","",$F29-$C29-$M29-$N29)</f>
+        <v/>
+      </c>
+      <c r="H29" s="19">
+        <f>IF($G29="","",$G29/$C29)</f>
+        <v/>
+      </c>
+      <c r="I29" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="J28" s="16">
-        <f>$C28/$I28</f>
-        <v/>
-      </c>
-      <c r="K28" s="16">
-        <f>IF($F28="","",$F28/$I28)</f>
-        <v/>
-      </c>
-      <c r="L28" s="16">
-        <f>IF($G28="","",$G28/$I28)</f>
-        <v/>
-      </c>
-      <c r="M28" s="17">
-        <f>IF($F28="","",$F28*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="N28" s="16" t="n">
+      <c r="J29" s="16">
+        <f>$C29/$I29</f>
+        <v/>
+      </c>
+      <c r="K29" s="16">
+        <f>IF($F29="","",$F29/$I29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="16">
+        <f>IF($G29="","",$G29/$I29)</f>
+        <v/>
+      </c>
+      <c r="M29" s="17">
+        <f>IF($F29="","",$F29*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N29" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="O28" s="21" t="n">
+      <c r="O29" s="21" t="n">
         <v>60</v>
       </c>
-      <c r="P28" s="21" t="n">
+      <c r="P29" s="21" t="n">
         <v>15.6</v>
       </c>
-      <c r="Q28" s="22" t="inlineStr">
+      <c r="Q29" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="R28" s="22" t="inlineStr">
+      <c r="R29" s="22" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="S28" s="22" t="inlineStr">
+      <c r="S29" s="22" t="inlineStr">
         <is>
           <t>FB2026-44192</t>
         </is>
       </c>
-      <c r="T28" s="22" t="inlineStr">
+      <c r="T29" s="22" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="U28" s="14" t="inlineStr">
+      <c r="U29" s="14" t="inlineStr">
         <is>
           <t>Vinted, acheteur en Italie</t>
         </is>
       </c>
-      <c r="V28" s="14" t="inlineStr"/>
-      <c r="W28" s="14" t="inlineStr">
+      <c r="V29" s="14" t="inlineStr"/>
+      <c r="W29" s="14" t="inlineStr">
         <is>
           <t>VENDUE</t>
         </is>
       </c>
-      <c r="X28" s="14" t="inlineStr">
+      <c r="X29" s="14" t="inlineStr">
         <is>
           <t>12/08/2026</t>
         </is>
       </c>
-      <c r="Y28" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>EMPORIO ARMANI baskets P.36 — neuves</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="n">
-        <v>51.12</v>
-      </c>
-      <c r="C29" s="6">
-        <f>$B29+$Y29*Paramètres!$B$13</f>
-        <v/>
-      </c>
-      <c r="D29" s="7">
-        <f>$C29/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
-        <v/>
-      </c>
-      <c r="E29" s="6">
-        <f>CEILING($D29*Paramètres!$B$24,1)</f>
-        <v/>
-      </c>
-      <c r="F29" s="8" t="n">
-        <v>69</v>
-      </c>
-      <c r="G29" s="8">
-        <f>IF($F29="","",$F29-$C29-$M29-$N29)</f>
-        <v/>
-      </c>
-      <c r="H29" s="9">
-        <f>IF($G29="","",$G29/$C29)</f>
-        <v/>
-      </c>
-      <c r="I29" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J29" s="6">
-        <f>$C29/$I29</f>
-        <v/>
-      </c>
-      <c r="K29" s="6">
-        <f>IF($F29="","",$F29/$I29)</f>
-        <v/>
-      </c>
-      <c r="L29" s="6">
-        <f>IF($G29="","",$G29/$I29)</f>
-        <v/>
-      </c>
-      <c r="M29" s="7">
-        <f>IF($F29="","",$F29*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="N29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="P29" s="11" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="Q29" s="12" t="inlineStr">
-        <is>
-          <t>ADN Lyon</t>
-        </is>
-      </c>
-      <c r="R29" s="12" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="S29" s="12" t="inlineStr">
-        <is>
-          <t>FB2026-6023</t>
-        </is>
-      </c>
-      <c r="T29" s="12" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="U29" s="4" t="inlineStr">
-        <is>
-          <t>Leboncoin</t>
-        </is>
-      </c>
-      <c r="V29" s="4" t="inlineStr"/>
-      <c r="W29" s="4" t="inlineStr">
-        <is>
-          <t>Liquider</t>
-        </is>
-      </c>
-      <c r="X29" s="4" t="inlineStr"/>
-      <c r="Y29" s="4" t="n">
+      <c r="Y29" s="14" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>NEW BALANCE sneakers P.38 — neuves</t>
+          <t>EMPORIO ARMANI baskets P.36 — neuves</t>
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>38.34</v>
+        <v>51.12</v>
       </c>
       <c r="C30" s="6">
         <f>$B30+$Y30*Paramètres!$B$13</f>
@@ -3083,7 +3082,7 @@
         <v/>
       </c>
       <c r="F30" s="8" t="n">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="G30" s="8">
         <f>IF($F30="","",$F30-$C30-$M30-$N30)</f>
@@ -3116,10 +3115,10 @@
         <v>0</v>
       </c>
       <c r="O30" s="11" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="P30" s="11" t="n">
-        <v>7.8</v>
+        <v>10.4</v>
       </c>
       <c r="Q30" s="12" t="inlineStr">
         <is>
@@ -3138,7 +3137,7 @@
       </c>
       <c r="T30" s="12" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>150</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
@@ -3160,11 +3159,11 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>NEW BALANCE baskets montantes P.44 — neuves</t>
+          <t>NEW BALANCE sneakers P.38 — neuves</t>
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>51.12</v>
+        <v>38.34</v>
       </c>
       <c r="C31" s="6">
         <f>$B31+$Y31*Paramètres!$B$13</f>
@@ -3179,7 +3178,7 @@
         <v/>
       </c>
       <c r="F31" s="8" t="n">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="G31" s="8">
         <f>IF($F31="","",$F31-$C31-$M31-$N31)</f>
@@ -3212,10 +3211,10 @@
         <v>0</v>
       </c>
       <c r="O31" s="11" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="P31" s="11" t="n">
-        <v>10.4</v>
+        <v>7.8</v>
       </c>
       <c r="Q31" s="12" t="inlineStr">
         <is>
@@ -3234,7 +3233,7 @@
       </c>
       <c r="T31" s="12" t="inlineStr">
         <is>
-          <t>156</t>
+          <t>114</t>
         </is>
       </c>
       <c r="U31" s="4" t="inlineStr">
@@ -3256,11 +3255,11 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>TOMMY JEANS baskets basses P.40 — neuves</t>
+          <t>NEW BALANCE baskets montantes P.44 — neuves</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>52.4</v>
+        <v>51.12</v>
       </c>
       <c r="C32" s="6">
         <f>$B32+$Y32*Paramètres!$B$13</f>
@@ -3308,10 +3307,10 @@
         <v>0</v>
       </c>
       <c r="O32" s="11" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P32" s="11" t="n">
-        <v>10.66</v>
+        <v>10.4</v>
       </c>
       <c r="Q32" s="12" t="inlineStr">
         <is>
@@ -3330,12 +3329,12 @@
       </c>
       <c r="T32" s="12" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>156</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
+          <t>Leboncoin</t>
         </is>
       </c>
       <c r="V32" s="4" t="inlineStr"/>
@@ -3350,113 +3349,109 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>LACOSTE sneakers P.42 — neuves</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n">
-        <v>57.51</v>
-      </c>
-      <c r="C33" s="16">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>TOMMY JEANS baskets basses P.40 — neuves</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="C33" s="6">
         <f>$B33+$Y33*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="7">
         <f>$C33/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E33" s="16">
+      <c r="E33" s="6">
         <f>CEILING($D33*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F33" s="18" t="n">
-        <v>70</v>
-      </c>
-      <c r="G33" s="18">
+      <c r="F33" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="G33" s="8">
         <f>IF($F33="","",$F33-$C33-$M33-$N33)</f>
         <v/>
       </c>
-      <c r="H33" s="19">
+      <c r="H33" s="9">
         <f>IF($G33="","",$G33/$C33)</f>
         <v/>
       </c>
-      <c r="I33" s="20" t="n">
+      <c r="I33" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J33" s="16">
+      <c r="J33" s="6">
         <f>$C33/$I33</f>
         <v/>
       </c>
-      <c r="K33" s="16">
+      <c r="K33" s="6">
         <f>IF($F33="","",$F33/$I33)</f>
         <v/>
       </c>
-      <c r="L33" s="16">
+      <c r="L33" s="6">
         <f>IF($G33="","",$G33/$I33)</f>
         <v/>
       </c>
-      <c r="M33" s="17">
+      <c r="M33" s="7">
         <f>IF($F33="","",$F33*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N33" s="16" t="n">
+      <c r="N33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O33" s="21" t="n">
-        <v>45</v>
-      </c>
-      <c r="P33" s="21" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="Q33" s="22" t="inlineStr">
+      <c r="O33" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="P33" s="11" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="Q33" s="12" t="inlineStr">
         <is>
           <t>ADN Lyon</t>
         </is>
       </c>
-      <c r="R33" s="22" t="inlineStr">
+      <c r="R33" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="S33" s="22" t="inlineStr">
+      <c r="S33" s="12" t="inlineStr">
         <is>
           <t>FB2026-6023</t>
         </is>
       </c>
-      <c r="T33" s="22" t="inlineStr">
-        <is>
-          <t>141</t>
-        </is>
-      </c>
-      <c r="U33" s="14" t="inlineStr">
-        <is>
-          <t>date à compléter</t>
-        </is>
-      </c>
-      <c r="V33" s="14" t="inlineStr"/>
-      <c r="W33" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="X33" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="Y33" s="14" t="n">
+      <c r="T33" s="12" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="U33" s="4" t="inlineStr">
+        <is>
+          <t>Leboncoin + eBay</t>
+        </is>
+      </c>
+      <c r="V33" s="4" t="inlineStr"/>
+      <c r="W33" s="4" t="inlineStr">
+        <is>
+          <t>Liquider</t>
+        </is>
+      </c>
+      <c r="X33" s="4" t="inlineStr"/>
+      <c r="Y33" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>T-shirt BALENCIAGA T.2 — neuf</t>
+          <t>LACOSTE sneakers P.42 — neuves</t>
         </is>
       </c>
       <c r="B34" s="15" t="n">
-        <v>113.4</v>
+        <v>57.51</v>
       </c>
       <c r="C34" s="16">
         <f>$B34+$Y34*Paramètres!$B$13</f>
@@ -3471,7 +3466,7 @@
         <v/>
       </c>
       <c r="F34" s="18" t="n">
-        <v>125</v>
+        <v>70</v>
       </c>
       <c r="G34" s="18">
         <f>IF($F34="","",$F34-$C34-$M34-$N34)</f>
@@ -3504,14 +3499,14 @@
         <v>0</v>
       </c>
       <c r="O34" s="21" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="P34" s="21" t="n">
-        <v>23.4</v>
+        <v>11.7</v>
       </c>
       <c r="Q34" s="22" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="R34" s="22" t="inlineStr">
@@ -3521,12 +3516,12 @@
       </c>
       <c r="S34" s="22" t="inlineStr">
         <is>
-          <t>FB2026-44194</t>
+          <t>FB2026-6023</t>
         </is>
       </c>
       <c r="T34" s="22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>141</t>
         </is>
       </c>
       <c r="U34" s="14" t="inlineStr">
@@ -3552,11 +3547,11 @@
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>Veste en jean ARMANI EXCHANGE T.S — neuve</t>
+          <t>T-shirt BALENCIAGA T.2 — neuf</t>
         </is>
       </c>
       <c r="B35" s="15" t="n">
-        <v>25.2</v>
+        <v>113.4</v>
       </c>
       <c r="C35" s="16">
         <f>$B35+$Y35*Paramètres!$B$13</f>
@@ -3571,7 +3566,7 @@
         <v/>
       </c>
       <c r="F35" s="18" t="n">
-        <v>35</v>
+        <v>125</v>
       </c>
       <c r="G35" s="18">
         <f>IF($F35="","",$F35-$C35-$M35-$N35)</f>
@@ -3604,10 +3599,10 @@
         <v>0</v>
       </c>
       <c r="O35" s="21" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="P35" s="21" t="n">
-        <v>5.2</v>
+        <v>23.4</v>
       </c>
       <c r="Q35" s="22" t="inlineStr">
         <is>
@@ -3616,17 +3611,17 @@
       </c>
       <c r="R35" s="22" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="S35" s="22" t="inlineStr">
         <is>
-          <t>FB2026-43717</t>
+          <t>FB2026-44194</t>
         </is>
       </c>
       <c r="T35" s="22" t="inlineStr">
         <is>
-          <t>168</t>
+          <t>9</t>
         </is>
       </c>
       <c r="U35" s="14" t="inlineStr">
@@ -3650,113 +3645,109 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>Baskets NIKE Air Max Moto 2K P.44.5 — neuves</t>
-        </is>
-      </c>
-      <c r="B36" s="15" t="n">
-        <v>50.4</v>
-      </c>
-      <c r="C36" s="16">
+      <c r="A36" s="23" t="inlineStr">
+        <is>
+          <t>Lot de 4 toupies BEYBLADE HASBRO</t>
+        </is>
+      </c>
+      <c r="B36" s="24" t="n">
+        <v>38.34</v>
+      </c>
+      <c r="C36" s="25">
         <f>$B36+$Y36*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D36" s="17">
+      <c r="D36" s="26">
         <f>$C36/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E36" s="16">
+      <c r="E36" s="25">
         <f>CEILING($D36*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F36" s="18" t="n">
-        <v>60</v>
-      </c>
-      <c r="G36" s="18">
+      <c r="F36" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="G36" s="27">
         <f>IF($F36="","",$F36-$C36-$M36-$N36)</f>
         <v/>
       </c>
-      <c r="H36" s="19">
+      <c r="H36" s="28">
         <f>IF($G36="","",$G36/$C36)</f>
         <v/>
       </c>
-      <c r="I36" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J36" s="16">
+      <c r="I36" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="J36" s="25">
         <f>$C36/$I36</f>
         <v/>
       </c>
-      <c r="K36" s="16">
+      <c r="K36" s="25">
         <f>IF($F36="","",$F36/$I36)</f>
         <v/>
       </c>
-      <c r="L36" s="16">
+      <c r="L36" s="25">
         <f>IF($G36="","",$G36/$I36)</f>
         <v/>
       </c>
-      <c r="M36" s="17">
+      <c r="M36" s="26">
         <f>IF($F36="","",$F36*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N36" s="16" t="n">
+      <c r="N36" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="O36" s="21" t="n">
-        <v>40</v>
-      </c>
-      <c r="P36" s="21" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="Q36" s="22" t="inlineStr">
+      <c r="O36" s="30" t="n">
+        <v>30</v>
+      </c>
+      <c r="P36" s="30" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Q36" s="31" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="R36" s="22" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="S36" s="22" t="inlineStr">
-        <is>
-          <t>FB2026-43716</t>
-        </is>
-      </c>
-      <c r="T36" s="22" t="inlineStr">
-        <is>
-          <t>170</t>
-        </is>
-      </c>
-      <c r="U36" s="14" t="inlineStr">
-        <is>
-          <t>date à compléter</t>
-        </is>
-      </c>
-      <c r="V36" s="14" t="inlineStr"/>
-      <c r="W36" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="X36" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="Y36" s="14" t="n">
+      <c r="R36" s="31" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="S36" s="31" t="inlineStr">
+        <is>
+          <t>FB2026-44192</t>
+        </is>
+      </c>
+      <c r="T36" s="31" t="inlineStr">
+        <is>
+          <t>299</t>
+        </is>
+      </c>
+      <c r="U36" s="23" t="inlineStr">
+        <is>
+          <t>Leboncoin + eBay, en lot</t>
+        </is>
+      </c>
+      <c r="V36" s="23" t="inlineStr"/>
+      <c r="W36" s="23" t="inlineStr">
+        <is>
+          <t>Marge faible</t>
+        </is>
+      </c>
+      <c r="X36" s="23" t="inlineStr"/>
+      <c r="Y36" s="23" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>Sac demi-lune nylon noir KARL LAGERFELD JEANS — neuf avec étiquette</t>
+          <t>Veste en jean ARMANI EXCHANGE T.S — neuve</t>
         </is>
       </c>
       <c r="B37" s="15" t="n">
-        <v>50.4</v>
+        <v>25.2</v>
       </c>
       <c r="C37" s="16">
         <f>$B37+$Y37*Paramètres!$B$13</f>
@@ -3771,7 +3762,7 @@
         <v/>
       </c>
       <c r="F37" s="18" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="G37" s="18">
         <f>IF($F37="","",$F37-$C37-$M37-$N37)</f>
@@ -3804,10 +3795,10 @@
         <v>0</v>
       </c>
       <c r="O37" s="21" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="P37" s="21" t="n">
-        <v>10.4</v>
+        <v>5.2</v>
       </c>
       <c r="Q37" s="22" t="inlineStr">
         <is>
@@ -3821,12 +3812,12 @@
       </c>
       <c r="S37" s="22" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>FB2026-43717</t>
         </is>
       </c>
       <c r="T37" s="22" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>168</t>
         </is>
       </c>
       <c r="U37" s="14" t="inlineStr">
@@ -3852,11 +3843,11 @@
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>Baskets HOKA P.37 1/3 — neuves</t>
+          <t>Baskets NIKE Air Max Moto 2K P.44.5 — neuves</t>
         </is>
       </c>
       <c r="B38" s="15" t="n">
-        <v>63</v>
+        <v>50.4</v>
       </c>
       <c r="C38" s="16">
         <f>$B38+$Y38*Paramètres!$B$13</f>
@@ -3871,7 +3862,7 @@
         <v/>
       </c>
       <c r="F38" s="18" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="G38" s="18">
         <f>IF($F38="","",$F38-$C38-$M38-$N38)</f>
@@ -3904,10 +3895,10 @@
         <v>0</v>
       </c>
       <c r="O38" s="21" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="P38" s="21" t="n">
-        <v>13</v>
+        <v>10.4</v>
       </c>
       <c r="Q38" s="22" t="inlineStr">
         <is>
@@ -3926,7 +3917,7 @@
       </c>
       <c r="T38" s="22" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>170</t>
         </is>
       </c>
       <c r="U38" s="14" t="inlineStr">
@@ -3950,190 +3941,202 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="23" t="inlineStr">
-        <is>
-          <t>Lot de 4 toupies BEYBLADE HASBRO</t>
-        </is>
-      </c>
-      <c r="B39" s="24" t="n">
-        <v>19.17</v>
-      </c>
-      <c r="C39" s="25">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Sac demi-lune nylon noir KARL LAGERFELD JEANS — neuf avec étiquette</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="C39" s="16">
         <f>$B39+$Y39*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D39" s="26">
+      <c r="D39" s="17">
         <f>$C39/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E39" s="25">
+      <c r="E39" s="16">
         <f>CEILING($D39*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F39" s="27" t="n"/>
-      <c r="G39" s="28">
+      <c r="F39" s="18" t="n">
+        <v>60</v>
+      </c>
+      <c r="G39" s="18">
         <f>IF($F39="","",$F39-$C39-$M39-$N39)</f>
         <v/>
       </c>
-      <c r="H39" s="29">
+      <c r="H39" s="19">
         <f>IF($G39="","",$G39/$C39)</f>
         <v/>
       </c>
-      <c r="I39" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="J39" s="25">
+      <c r="I39" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J39" s="16">
         <f>$C39/$I39</f>
         <v/>
       </c>
-      <c r="K39" s="25">
+      <c r="K39" s="16">
         <f>IF($F39="","",$F39/$I39)</f>
         <v/>
       </c>
-      <c r="L39" s="25">
+      <c r="L39" s="16">
         <f>IF($G39="","",$G39/$I39)</f>
         <v/>
       </c>
-      <c r="M39" s="26">
+      <c r="M39" s="17">
         <f>IF($F39="","",$F39*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N39" s="25" t="n">
+      <c r="N39" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="O39" s="31" t="n">
-        <v>15</v>
-      </c>
-      <c r="P39" s="31" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="Q39" s="32" t="inlineStr">
+      <c r="O39" s="21" t="n">
+        <v>40</v>
+      </c>
+      <c r="P39" s="21" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="Q39" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="R39" s="32" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="S39" s="32" t="inlineStr">
-        <is>
-          <t>FB2026-44192</t>
-        </is>
-      </c>
-      <c r="T39" s="32" t="inlineStr">
-        <is>
-          <t>159</t>
-        </is>
-      </c>
-      <c r="U39" s="23" t="inlineStr">
-        <is>
-          <t>Leboncoin + eBay</t>
-        </is>
-      </c>
-      <c r="V39" s="23" t="inlineStr"/>
-      <c r="W39" s="23" t="inlineStr">
-        <is>
-          <t>PRIX À ÉTABLIR</t>
-        </is>
-      </c>
-      <c r="X39" s="23" t="inlineStr"/>
-      <c r="Y39" s="23" t="n">
+      <c r="R39" s="22" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="S39" s="22" t="inlineStr">
+        <is>
+          <t>FB2026-43716</t>
+        </is>
+      </c>
+      <c r="T39" s="22" t="inlineStr">
+        <is>
+          <t>431</t>
+        </is>
+      </c>
+      <c r="U39" s="14" t="inlineStr">
+        <is>
+          <t>date à compléter</t>
+        </is>
+      </c>
+      <c r="V39" s="14" t="inlineStr"/>
+      <c r="W39" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="X39" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="Y39" s="14" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="23" t="inlineStr">
-        <is>
-          <t>Lot de 4 toupies BEYBLADE HASBRO</t>
-        </is>
-      </c>
-      <c r="B40" s="24" t="n">
-        <v>38.34</v>
-      </c>
-      <c r="C40" s="25">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>Baskets HOKA P.37 1/3 — neuves</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="n">
+        <v>63</v>
+      </c>
+      <c r="C40" s="16">
         <f>$B40+$Y40*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D40" s="26">
+      <c r="D40" s="17">
         <f>$C40/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E40" s="25">
+      <c r="E40" s="16">
         <f>CEILING($D40*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F40" s="27" t="n"/>
-      <c r="G40" s="28">
+      <c r="F40" s="18" t="n">
+        <v>70</v>
+      </c>
+      <c r="G40" s="18">
         <f>IF($F40="","",$F40-$C40-$M40-$N40)</f>
         <v/>
       </c>
-      <c r="H40" s="29">
+      <c r="H40" s="19">
         <f>IF($G40="","",$G40/$C40)</f>
         <v/>
       </c>
-      <c r="I40" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="J40" s="25">
+      <c r="I40" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="16">
         <f>$C40/$I40</f>
         <v/>
       </c>
-      <c r="K40" s="25">
+      <c r="K40" s="16">
         <f>IF($F40="","",$F40/$I40)</f>
         <v/>
       </c>
-      <c r="L40" s="25">
+      <c r="L40" s="16">
         <f>IF($G40="","",$G40/$I40)</f>
         <v/>
       </c>
-      <c r="M40" s="26">
+      <c r="M40" s="17">
         <f>IF($F40="","",$F40*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N40" s="25" t="n">
+      <c r="N40" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="O40" s="31" t="n">
-        <v>30</v>
-      </c>
-      <c r="P40" s="31" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="Q40" s="32" t="inlineStr">
+      <c r="O40" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="P40" s="21" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q40" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="R40" s="32" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="S40" s="32" t="inlineStr">
-        <is>
-          <t>FB2026-44192</t>
-        </is>
-      </c>
-      <c r="T40" s="32" t="inlineStr">
-        <is>
-          <t>299</t>
-        </is>
-      </c>
-      <c r="U40" s="23" t="inlineStr">
-        <is>
-          <t>Leboncoin + eBay</t>
-        </is>
-      </c>
-      <c r="V40" s="23" t="inlineStr"/>
-      <c r="W40" s="23" t="inlineStr">
-        <is>
-          <t>PRIX À ÉTABLIR</t>
-        </is>
-      </c>
-      <c r="X40" s="23" t="inlineStr"/>
-      <c r="Y40" s="23" t="n">
+      <c r="R40" s="22" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="S40" s="22" t="inlineStr">
+        <is>
+          <t>FB2026-43716</t>
+        </is>
+      </c>
+      <c r="T40" s="22" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="U40" s="14" t="inlineStr">
+        <is>
+          <t>date à compléter</t>
+        </is>
+      </c>
+      <c r="V40" s="14" t="inlineStr"/>
+      <c r="W40" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="X40" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="Y40" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4232,59 +4235,59 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="33" t="inlineStr">
+      <c r="A42" s="32" t="inlineStr">
         <is>
           <t>TOTAL — 36 lots</t>
         </is>
       </c>
-      <c r="B42" s="34">
+      <c r="B42" s="33">
         <f>SUM(B6:B41)</f>
         <v/>
       </c>
-      <c r="C42" s="34">
+      <c r="C42" s="33">
         <f>SUM(C6:C41)</f>
         <v/>
       </c>
-      <c r="D42" s="35" t="n"/>
-      <c r="E42" s="35" t="n"/>
-      <c r="F42" s="34">
+      <c r="D42" s="34" t="n"/>
+      <c r="E42" s="34" t="n"/>
+      <c r="F42" s="33">
         <f>SUM(F6:F41)</f>
         <v/>
       </c>
-      <c r="G42" s="34">
+      <c r="G42" s="33">
         <f>SUM(G6:G41)</f>
         <v/>
       </c>
-      <c r="H42" s="36">
+      <c r="H42" s="35">
         <f>G42/C42</f>
         <v/>
       </c>
-      <c r="I42" s="37">
+      <c r="I42" s="36">
         <f>SUM(I6:I41)</f>
         <v/>
       </c>
-      <c r="J42" s="35" t="n"/>
-      <c r="K42" s="35" t="n"/>
-      <c r="L42" s="35" t="n"/>
-      <c r="M42" s="34">
+      <c r="J42" s="34" t="n"/>
+      <c r="K42" s="34" t="n"/>
+      <c r="L42" s="34" t="n"/>
+      <c r="M42" s="33">
         <f>SUM(M6:M41)</f>
         <v/>
       </c>
-      <c r="N42" s="34">
+      <c r="N42" s="33">
         <f>SUM(N6:N41)</f>
         <v/>
       </c>
-      <c r="O42" s="35" t="n"/>
-      <c r="P42" s="35" t="n"/>
-      <c r="Q42" s="35" t="n"/>
-      <c r="R42" s="35" t="n"/>
-      <c r="S42" s="35" t="n"/>
-      <c r="T42" s="35" t="n"/>
-      <c r="U42" s="35" t="n"/>
-      <c r="V42" s="35" t="n"/>
-      <c r="W42" s="35" t="n"/>
-      <c r="X42" s="35" t="n"/>
-      <c r="Y42" s="35" t="n"/>
+      <c r="O42" s="34" t="n"/>
+      <c r="P42" s="34" t="n"/>
+      <c r="Q42" s="34" t="n"/>
+      <c r="R42" s="34" t="n"/>
+      <c r="S42" s="34" t="n"/>
+      <c r="T42" s="34" t="n"/>
+      <c r="U42" s="34" t="n"/>
+      <c r="V42" s="34" t="n"/>
+      <c r="W42" s="34" t="n"/>
+      <c r="X42" s="34" t="n"/>
+      <c r="Y42" s="34" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:Y41"/>
@@ -4319,14 +4322,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="38" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
         <is>
           <t>CAPITAL ENGAGÉ</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="39" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
         <is>
           <t>Marchandise ADN</t>
         </is>
@@ -4336,7 +4339,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="39" t="inlineStr">
+      <c r="A5" s="38" t="inlineStr">
         <is>
           <t>Livraison ADN</t>
         </is>
@@ -4347,7 +4350,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="39" t="inlineStr">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>Achats hors ADN (pompes, Pokémon)</t>
         </is>
@@ -4357,25 +4360,25 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="40" t="inlineStr">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>TOTAL ENGAGÉ</t>
         </is>
       </c>
-      <c r="B7" s="34">
+      <c r="B7" s="33">
         <f>'Stock complet'!C42</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="38" t="inlineStr">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>CHIFFRE D'AFFAIRES ET MARGE</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="40" t="inlineStr">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>Chiffre d'affaires attendu</t>
         </is>
@@ -4391,7 +4394,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="39" t="inlineStr">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>− URSSAF + CFP</t>
         </is>
@@ -4402,7 +4405,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="39" t="inlineStr">
+      <c r="A12" s="38" t="inlineStr">
         <is>
           <t>− Commission carte</t>
         </is>
@@ -4413,17 +4416,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="40">
+      <c r="A13" s="39">
         <f> Marge brute</f>
         <v/>
       </c>
-      <c r="B13" s="34">
+      <c r="B13" s="33">
         <f>'Stock complet'!G42</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="39" t="inlineStr">
+      <c r="A14" s="38" t="inlineStr">
         <is>
           <t>− Emballage</t>
         </is>
@@ -4434,7 +4437,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="39" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
         <is>
           <t>− Frais fixe carte</t>
         </is>
@@ -4445,17 +4448,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="40">
+      <c r="A16" s="39">
         <f> Marge avant impôt</f>
         <v/>
       </c>
-      <c r="B16" s="34">
+      <c r="B16" s="33">
         <f>B13+B14+B15</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="39" t="inlineStr">
+      <c r="A17" s="38" t="inlineStr">
         <is>
           <t>Base imposable</t>
         </is>
@@ -4466,7 +4469,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="39" t="inlineStr">
+      <c r="A18" s="38" t="inlineStr">
         <is>
           <t>− Impôt estimé</t>
         </is>
@@ -4477,81 +4480,81 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="40">
+      <c r="A19" s="39">
         <f> CE QUI RESTE</f>
         <v/>
       </c>
-      <c r="B19" s="41">
+      <c r="B19" s="40">
         <f>B16+B18</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="38" t="inlineStr">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t>RENDEMENT</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="39" t="inlineStr">
+      <c r="A22" s="38" t="inlineStr">
         <is>
           <t>Marge nette / capital engagé</t>
         </is>
       </c>
-      <c r="B22" s="42">
+      <c r="B22" s="41">
         <f>B19/B7</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="39" t="inlineStr">
+      <c r="A23" s="38" t="inlineStr">
         <is>
           <t>Articles physiques</t>
         </is>
       </c>
-      <c r="B23" s="43">
+      <c r="B23" s="42">
         <f>'Stock complet'!I42</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="38" t="inlineStr">
+      <c r="A25" s="37" t="inlineStr">
         <is>
           <t>À FAIRE</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="39" t="inlineStr">
-        <is>
-          <t>3 lots sans prix : Yeezy 700 V3 et les deux lots de toupies Beyblade.</t>
+      <c r="A26" s="38" t="inlineStr">
+        <is>
+          <t>1 lot sans prix : Yeezy 700 V3, en attente d'authentification.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="39" t="inlineStr">
+      <c r="A27" s="38" t="inlineStr">
         <is>
           <t>Dates de vente à compléter sur les 6 ventes récentes.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="39" t="inlineStr">
+      <c r="A28" s="38" t="inlineStr">
         <is>
           <t>Facture manquante : lot n°84, les 2 pompes Robby.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="44" t="inlineStr">
+      <c r="A29" s="43" t="inlineStr">
         <is>
           <t>SEUIL D'ÉQUILIBRE : ne jamais vendre en dessous, la vente coûterait de l'argent.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="39" t="inlineStr">
+      <c r="A30" s="38" t="inlineStr">
         <is>
           <t>PRIX PLANCHER : 30 % au-dessus du seuil. Le plus bas acceptable, famille comprise.</t>
         </is>
@@ -4598,19 +4601,19 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>CHARGES SUR LE CHIFFRE D'AFFAIRES</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="39" t="inlineStr">
+      <c r="A5" s="38" t="inlineStr">
         <is>
           <t>Cotisations URSSAF (achat-revente BIC)</t>
         </is>
       </c>
-      <c r="B5" s="45" t="n">
+      <c r="B5" s="44" t="n">
         <v>0.123</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -4620,22 +4623,22 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="39" t="inlineStr">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>CFP — formation professionnelle</t>
         </is>
       </c>
-      <c r="B6" s="45" t="n">
+      <c r="B6" s="44" t="n">
         <v>0.001</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>Commission carte Shopify Payments</t>
         </is>
       </c>
-      <c r="B7" s="45" t="n">
+      <c r="B7" s="44" t="n">
         <v>0.015</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -4645,24 +4648,24 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="38" t="inlineStr">
         <is>
           <t>Frais fixe par transaction carte</t>
         </is>
       </c>
-      <c r="B8" s="46" t="n">
+      <c r="B8" s="45" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="38" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>LIVRAISON DES LOTS</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="39" t="inlineStr">
+      <c r="A11" s="38" t="inlineStr">
         <is>
           <t>Total des factures de livraison ADN</t>
         </is>
@@ -4677,7 +4680,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="39" t="inlineStr">
+      <c r="A12" s="38" t="inlineStr">
         <is>
           <t>Unités de vente reçues d'ADN</t>
         </is>
@@ -4692,7 +4695,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="39" t="inlineStr">
+      <c r="A13" s="38" t="inlineStr">
         <is>
           <t>Livraison par unité de vente</t>
         </is>
@@ -4708,19 +4711,19 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="38" t="inlineStr">
+      <c r="A15" s="37" t="inlineStr">
         <is>
           <t>IMPÔT SUR LE REVENU — MICRO-BIC</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="39" t="inlineStr">
+      <c r="A16" s="38" t="inlineStr">
         <is>
           <t>Abattement forfaitaire</t>
         </is>
       </c>
-      <c r="B16" s="45" t="n">
+      <c r="B16" s="44" t="n">
         <v>0.71</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -4730,12 +4733,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="39" t="inlineStr">
+      <c r="A17" s="38" t="inlineStr">
         <is>
           <t>Tranche marginale du foyer</t>
         </is>
       </c>
-      <c r="B17" s="45" t="n">
+      <c r="B17" s="44" t="n">
         <v>0.11</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -4745,46 +4748,46 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="38" t="inlineStr">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t>FRAIS DE VENTE</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="39" t="inlineStr">
+      <c r="A20" s="38" t="inlineStr">
         <is>
           <t>Emballage par colis</t>
         </is>
       </c>
-      <c r="B20" s="46" t="n">
+      <c r="B20" s="45" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="39" t="inlineStr">
+      <c r="A21" s="38" t="inlineStr">
         <is>
           <t>Nombre d'annonces prévues</t>
         </is>
       </c>
-      <c r="B21" s="47" t="n">
+      <c r="B21" s="46" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="38" t="inlineStr">
+      <c r="A23" s="37" t="inlineStr">
         <is>
           <t>PLANCHER DE NÉGOCIATION</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="39" t="inlineStr">
+      <c r="A24" s="38" t="inlineStr">
         <is>
           <t>Coefficient sur le seuil d'équilibre</t>
         </is>
       </c>
-      <c r="B24" s="48" t="n">
+      <c r="B24" s="47" t="n">
         <v>1.3</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -6382,67 +6385,67 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="35" t="n"/>
-      <c r="B39" s="35" t="n"/>
-      <c r="C39" s="35" t="n"/>
-      <c r="D39" s="35" t="n"/>
-      <c r="E39" s="35" t="n"/>
-      <c r="F39" s="33" t="inlineStr">
+      <c r="A39" s="34" t="n"/>
+      <c r="B39" s="34" t="n"/>
+      <c r="C39" s="34" t="n"/>
+      <c r="D39" s="34" t="n"/>
+      <c r="E39" s="34" t="n"/>
+      <c r="F39" s="32" t="inlineStr">
         <is>
           <t>TOTAL MARCHANDISE</t>
         </is>
       </c>
-      <c r="G39" s="34">
+      <c r="G39" s="33">
         <f>SUM(G5:G38)</f>
         <v/>
       </c>
-      <c r="H39" s="34">
+      <c r="H39" s="33">
         <f>SUM(H5:H38)</f>
         <v/>
       </c>
-      <c r="I39" s="34">
+      <c r="I39" s="33">
         <f>SUM(I5:I38)</f>
         <v/>
       </c>
-      <c r="J39" s="34">
+      <c r="J39" s="33">
         <f>SUM(J5:J38)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="38" t="inlineStr">
+      <c r="A41" s="37" t="inlineStr">
         <is>
           <t>FACTURES DE LIVRAISON</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="49" t="inlineStr">
+      <c r="A42" s="48" t="inlineStr">
         <is>
           <t>Facture</t>
         </is>
       </c>
-      <c r="B42" s="49" t="inlineStr">
+      <c r="B42" s="48" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C42" s="49" t="inlineStr">
+      <c r="C42" s="48" t="inlineStr">
         <is>
           <t>Maison</t>
         </is>
       </c>
-      <c r="D42" s="49" t="inlineStr">
+      <c r="D42" s="48" t="inlineStr">
         <is>
           <t>Commande</t>
         </is>
       </c>
-      <c r="E42" s="49" t="inlineStr">
+      <c r="E42" s="48" t="inlineStr">
         <is>
           <t>Désignation</t>
         </is>
       </c>
-      <c r="F42" s="49" t="inlineStr">
+      <c r="F42" s="48" t="inlineStr">
         <is>
           <t>Total TTC</t>
         </is>
@@ -6599,16 +6602,16 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="35" t="n"/>
-      <c r="B48" s="35" t="n"/>
-      <c r="C48" s="35" t="n"/>
-      <c r="D48" s="35" t="n"/>
-      <c r="E48" s="33" t="inlineStr">
+      <c r="A48" s="34" t="n"/>
+      <c r="B48" s="34" t="n"/>
+      <c r="C48" s="34" t="n"/>
+      <c r="D48" s="34" t="n"/>
+      <c r="E48" s="32" t="inlineStr">
         <is>
           <t>TOTAL LIVRAISON</t>
         </is>
       </c>
-      <c r="F48" s="34">
+      <c r="F48" s="33">
         <f>SUM(F43:F47)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
ventes: prix exacts, les huit ventes sont positives
Prix corriges : Balenciaga 135 EUR, Hoka 80, sac Karl Lagerfeld 70,
Nike Air Max 70, Lacoste 70, veste Armani Exchange 40. La Salomon a
100 EUR n'est pas encore encaissee, Vinted retenant le paiement jusqu'a
validation par l'acheteur.

593 EUR de ventes, 44,78 EUR de marge — toutes positives, contre quatre
en perte avec les prix approximatifs precedents.

Position de tresorerie ajoutee : 465 EUR encaisses, 386,75 EUR
reinvestis, 78,25 EUR en caisse dont 57,66 EUR d'URSSAF dus. Tresorerie
reellement libre : 20,59 EUR.

Nouveaux achats Interencheres de 386,75 EUR a integrer des reception de
la facture.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhpqQ2qsQi6zYv1VAx4s32
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-stock.xlsx
+++ b/exports/maison-nsaia-stock.xlsx
@@ -3042,13 +3042,13 @@
       </c>
       <c r="U29" s="14" t="inlineStr">
         <is>
-          <t>Vinted, acheteur en Italie</t>
+          <t>Vinted, Italie — non encaissé</t>
         </is>
       </c>
       <c r="V29" s="14" t="inlineStr"/>
       <c r="W29" s="14" t="inlineStr">
         <is>
-          <t>VENDUE</t>
+          <t>VENDUE, en attente</t>
         </is>
       </c>
       <c r="X29" s="14" t="inlineStr">
@@ -3061,301 +3061,313 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>EMPORIO ARMANI baskets P.36 — neuves</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>51.12</v>
-      </c>
-      <c r="C30" s="6">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>T-shirt BALENCIAGA T.2 — neuf</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
+        <v>113.4</v>
+      </c>
+      <c r="C30" s="16">
         <f>$B30+$Y30*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="17">
         <f>$C30/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E30" s="6">
+      <c r="E30" s="16">
         <f>CEILING($D30*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F30" s="8" t="n">
-        <v>69</v>
-      </c>
-      <c r="G30" s="8">
+      <c r="F30" s="18" t="n">
+        <v>135</v>
+      </c>
+      <c r="G30" s="18">
         <f>IF($F30="","",$F30-$C30-$M30-$N30)</f>
         <v/>
       </c>
-      <c r="H30" s="9">
+      <c r="H30" s="19">
         <f>IF($G30="","",$G30/$C30)</f>
         <v/>
       </c>
-      <c r="I30" s="10" t="n">
+      <c r="I30" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="J30" s="6">
+      <c r="J30" s="16">
         <f>$C30/$I30</f>
         <v/>
       </c>
-      <c r="K30" s="6">
+      <c r="K30" s="16">
         <f>IF($F30="","",$F30/$I30)</f>
         <v/>
       </c>
-      <c r="L30" s="6">
+      <c r="L30" s="16">
         <f>IF($G30="","",$G30/$I30)</f>
         <v/>
       </c>
-      <c r="M30" s="7">
+      <c r="M30" s="17">
         <f>IF($F30="","",$F30*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N30" s="6" t="n">
+      <c r="N30" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="O30" s="11" t="n">
+      <c r="O30" s="21" t="n">
+        <v>90</v>
+      </c>
+      <c r="P30" s="21" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="Q30" s="22" t="inlineStr">
+        <is>
+          <t>ADN Le Mans</t>
+        </is>
+      </c>
+      <c r="R30" s="22" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="S30" s="22" t="inlineStr">
+        <is>
+          <t>FB2026-44194</t>
+        </is>
+      </c>
+      <c r="T30" s="22" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="U30" s="14" t="inlineStr">
+        <is>
+          <t>vendu</t>
+        </is>
+      </c>
+      <c r="V30" s="14" t="inlineStr"/>
+      <c r="W30" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="X30" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="Y30" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Baskets NIKE Air Max Moto 2K P.44.5 — neuves</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="C31" s="16">
+        <f>$B31+$Y31*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D31" s="17">
+        <f>$C31/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
+        <v/>
+      </c>
+      <c r="E31" s="16">
+        <f>CEILING($D31*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F31" s="18" t="n">
+        <v>70</v>
+      </c>
+      <c r="G31" s="18">
+        <f>IF($F31="","",$F31-$C31-$M31-$N31)</f>
+        <v/>
+      </c>
+      <c r="H31" s="19">
+        <f>IF($G31="","",$G31/$C31)</f>
+        <v/>
+      </c>
+      <c r="I31" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" s="16">
+        <f>$C31/$I31</f>
+        <v/>
+      </c>
+      <c r="K31" s="16">
+        <f>IF($F31="","",$F31/$I31)</f>
+        <v/>
+      </c>
+      <c r="L31" s="16">
+        <f>IF($G31="","",$G31/$I31)</f>
+        <v/>
+      </c>
+      <c r="M31" s="17">
+        <f>IF($F31="","",$F31*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N31" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="P30" s="11" t="n">
+      <c r="P31" s="21" t="n">
         <v>10.4</v>
       </c>
-      <c r="Q30" s="12" t="inlineStr">
-        <is>
-          <t>ADN Lyon</t>
-        </is>
-      </c>
-      <c r="R30" s="12" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="S30" s="12" t="inlineStr">
-        <is>
-          <t>FB2026-6023</t>
-        </is>
-      </c>
-      <c r="T30" s="12" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="U30" s="4" t="inlineStr">
-        <is>
-          <t>Leboncoin</t>
-        </is>
-      </c>
-      <c r="V30" s="4" t="inlineStr"/>
-      <c r="W30" s="4" t="inlineStr">
-        <is>
-          <t>Liquider</t>
-        </is>
-      </c>
-      <c r="X30" s="4" t="inlineStr"/>
-      <c r="Y30" s="4" t="n">
+      <c r="Q31" s="22" t="inlineStr">
+        <is>
+          <t>ADN Le Mans</t>
+        </is>
+      </c>
+      <c r="R31" s="22" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="S31" s="22" t="inlineStr">
+        <is>
+          <t>FB2026-43716</t>
+        </is>
+      </c>
+      <c r="T31" s="22" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="U31" s="14" t="inlineStr">
+        <is>
+          <t>vendu</t>
+        </is>
+      </c>
+      <c r="V31" s="14" t="inlineStr"/>
+      <c r="W31" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="X31" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="Y31" s="14" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>NEW BALANCE sneakers P.38 — neuves</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="n">
-        <v>38.34</v>
-      </c>
-      <c r="C31" s="6">
-        <f>$B31+$Y31*Paramètres!$B$13</f>
-        <v/>
-      </c>
-      <c r="D31" s="7">
-        <f>$C31/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
-        <v/>
-      </c>
-      <c r="E31" s="6">
-        <f>CEILING($D31*Paramètres!$B$24,1)</f>
-        <v/>
-      </c>
-      <c r="F31" s="8" t="n">
-        <v>54</v>
-      </c>
-      <c r="G31" s="8">
-        <f>IF($F31="","",$F31-$C31-$M31-$N31)</f>
-        <v/>
-      </c>
-      <c r="H31" s="9">
-        <f>IF($G31="","",$G31/$C31)</f>
-        <v/>
-      </c>
-      <c r="I31" s="10" t="n">
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>Sac demi-lune nylon noir KARL LAGERFELD JEANS — neuf avec étiquette</t>
+        </is>
+      </c>
+      <c r="B32" s="15" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="C32" s="16">
+        <f>$B32+$Y32*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D32" s="17">
+        <f>$C32/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
+        <v/>
+      </c>
+      <c r="E32" s="16">
+        <f>CEILING($D32*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F32" s="18" t="n">
+        <v>70</v>
+      </c>
+      <c r="G32" s="18">
+        <f>IF($F32="","",$F32-$C32-$M32-$N32)</f>
+        <v/>
+      </c>
+      <c r="H32" s="19">
+        <f>IF($G32="","",$G32/$C32)</f>
+        <v/>
+      </c>
+      <c r="I32" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="J31" s="6">
-        <f>$C31/$I31</f>
-        <v/>
-      </c>
-      <c r="K31" s="6">
-        <f>IF($F31="","",$F31/$I31)</f>
-        <v/>
-      </c>
-      <c r="L31" s="6">
-        <f>IF($G31="","",$G31/$I31)</f>
-        <v/>
-      </c>
-      <c r="M31" s="7">
-        <f>IF($F31="","",$F31*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="N31" s="6" t="n">
+      <c r="J32" s="16">
+        <f>$C32/$I32</f>
+        <v/>
+      </c>
+      <c r="K32" s="16">
+        <f>IF($F32="","",$F32/$I32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="16">
+        <f>IF($G32="","",$G32/$I32)</f>
+        <v/>
+      </c>
+      <c r="M32" s="17">
+        <f>IF($F32="","",$F32*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N32" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="O31" s="11" t="n">
-        <v>30</v>
-      </c>
-      <c r="P31" s="11" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="Q31" s="12" t="inlineStr">
-        <is>
-          <t>ADN Lyon</t>
-        </is>
-      </c>
-      <c r="R31" s="12" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="S31" s="12" t="inlineStr">
-        <is>
-          <t>FB2026-6023</t>
-        </is>
-      </c>
-      <c r="T31" s="12" t="inlineStr">
-        <is>
-          <t>114</t>
-        </is>
-      </c>
-      <c r="U31" s="4" t="inlineStr">
-        <is>
-          <t>Leboncoin</t>
-        </is>
-      </c>
-      <c r="V31" s="4" t="inlineStr"/>
-      <c r="W31" s="4" t="inlineStr">
-        <is>
-          <t>Liquider</t>
-        </is>
-      </c>
-      <c r="X31" s="4" t="inlineStr"/>
-      <c r="Y31" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>NEW BALANCE baskets montantes P.44 — neuves</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="n">
-        <v>51.12</v>
-      </c>
-      <c r="C32" s="6">
-        <f>$B32+$Y32*Paramètres!$B$13</f>
-        <v/>
-      </c>
-      <c r="D32" s="7">
-        <f>$C32/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
-        <v/>
-      </c>
-      <c r="E32" s="6">
-        <f>CEILING($D32*Paramètres!$B$24,1)</f>
-        <v/>
-      </c>
-      <c r="F32" s="8" t="n">
-        <v>65</v>
-      </c>
-      <c r="G32" s="8">
-        <f>IF($F32="","",$F32-$C32-$M32-$N32)</f>
-        <v/>
-      </c>
-      <c r="H32" s="9">
-        <f>IF($G32="","",$G32/$C32)</f>
-        <v/>
-      </c>
-      <c r="I32" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J32" s="6">
-        <f>$C32/$I32</f>
-        <v/>
-      </c>
-      <c r="K32" s="6">
-        <f>IF($F32="","",$F32/$I32)</f>
-        <v/>
-      </c>
-      <c r="L32" s="6">
-        <f>IF($G32="","",$G32/$I32)</f>
-        <v/>
-      </c>
-      <c r="M32" s="7">
-        <f>IF($F32="","",$F32*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="N32" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O32" s="11" t="n">
+      <c r="O32" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="P32" s="11" t="n">
+      <c r="P32" s="21" t="n">
         <v>10.4</v>
       </c>
-      <c r="Q32" s="12" t="inlineStr">
-        <is>
-          <t>ADN Lyon</t>
-        </is>
-      </c>
-      <c r="R32" s="12" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="S32" s="12" t="inlineStr">
-        <is>
-          <t>FB2026-6023</t>
-        </is>
-      </c>
-      <c r="T32" s="12" t="inlineStr">
-        <is>
-          <t>156</t>
-        </is>
-      </c>
-      <c r="U32" s="4" t="inlineStr">
-        <is>
-          <t>Leboncoin</t>
-        </is>
-      </c>
-      <c r="V32" s="4" t="inlineStr"/>
-      <c r="W32" s="4" t="inlineStr">
-        <is>
-          <t>Liquider</t>
-        </is>
-      </c>
-      <c r="X32" s="4" t="inlineStr"/>
-      <c r="Y32" s="4" t="n">
+      <c r="Q32" s="22" t="inlineStr">
+        <is>
+          <t>ADN Le Mans</t>
+        </is>
+      </c>
+      <c r="R32" s="22" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="S32" s="22" t="inlineStr">
+        <is>
+          <t>FB2026-43716</t>
+        </is>
+      </c>
+      <c r="T32" s="22" t="inlineStr">
+        <is>
+          <t>431</t>
+        </is>
+      </c>
+      <c r="U32" s="14" t="inlineStr">
+        <is>
+          <t>vendu</t>
+        </is>
+      </c>
+      <c r="V32" s="14" t="inlineStr"/>
+      <c r="W32" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="X32" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="Y32" s="14" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>TOMMY JEANS baskets basses P.40 — neuves</t>
+          <t>EMPORIO ARMANI baskets P.36 — neuves</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>52.4</v>
+        <v>51.12</v>
       </c>
       <c r="C33" s="6">
         <f>$B33+$Y33*Paramètres!$B$13</f>
@@ -3370,7 +3382,7 @@
         <v/>
       </c>
       <c r="F33" s="8" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G33" s="8">
         <f>IF($F33="","",$F33-$C33-$M33-$N33)</f>
@@ -3403,10 +3415,10 @@
         <v>0</v>
       </c>
       <c r="O33" s="11" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P33" s="11" t="n">
-        <v>10.66</v>
+        <v>10.4</v>
       </c>
       <c r="Q33" s="12" t="inlineStr">
         <is>
@@ -3425,12 +3437,12 @@
       </c>
       <c r="T33" s="12" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>150</t>
         </is>
       </c>
       <c r="U33" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
+          <t>Leboncoin</t>
         </is>
       </c>
       <c r="V33" s="4" t="inlineStr"/>
@@ -3447,11 +3459,11 @@
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>LACOSTE sneakers P.42 — neuves</t>
+          <t>Baskets HOKA P.37 1/3 — neuves</t>
         </is>
       </c>
       <c r="B34" s="15" t="n">
-        <v>57.51</v>
+        <v>63</v>
       </c>
       <c r="C34" s="16">
         <f>$B34+$Y34*Paramètres!$B$13</f>
@@ -3466,7 +3478,7 @@
         <v/>
       </c>
       <c r="F34" s="18" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="G34" s="18">
         <f>IF($F34="","",$F34-$C34-$M34-$N34)</f>
@@ -3499,34 +3511,34 @@
         <v>0</v>
       </c>
       <c r="O34" s="21" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="P34" s="21" t="n">
-        <v>11.7</v>
+        <v>13</v>
       </c>
       <c r="Q34" s="22" t="inlineStr">
         <is>
-          <t>ADN Lyon</t>
+          <t>ADN Le Mans</t>
         </is>
       </c>
       <c r="R34" s="22" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>28/07/2026</t>
         </is>
       </c>
       <c r="S34" s="22" t="inlineStr">
         <is>
-          <t>FB2026-6023</t>
+          <t>FB2026-43716</t>
         </is>
       </c>
       <c r="T34" s="22" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>103</t>
         </is>
       </c>
       <c r="U34" s="14" t="inlineStr">
         <is>
-          <t>date à compléter</t>
+          <t>vendu</t>
         </is>
       </c>
       <c r="V34" s="14" t="inlineStr"/>
@@ -3545,409 +3557,401 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="14" t="inlineStr">
-        <is>
-          <t>T-shirt BALENCIAGA T.2 — neuf</t>
-        </is>
-      </c>
-      <c r="B35" s="15" t="n">
-        <v>113.4</v>
-      </c>
-      <c r="C35" s="16">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>NEW BALANCE sneakers P.38 — neuves</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>38.34</v>
+      </c>
+      <c r="C35" s="6">
         <f>$B35+$Y35*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D35" s="17">
+      <c r="D35" s="7">
         <f>$C35/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E35" s="16">
+      <c r="E35" s="6">
         <f>CEILING($D35*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F35" s="18" t="n">
-        <v>125</v>
-      </c>
-      <c r="G35" s="18">
+      <c r="F35" s="8" t="n">
+        <v>54</v>
+      </c>
+      <c r="G35" s="8">
         <f>IF($F35="","",$F35-$C35-$M35-$N35)</f>
         <v/>
       </c>
-      <c r="H35" s="19">
+      <c r="H35" s="9">
         <f>IF($G35="","",$G35/$C35)</f>
         <v/>
       </c>
-      <c r="I35" s="20" t="n">
+      <c r="I35" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J35" s="16">
+      <c r="J35" s="6">
         <f>$C35/$I35</f>
         <v/>
       </c>
-      <c r="K35" s="16">
+      <c r="K35" s="6">
         <f>IF($F35="","",$F35/$I35)</f>
         <v/>
       </c>
-      <c r="L35" s="16">
+      <c r="L35" s="6">
         <f>IF($G35="","",$G35/$I35)</f>
         <v/>
       </c>
-      <c r="M35" s="17">
+      <c r="M35" s="7">
         <f>IF($F35="","",$F35*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N35" s="16" t="n">
+      <c r="N35" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O35" s="21" t="n">
-        <v>90</v>
-      </c>
-      <c r="P35" s="21" t="n">
-        <v>23.4</v>
-      </c>
-      <c r="Q35" s="22" t="inlineStr">
+      <c r="O35" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="P35" s="11" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Q35" s="12" t="inlineStr">
+        <is>
+          <t>ADN Lyon</t>
+        </is>
+      </c>
+      <c r="R35" s="12" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="S35" s="12" t="inlineStr">
+        <is>
+          <t>FB2026-6023</t>
+        </is>
+      </c>
+      <c r="T35" s="12" t="inlineStr">
+        <is>
+          <t>114</t>
+        </is>
+      </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>Leboncoin</t>
+        </is>
+      </c>
+      <c r="V35" s="4" t="inlineStr"/>
+      <c r="W35" s="4" t="inlineStr">
+        <is>
+          <t>Liquider</t>
+        </is>
+      </c>
+      <c r="X35" s="4" t="inlineStr"/>
+      <c r="Y35" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Veste en jean ARMANI EXCHANGE T.S — neuve</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="C36" s="16">
+        <f>$B36+$Y36*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D36" s="17">
+        <f>$C36/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
+        <v/>
+      </c>
+      <c r="E36" s="16">
+        <f>CEILING($D36*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F36" s="18" t="n">
+        <v>40</v>
+      </c>
+      <c r="G36" s="18">
+        <f>IF($F36="","",$F36-$C36-$M36-$N36)</f>
+        <v/>
+      </c>
+      <c r="H36" s="19">
+        <f>IF($G36="","",$G36/$C36)</f>
+        <v/>
+      </c>
+      <c r="I36" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" s="16">
+        <f>$C36/$I36</f>
+        <v/>
+      </c>
+      <c r="K36" s="16">
+        <f>IF($F36="","",$F36/$I36)</f>
+        <v/>
+      </c>
+      <c r="L36" s="16">
+        <f>IF($G36="","",$G36/$I36)</f>
+        <v/>
+      </c>
+      <c r="M36" s="17">
+        <f>IF($F36="","",$F36*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N36" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="P36" s="21" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="Q36" s="22" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="R35" s="22" t="inlineStr">
+      <c r="R36" s="22" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="S36" s="22" t="inlineStr">
+        <is>
+          <t>FB2026-43717</t>
+        </is>
+      </c>
+      <c r="T36" s="22" t="inlineStr">
+        <is>
+          <t>168</t>
+        </is>
+      </c>
+      <c r="U36" s="14" t="inlineStr">
+        <is>
+          <t>vendu</t>
+        </is>
+      </c>
+      <c r="V36" s="14" t="inlineStr"/>
+      <c r="W36" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="X36" s="14" t="inlineStr">
+        <is>
+          <t>VENDU</t>
+        </is>
+      </c>
+      <c r="Y36" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>NEW BALANCE baskets montantes P.44 — neuves</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="C37" s="6">
+        <f>$B37+$Y37*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D37" s="7">
+        <f>$C37/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
+        <v/>
+      </c>
+      <c r="E37" s="6">
+        <f>CEILING($D37*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="G37" s="8">
+        <f>IF($F37="","",$F37-$C37-$M37-$N37)</f>
+        <v/>
+      </c>
+      <c r="H37" s="9">
+        <f>IF($G37="","",$G37/$C37)</f>
+        <v/>
+      </c>
+      <c r="I37" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="6">
+        <f>$C37/$I37</f>
+        <v/>
+      </c>
+      <c r="K37" s="6">
+        <f>IF($F37="","",$F37/$I37)</f>
+        <v/>
+      </c>
+      <c r="L37" s="6">
+        <f>IF($G37="","",$G37/$I37)</f>
+        <v/>
+      </c>
+      <c r="M37" s="7">
+        <f>IF($F37="","",$F37*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="11" t="n">
+        <v>40</v>
+      </c>
+      <c r="P37" s="11" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="Q37" s="12" t="inlineStr">
+        <is>
+          <t>ADN Lyon</t>
+        </is>
+      </c>
+      <c r="R37" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="S35" s="22" t="inlineStr">
-        <is>
-          <t>FB2026-44194</t>
-        </is>
-      </c>
-      <c r="T35" s="22" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="U35" s="14" t="inlineStr">
-        <is>
-          <t>date à compléter</t>
-        </is>
-      </c>
-      <c r="V35" s="14" t="inlineStr"/>
-      <c r="W35" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="X35" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="Y35" s="14" t="n">
+      <c r="S37" s="12" t="inlineStr">
+        <is>
+          <t>FB2026-6023</t>
+        </is>
+      </c>
+      <c r="T37" s="12" t="inlineStr">
+        <is>
+          <t>156</t>
+        </is>
+      </c>
+      <c r="U37" s="4" t="inlineStr">
+        <is>
+          <t>Leboncoin</t>
+        </is>
+      </c>
+      <c r="V37" s="4" t="inlineStr"/>
+      <c r="W37" s="4" t="inlineStr">
+        <is>
+          <t>Liquider</t>
+        </is>
+      </c>
+      <c r="X37" s="4" t="inlineStr"/>
+      <c r="Y37" s="4" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="23" t="inlineStr">
-        <is>
-          <t>Lot de 4 toupies BEYBLADE HASBRO</t>
-        </is>
-      </c>
-      <c r="B36" s="24" t="n">
-        <v>38.34</v>
-      </c>
-      <c r="C36" s="25">
-        <f>$B36+$Y36*Paramètres!$B$13</f>
-        <v/>
-      </c>
-      <c r="D36" s="26">
-        <f>$C36/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
-        <v/>
-      </c>
-      <c r="E36" s="25">
-        <f>CEILING($D36*Paramètres!$B$24,1)</f>
-        <v/>
-      </c>
-      <c r="F36" s="27" t="n">
-        <v>49</v>
-      </c>
-      <c r="G36" s="27">
-        <f>IF($F36="","",$F36-$C36-$M36-$N36)</f>
-        <v/>
-      </c>
-      <c r="H36" s="28">
-        <f>IF($G36="","",$G36/$C36)</f>
-        <v/>
-      </c>
-      <c r="I36" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="J36" s="25">
-        <f>$C36/$I36</f>
-        <v/>
-      </c>
-      <c r="K36" s="25">
-        <f>IF($F36="","",$F36/$I36)</f>
-        <v/>
-      </c>
-      <c r="L36" s="25">
-        <f>IF($G36="","",$G36/$I36)</f>
-        <v/>
-      </c>
-      <c r="M36" s="26">
-        <f>IF($F36="","",$F36*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="N36" s="25" t="n">
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>TOMMY JEANS baskets basses P.40 — neuves</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="C38" s="6">
+        <f>$B38+$Y38*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D38" s="7">
+        <f>$C38/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
+        <v/>
+      </c>
+      <c r="E38" s="6">
+        <f>CEILING($D38*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F38" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="G38" s="8">
+        <f>IF($F38="","",$F38-$C38-$M38-$N38)</f>
+        <v/>
+      </c>
+      <c r="H38" s="9">
+        <f>IF($G38="","",$G38/$C38)</f>
+        <v/>
+      </c>
+      <c r="I38" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" s="6">
+        <f>$C38/$I38</f>
+        <v/>
+      </c>
+      <c r="K38" s="6">
+        <f>IF($F38="","",$F38/$I38)</f>
+        <v/>
+      </c>
+      <c r="L38" s="6">
+        <f>IF($G38="","",$G38/$I38)</f>
+        <v/>
+      </c>
+      <c r="M38" s="7">
+        <f>IF($F38="","",$F38*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N38" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O36" s="30" t="n">
-        <v>30</v>
-      </c>
-      <c r="P36" s="30" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="Q36" s="31" t="inlineStr">
-        <is>
-          <t>ADN Le Mans</t>
-        </is>
-      </c>
-      <c r="R36" s="31" t="inlineStr">
+      <c r="O38" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="P38" s="11" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="Q38" s="12" t="inlineStr">
+        <is>
+          <t>ADN Lyon</t>
+        </is>
+      </c>
+      <c r="R38" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="S36" s="31" t="inlineStr">
-        <is>
-          <t>FB2026-44192</t>
-        </is>
-      </c>
-      <c r="T36" s="31" t="inlineStr">
-        <is>
-          <t>299</t>
-        </is>
-      </c>
-      <c r="U36" s="23" t="inlineStr">
-        <is>
-          <t>Leboncoin + eBay, en lot</t>
-        </is>
-      </c>
-      <c r="V36" s="23" t="inlineStr"/>
-      <c r="W36" s="23" t="inlineStr">
-        <is>
-          <t>Marge faible</t>
-        </is>
-      </c>
-      <c r="X36" s="23" t="inlineStr"/>
-      <c r="Y36" s="23" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="14" t="inlineStr">
-        <is>
-          <t>Veste en jean ARMANI EXCHANGE T.S — neuve</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="C37" s="16">
-        <f>$B37+$Y37*Paramètres!$B$13</f>
-        <v/>
-      </c>
-      <c r="D37" s="17">
-        <f>$C37/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
-        <v/>
-      </c>
-      <c r="E37" s="16">
-        <f>CEILING($D37*Paramètres!$B$24,1)</f>
-        <v/>
-      </c>
-      <c r="F37" s="18" t="n">
-        <v>35</v>
-      </c>
-      <c r="G37" s="18">
-        <f>IF($F37="","",$F37-$C37-$M37-$N37)</f>
-        <v/>
-      </c>
-      <c r="H37" s="19">
-        <f>IF($G37="","",$G37/$C37)</f>
-        <v/>
-      </c>
-      <c r="I37" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J37" s="16">
-        <f>$C37/$I37</f>
-        <v/>
-      </c>
-      <c r="K37" s="16">
-        <f>IF($F37="","",$F37/$I37)</f>
-        <v/>
-      </c>
-      <c r="L37" s="16">
-        <f>IF($G37="","",$G37/$I37)</f>
-        <v/>
-      </c>
-      <c r="M37" s="17">
-        <f>IF($F37="","",$F37*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="N37" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" s="21" t="n">
-        <v>20</v>
-      </c>
-      <c r="P37" s="21" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="Q37" s="22" t="inlineStr">
-        <is>
-          <t>ADN Le Mans</t>
-        </is>
-      </c>
-      <c r="R37" s="22" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="S37" s="22" t="inlineStr">
-        <is>
-          <t>FB2026-43717</t>
-        </is>
-      </c>
-      <c r="T37" s="22" t="inlineStr">
-        <is>
-          <t>168</t>
-        </is>
-      </c>
-      <c r="U37" s="14" t="inlineStr">
-        <is>
-          <t>date à compléter</t>
-        </is>
-      </c>
-      <c r="V37" s="14" t="inlineStr"/>
-      <c r="W37" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="X37" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="Y37" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="14" t="inlineStr">
-        <is>
-          <t>Baskets NIKE Air Max Moto 2K P.44.5 — neuves</t>
-        </is>
-      </c>
-      <c r="B38" s="15" t="n">
-        <v>50.4</v>
-      </c>
-      <c r="C38" s="16">
-        <f>$B38+$Y38*Paramètres!$B$13</f>
-        <v/>
-      </c>
-      <c r="D38" s="17">
-        <f>$C38/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
-        <v/>
-      </c>
-      <c r="E38" s="16">
-        <f>CEILING($D38*Paramètres!$B$24,1)</f>
-        <v/>
-      </c>
-      <c r="F38" s="18" t="n">
-        <v>60</v>
-      </c>
-      <c r="G38" s="18">
-        <f>IF($F38="","",$F38-$C38-$M38-$N38)</f>
-        <v/>
-      </c>
-      <c r="H38" s="19">
-        <f>IF($G38="","",$G38/$C38)</f>
-        <v/>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J38" s="16">
-        <f>$C38/$I38</f>
-        <v/>
-      </c>
-      <c r="K38" s="16">
-        <f>IF($F38="","",$F38/$I38)</f>
-        <v/>
-      </c>
-      <c r="L38" s="16">
-        <f>IF($G38="","",$G38/$I38)</f>
-        <v/>
-      </c>
-      <c r="M38" s="17">
-        <f>IF($F38="","",$F38*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="N38" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" s="21" t="n">
-        <v>40</v>
-      </c>
-      <c r="P38" s="21" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="Q38" s="22" t="inlineStr">
-        <is>
-          <t>ADN Le Mans</t>
-        </is>
-      </c>
-      <c r="R38" s="22" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="S38" s="22" t="inlineStr">
-        <is>
-          <t>FB2026-43716</t>
-        </is>
-      </c>
-      <c r="T38" s="22" t="inlineStr">
-        <is>
-          <t>170</t>
-        </is>
-      </c>
-      <c r="U38" s="14" t="inlineStr">
-        <is>
-          <t>date à compléter</t>
-        </is>
-      </c>
-      <c r="V38" s="14" t="inlineStr"/>
-      <c r="W38" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="X38" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="Y38" s="14" t="n">
+      <c r="S38" s="12" t="inlineStr">
+        <is>
+          <t>FB2026-6023</t>
+        </is>
+      </c>
+      <c r="T38" s="12" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="U38" s="4" t="inlineStr">
+        <is>
+          <t>Leboncoin + eBay</t>
+        </is>
+      </c>
+      <c r="V38" s="4" t="inlineStr"/>
+      <c r="W38" s="4" t="inlineStr">
+        <is>
+          <t>Liquider</t>
+        </is>
+      </c>
+      <c r="X38" s="4" t="inlineStr"/>
+      <c r="Y38" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>Sac demi-lune nylon noir KARL LAGERFELD JEANS — neuf avec étiquette</t>
+          <t>LACOSTE sneakers P.42 — neuves</t>
         </is>
       </c>
       <c r="B39" s="15" t="n">
-        <v>50.4</v>
+        <v>57.51</v>
       </c>
       <c r="C39" s="16">
         <f>$B39+$Y39*Paramètres!$B$13</f>
@@ -3962,7 +3966,7 @@
         <v/>
       </c>
       <c r="F39" s="18" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="G39" s="18">
         <f>IF($F39="","",$F39-$C39-$M39-$N39)</f>
@@ -3995,34 +3999,34 @@
         <v>0</v>
       </c>
       <c r="O39" s="21" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="P39" s="21" t="n">
-        <v>10.4</v>
+        <v>11.7</v>
       </c>
       <c r="Q39" s="22" t="inlineStr">
         <is>
-          <t>ADN Le Mans</t>
+          <t>ADN Lyon</t>
         </is>
       </c>
       <c r="R39" s="22" t="inlineStr">
         <is>
-          <t>28/07/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="S39" s="22" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>FB2026-6023</t>
         </is>
       </c>
       <c r="T39" s="22" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>141</t>
         </is>
       </c>
       <c r="U39" s="14" t="inlineStr">
         <is>
-          <t>date à compléter</t>
+          <t>vendu</t>
         </is>
       </c>
       <c r="V39" s="14" t="inlineStr"/>
@@ -4041,102 +4045,98 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="inlineStr">
-        <is>
-          <t>Baskets HOKA P.37 1/3 — neuves</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="n">
-        <v>63</v>
-      </c>
-      <c r="C40" s="16">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>Lot de 4 toupies BEYBLADE HASBRO</t>
+        </is>
+      </c>
+      <c r="B40" s="24" t="n">
+        <v>38.34</v>
+      </c>
+      <c r="C40" s="25">
         <f>$B40+$Y40*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D40" s="17">
+      <c r="D40" s="26">
         <f>$C40/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E40" s="16">
+      <c r="E40" s="25">
         <f>CEILING($D40*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F40" s="18" t="n">
-        <v>70</v>
-      </c>
-      <c r="G40" s="18">
+      <c r="F40" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="G40" s="27">
         <f>IF($F40="","",$F40-$C40-$M40-$N40)</f>
         <v/>
       </c>
-      <c r="H40" s="19">
+      <c r="H40" s="28">
         <f>IF($G40="","",$G40/$C40)</f>
         <v/>
       </c>
-      <c r="I40" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J40" s="16">
+      <c r="I40" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="J40" s="25">
         <f>$C40/$I40</f>
         <v/>
       </c>
-      <c r="K40" s="16">
+      <c r="K40" s="25">
         <f>IF($F40="","",$F40/$I40)</f>
         <v/>
       </c>
-      <c r="L40" s="16">
+      <c r="L40" s="25">
         <f>IF($G40="","",$G40/$I40)</f>
         <v/>
       </c>
-      <c r="M40" s="17">
+      <c r="M40" s="26">
         <f>IF($F40="","",$F40*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N40" s="16" t="n">
+      <c r="N40" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="O40" s="21" t="n">
-        <v>50</v>
-      </c>
-      <c r="P40" s="21" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q40" s="22" t="inlineStr">
+      <c r="O40" s="30" t="n">
+        <v>30</v>
+      </c>
+      <c r="P40" s="30" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Q40" s="31" t="inlineStr">
         <is>
           <t>ADN Le Mans</t>
         </is>
       </c>
-      <c r="R40" s="22" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="S40" s="22" t="inlineStr">
-        <is>
-          <t>FB2026-43716</t>
-        </is>
-      </c>
-      <c r="T40" s="22" t="inlineStr">
-        <is>
-          <t>103</t>
-        </is>
-      </c>
-      <c r="U40" s="14" t="inlineStr">
-        <is>
-          <t>date à compléter</t>
-        </is>
-      </c>
-      <c r="V40" s="14" t="inlineStr"/>
-      <c r="W40" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="X40" s="14" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="Y40" s="14" t="n">
+      <c r="R40" s="31" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="S40" s="31" t="inlineStr">
+        <is>
+          <t>FB2026-44192</t>
+        </is>
+      </c>
+      <c r="T40" s="31" t="inlineStr">
+        <is>
+          <t>299</t>
+        </is>
+      </c>
+      <c r="U40" s="23" t="inlineStr">
+        <is>
+          <t>Leboncoin + eBay, en lot</t>
+        </is>
+      </c>
+      <c r="V40" s="23" t="inlineStr"/>
+      <c r="W40" s="23" t="inlineStr">
+        <is>
+          <t>Marge faible</t>
+        </is>
+      </c>
+      <c r="X40" s="23" t="inlineStr"/>
+      <c r="Y40" s="23" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Hoka et Nike reclassees en prelevements: le CA passe de 493 a 343 EUR
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-stock.xlsx
+++ b/exports/maison-nsaia-stock.xlsx
@@ -140,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -175,6 +175,7 @@
     <xf numFmtId="3" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3071,7 +3072,7 @@
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
-          <t>Baskets NIKE Air Max Moto 2K P.44.5 — neuves</t>
+          <t>Sac demi-lune nylon noir KARL LAGERFELD JEANS — neuf avec étiquette</t>
         </is>
       </c>
       <c r="B30" s="14" t="n">
@@ -3145,7 +3146,7 @@
       </c>
       <c r="T30" s="21" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>431</t>
         </is>
       </c>
       <c r="U30" s="13" t="inlineStr">
@@ -3169,113 +3170,109 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>Sac demi-lune nylon noir KARL LAGERFELD JEANS — neuf avec étiquette</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="n">
-        <v>50.4</v>
-      </c>
-      <c r="C31" s="15">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>EMPORIO ARMANI baskets P.36 — neuves</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="C31" s="6">
         <f>$B31+$Y31*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D31" s="16">
+      <c r="D31" s="7">
         <f>$C31/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E31" s="15">
+      <c r="E31" s="6">
         <f>CEILING($D31*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F31" s="17" t="n">
-        <v>70</v>
-      </c>
-      <c r="G31" s="17">
+      <c r="F31" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="G31" s="8">
         <f>IF($F31="","",$F31-$C31-$M31-$N31)</f>
         <v/>
       </c>
-      <c r="H31" s="18">
+      <c r="H31" s="9">
         <f>IF($G31="","",$G31/$C31)</f>
         <v/>
       </c>
-      <c r="I31" s="19" t="n">
+      <c r="I31" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J31" s="15">
+      <c r="J31" s="6">
         <f>$C31/$I31</f>
         <v/>
       </c>
-      <c r="K31" s="15">
+      <c r="K31" s="6">
         <f>IF($F31="","",$F31/$I31)</f>
         <v/>
       </c>
-      <c r="L31" s="15">
+      <c r="L31" s="6">
         <f>IF($G31="","",$G31/$I31)</f>
         <v/>
       </c>
-      <c r="M31" s="16">
+      <c r="M31" s="7">
         <f>IF($F31="","",$F31*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N31" s="15" t="n">
+      <c r="N31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O31" s="20" t="n">
+      <c r="O31" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="P31" s="20" t="n">
+      <c r="P31" s="11" t="n">
         <v>10.4</v>
       </c>
-      <c r="Q31" s="21" t="inlineStr">
-        <is>
-          <t>ADN Le Mans</t>
-        </is>
-      </c>
-      <c r="R31" s="21" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="S31" s="21" t="inlineStr">
-        <is>
-          <t>FB2026-43716</t>
-        </is>
-      </c>
-      <c r="T31" s="21" t="inlineStr">
-        <is>
-          <t>431</t>
-        </is>
-      </c>
-      <c r="U31" s="13" t="inlineStr">
-        <is>
-          <t>vendu</t>
-        </is>
-      </c>
-      <c r="V31" s="13" t="inlineStr"/>
-      <c r="W31" s="13" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="X31" s="13" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="Y31" s="13" t="n">
+      <c r="Q31" s="12" t="inlineStr">
+        <is>
+          <t>ADN Lyon</t>
+        </is>
+      </c>
+      <c r="R31" s="12" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="S31" s="12" t="inlineStr">
+        <is>
+          <t>FB2026-6023</t>
+        </is>
+      </c>
+      <c r="T31" s="12" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="U31" s="4" t="inlineStr">
+        <is>
+          <t>Leboncoin</t>
+        </is>
+      </c>
+      <c r="V31" s="4" t="inlineStr"/>
+      <c r="W31" s="4" t="inlineStr">
+        <is>
+          <t>Liquider</t>
+        </is>
+      </c>
+      <c r="X31" s="4" t="inlineStr"/>
+      <c r="Y31" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>EMPORIO ARMANI baskets P.36 — neuves</t>
+          <t>NEW BALANCE sneakers P.38 — neuves</t>
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>51.12</v>
+        <v>38.34</v>
       </c>
       <c r="C32" s="6">
         <f>$B32+$Y32*Paramètres!$B$13</f>
@@ -3290,7 +3287,7 @@
         <v/>
       </c>
       <c r="F32" s="8" t="n">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="G32" s="8">
         <f>IF($F32="","",$F32-$C32-$M32-$N32)</f>
@@ -3323,10 +3320,10 @@
         <v>0</v>
       </c>
       <c r="O32" s="11" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="P32" s="11" t="n">
-        <v>10.4</v>
+        <v>7.8</v>
       </c>
       <c r="Q32" s="12" t="inlineStr">
         <is>
@@ -3345,7 +3342,7 @@
       </c>
       <c r="T32" s="12" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>114</t>
         </is>
       </c>
       <c r="U32" s="4" t="inlineStr">
@@ -3367,11 +3364,11 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Baskets HOKA P.37 1/3 — neuves</t>
+          <t>Veste en jean ARMANI EXCHANGE T.S — neuve</t>
         </is>
       </c>
       <c r="B33" s="14" t="n">
-        <v>63</v>
+        <v>25.2</v>
       </c>
       <c r="C33" s="15">
         <f>$B33+$Y33*Paramètres!$B$13</f>
@@ -3386,7 +3383,7 @@
         <v/>
       </c>
       <c r="F33" s="17" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="G33" s="17">
         <f>IF($F33="","",$F33-$C33-$M33-$N33)</f>
@@ -3419,10 +3416,10 @@
         <v>0</v>
       </c>
       <c r="O33" s="20" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="P33" s="20" t="n">
-        <v>13</v>
+        <v>5.2</v>
       </c>
       <c r="Q33" s="21" t="inlineStr">
         <is>
@@ -3436,12 +3433,12 @@
       </c>
       <c r="S33" s="21" t="inlineStr">
         <is>
-          <t>FB2026-43716</t>
+          <t>FB2026-43717</t>
         </is>
       </c>
       <c r="T33" s="21" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>168</t>
         </is>
       </c>
       <c r="U33" s="13" t="inlineStr">
@@ -3467,11 +3464,11 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>NEW BALANCE sneakers P.38 — neuves</t>
+          <t>NEW BALANCE baskets montantes P.44 — neuves</t>
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>38.34</v>
+        <v>51.12</v>
       </c>
       <c r="C34" s="6">
         <f>$B34+$Y34*Paramètres!$B$13</f>
@@ -3486,7 +3483,7 @@
         <v/>
       </c>
       <c r="F34" s="8" t="n">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="G34" s="8">
         <f>IF($F34="","",$F34-$C34-$M34-$N34)</f>
@@ -3519,10 +3516,10 @@
         <v>0</v>
       </c>
       <c r="O34" s="11" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="P34" s="11" t="n">
-        <v>7.8</v>
+        <v>10.4</v>
       </c>
       <c r="Q34" s="12" t="inlineStr">
         <is>
@@ -3541,7 +3538,7 @@
       </c>
       <c r="T34" s="12" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>156</t>
         </is>
       </c>
       <c r="U34" s="4" t="inlineStr">
@@ -3561,212 +3558,212 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
-        <is>
-          <t>Veste en jean ARMANI EXCHANGE T.S — neuve</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="C35" s="15">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>TOMMY JEANS baskets basses P.40 — neuves</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="C35" s="6">
         <f>$B35+$Y35*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D35" s="16">
+      <c r="D35" s="7">
         <f>$C35/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E35" s="15">
+      <c r="E35" s="6">
         <f>CEILING($D35*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F35" s="17" t="n">
-        <v>40</v>
-      </c>
-      <c r="G35" s="17">
+      <c r="F35" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="G35" s="8">
         <f>IF($F35="","",$F35-$C35-$M35-$N35)</f>
         <v/>
       </c>
-      <c r="H35" s="18">
+      <c r="H35" s="9">
         <f>IF($G35="","",$G35/$C35)</f>
         <v/>
       </c>
-      <c r="I35" s="19" t="n">
+      <c r="I35" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="J35" s="15">
+      <c r="J35" s="6">
         <f>$C35/$I35</f>
         <v/>
       </c>
-      <c r="K35" s="15">
+      <c r="K35" s="6">
         <f>IF($F35="","",$F35/$I35)</f>
         <v/>
       </c>
-      <c r="L35" s="15">
+      <c r="L35" s="6">
         <f>IF($G35="","",$G35/$I35)</f>
         <v/>
       </c>
-      <c r="M35" s="16">
+      <c r="M35" s="7">
         <f>IF($F35="","",$F35*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N35" s="15" t="n">
+      <c r="N35" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O35" s="20" t="n">
-        <v>20</v>
-      </c>
-      <c r="P35" s="20" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="Q35" s="21" t="inlineStr">
-        <is>
-          <t>ADN Le Mans</t>
-        </is>
-      </c>
-      <c r="R35" s="21" t="inlineStr">
-        <is>
-          <t>28/07/2026</t>
-        </is>
-      </c>
-      <c r="S35" s="21" t="inlineStr">
-        <is>
-          <t>FB2026-43717</t>
-        </is>
-      </c>
-      <c r="T35" s="21" t="inlineStr">
-        <is>
-          <t>168</t>
-        </is>
-      </c>
-      <c r="U35" s="13" t="inlineStr">
+      <c r="O35" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="P35" s="11" t="n">
+        <v>10.66</v>
+      </c>
+      <c r="Q35" s="12" t="inlineStr">
+        <is>
+          <t>ADN Lyon</t>
+        </is>
+      </c>
+      <c r="R35" s="12" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="S35" s="12" t="inlineStr">
+        <is>
+          <t>FB2026-6023</t>
+        </is>
+      </c>
+      <c r="T35" s="12" t="inlineStr">
+        <is>
+          <t>158</t>
+        </is>
+      </c>
+      <c r="U35" s="4" t="inlineStr">
+        <is>
+          <t>Leboncoin + eBay</t>
+        </is>
+      </c>
+      <c r="V35" s="4" t="inlineStr"/>
+      <c r="W35" s="4" t="inlineStr">
+        <is>
+          <t>Liquider</t>
+        </is>
+      </c>
+      <c r="X35" s="4" t="inlineStr"/>
+      <c r="Y35" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>LACOSTE sneakers P.42 — neuves</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="n">
+        <v>57.51</v>
+      </c>
+      <c r="C36" s="15">
+        <f>$B36+$Y36*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D36" s="16">
+        <f>$C36/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
+        <v/>
+      </c>
+      <c r="E36" s="15">
+        <f>CEILING($D36*Paramètres!$B$24,1)</f>
+        <v/>
+      </c>
+      <c r="F36" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="G36" s="17">
+        <f>IF($F36="","",$F36-$C36-$M36-$N36)</f>
+        <v/>
+      </c>
+      <c r="H36" s="18">
+        <f>IF($G36="","",$G36/$C36)</f>
+        <v/>
+      </c>
+      <c r="I36" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J36" s="15">
+        <f>$C36/$I36</f>
+        <v/>
+      </c>
+      <c r="K36" s="15">
+        <f>IF($F36="","",$F36/$I36)</f>
+        <v/>
+      </c>
+      <c r="L36" s="15">
+        <f>IF($G36="","",$G36/$I36)</f>
+        <v/>
+      </c>
+      <c r="M36" s="16">
+        <f>IF($F36="","",$F36*(Paramètres!$B$5+Paramètres!$B$6))</f>
+        <v/>
+      </c>
+      <c r="N36" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="P36" s="20" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="Q36" s="21" t="inlineStr">
+        <is>
+          <t>ADN Lyon</t>
+        </is>
+      </c>
+      <c r="R36" s="21" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
+      <c r="S36" s="21" t="inlineStr">
+        <is>
+          <t>FB2026-6023</t>
+        </is>
+      </c>
+      <c r="T36" s="21" t="inlineStr">
+        <is>
+          <t>141</t>
+        </is>
+      </c>
+      <c r="U36" s="13" t="inlineStr">
         <is>
           <t>vendu</t>
         </is>
       </c>
-      <c r="V35" s="13" t="inlineStr"/>
-      <c r="W35" s="13" t="inlineStr">
+      <c r="V36" s="13" t="inlineStr"/>
+      <c r="W36" s="13" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="X35" s="13" t="inlineStr">
+      <c r="X36" s="13" t="inlineStr">
         <is>
           <t>VENDU</t>
         </is>
       </c>
-      <c r="Y35" s="13" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>NEW BALANCE baskets montantes P.44 — neuves</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="n">
-        <v>51.12</v>
-      </c>
-      <c r="C36" s="6">
-        <f>$B36+$Y36*Paramètres!$B$13</f>
-        <v/>
-      </c>
-      <c r="D36" s="7">
-        <f>$C36/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
-        <v/>
-      </c>
-      <c r="E36" s="6">
-        <f>CEILING($D36*Paramètres!$B$24,1)</f>
-        <v/>
-      </c>
-      <c r="F36" s="8" t="n">
-        <v>65</v>
-      </c>
-      <c r="G36" s="8">
-        <f>IF($F36="","",$F36-$C36-$M36-$N36)</f>
-        <v/>
-      </c>
-      <c r="H36" s="9">
-        <f>IF($G36="","",$G36/$C36)</f>
-        <v/>
-      </c>
-      <c r="I36" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J36" s="6">
-        <f>$C36/$I36</f>
-        <v/>
-      </c>
-      <c r="K36" s="6">
-        <f>IF($F36="","",$F36/$I36)</f>
-        <v/>
-      </c>
-      <c r="L36" s="6">
-        <f>IF($G36="","",$G36/$I36)</f>
-        <v/>
-      </c>
-      <c r="M36" s="7">
-        <f>IF($F36="","",$F36*(Paramètres!$B$5+Paramètres!$B$6))</f>
-        <v/>
-      </c>
-      <c r="N36" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="P36" s="11" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="Q36" s="12" t="inlineStr">
-        <is>
-          <t>ADN Lyon</t>
-        </is>
-      </c>
-      <c r="R36" s="12" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="S36" s="12" t="inlineStr">
-        <is>
-          <t>FB2026-6023</t>
-        </is>
-      </c>
-      <c r="T36" s="12" t="inlineStr">
-        <is>
-          <t>156</t>
-        </is>
-      </c>
-      <c r="U36" s="4" t="inlineStr">
-        <is>
-          <t>Leboncoin</t>
-        </is>
-      </c>
-      <c r="V36" s="4" t="inlineStr"/>
-      <c r="W36" s="4" t="inlineStr">
-        <is>
-          <t>Liquider</t>
-        </is>
-      </c>
-      <c r="X36" s="4" t="inlineStr"/>
-      <c r="Y36" s="4" t="n">
+      <c r="Y36" s="13" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>TOMMY JEANS baskets basses P.40 — neuves</t>
+          <t>Pompe immergée ROBBY VP550W noir et bleu — produit d'occasion</t>
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>52.4</v>
+        <v>35.9</v>
       </c>
       <c r="C37" s="6">
-        <f>$B37+$Y37*Paramètres!$B$13</f>
+        <f>$B37</f>
         <v/>
       </c>
       <c r="D37" s="7">
@@ -3778,7 +3775,7 @@
         <v/>
       </c>
       <c r="F37" s="8" t="n">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="G37" s="8">
         <f>IF($F37="","",$F37-$C37-$M37-$N37)</f>
@@ -3810,41 +3807,37 @@
       <c r="N37" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O37" s="11" t="n">
-        <v>41</v>
-      </c>
-      <c r="P37" s="11" t="n">
-        <v>10.66</v>
-      </c>
+      <c r="O37" s="22" t="n"/>
+      <c r="P37" s="22" t="n"/>
       <c r="Q37" s="12" t="inlineStr">
         <is>
-          <t>ADN Lyon</t>
+          <t>ERA Enchères Rhône-Alpes</t>
         </is>
       </c>
       <c r="R37" s="12" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>26/07/2026</t>
         </is>
       </c>
       <c r="S37" s="12" t="inlineStr">
         <is>
-          <t>FB2026-6023</t>
+          <t>507148</t>
         </is>
       </c>
       <c r="T37" s="12" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>84</t>
         </is>
       </c>
       <c r="U37" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin + eBay</t>
+          <t>Leboncoin, main propre</t>
         </is>
       </c>
       <c r="V37" s="4" t="inlineStr"/>
       <c r="W37" s="4" t="inlineStr">
         <is>
-          <t>Liquider</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="X37" s="4" t="inlineStr"/>
@@ -3853,113 +3846,109 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>LACOSTE sneakers P.42 — neuves</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="n">
-        <v>57.51</v>
-      </c>
-      <c r="C38" s="15">
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>Lot de 4 toupies BEYBLADE HASBRO</t>
+        </is>
+      </c>
+      <c r="B38" s="24" t="n">
+        <v>38.34</v>
+      </c>
+      <c r="C38" s="25">
         <f>$B38+$Y38*Paramètres!$B$13</f>
         <v/>
       </c>
-      <c r="D38" s="16">
+      <c r="D38" s="26">
         <f>$C38/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E38" s="15">
+      <c r="E38" s="25">
         <f>CEILING($D38*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F38" s="17" t="n">
-        <v>70</v>
-      </c>
-      <c r="G38" s="17">
+      <c r="F38" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="G38" s="27">
         <f>IF($F38="","",$F38-$C38-$M38-$N38)</f>
         <v/>
       </c>
-      <c r="H38" s="18">
+      <c r="H38" s="28">
         <f>IF($G38="","",$G38/$C38)</f>
         <v/>
       </c>
-      <c r="I38" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J38" s="15">
+      <c r="I38" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="J38" s="25">
         <f>$C38/$I38</f>
         <v/>
       </c>
-      <c r="K38" s="15">
+      <c r="K38" s="25">
         <f>IF($F38="","",$F38/$I38)</f>
         <v/>
       </c>
-      <c r="L38" s="15">
+      <c r="L38" s="25">
         <f>IF($G38="","",$G38/$I38)</f>
         <v/>
       </c>
-      <c r="M38" s="16">
+      <c r="M38" s="26">
         <f>IF($F38="","",$F38*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N38" s="15" t="n">
+      <c r="N38" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="O38" s="20" t="n">
-        <v>45</v>
-      </c>
-      <c r="P38" s="20" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="Q38" s="21" t="inlineStr">
-        <is>
-          <t>ADN Lyon</t>
-        </is>
-      </c>
-      <c r="R38" s="21" t="inlineStr">
+      <c r="O38" s="30" t="n">
+        <v>30</v>
+      </c>
+      <c r="P38" s="30" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="Q38" s="31" t="inlineStr">
+        <is>
+          <t>ADN Le Mans</t>
+        </is>
+      </c>
+      <c r="R38" s="31" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="S38" s="21" t="inlineStr">
-        <is>
-          <t>FB2026-6023</t>
-        </is>
-      </c>
-      <c r="T38" s="21" t="inlineStr">
-        <is>
-          <t>141</t>
-        </is>
-      </c>
-      <c r="U38" s="13" t="inlineStr">
-        <is>
-          <t>vendu</t>
-        </is>
-      </c>
-      <c r="V38" s="13" t="inlineStr"/>
-      <c r="W38" s="13" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="X38" s="13" t="inlineStr">
-        <is>
-          <t>VENDU</t>
-        </is>
-      </c>
-      <c r="Y38" s="13" t="n">
+      <c r="S38" s="31" t="inlineStr">
+        <is>
+          <t>FB2026-44192</t>
+        </is>
+      </c>
+      <c r="T38" s="31" t="inlineStr">
+        <is>
+          <t>299</t>
+        </is>
+      </c>
+      <c r="U38" s="23" t="inlineStr">
+        <is>
+          <t>Leboncoin + eBay, en lot</t>
+        </is>
+      </c>
+      <c r="V38" s="23" t="inlineStr"/>
+      <c r="W38" s="23" t="inlineStr">
+        <is>
+          <t>Marge faible</t>
+        </is>
+      </c>
+      <c r="X38" s="23" t="inlineStr"/>
+      <c r="Y38" s="23" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Pompe immergée ROBBY VP550W noir et bleu — produit d'occasion</t>
+          <t>Pompe immergée ROBBY VP550W noir/gris — comme neuf, SOCLE CASSÉ</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>35.9</v>
+        <v>28.29</v>
       </c>
       <c r="C39" s="6">
         <f>$B39</f>
@@ -3974,7 +3963,7 @@
         <v/>
       </c>
       <c r="F39" s="8" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="G39" s="8">
         <f>IF($F39="","",$F39-$C39-$M39-$N39)</f>
@@ -4025,7 +4014,7 @@
       </c>
       <c r="T39" s="12" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>122</t>
         </is>
       </c>
       <c r="U39" s="4" t="inlineStr">
@@ -4036,7 +4025,7 @@
       <c r="V39" s="4" t="inlineStr"/>
       <c r="W39" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Marge faible</t>
         </is>
       </c>
       <c r="X39" s="4" t="inlineStr"/>
@@ -4045,109 +4034,105 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="23" t="inlineStr">
-        <is>
-          <t>Lot de 4 toupies BEYBLADE HASBRO</t>
-        </is>
-      </c>
-      <c r="B40" s="24" t="n">
-        <v>38.34</v>
-      </c>
-      <c r="C40" s="25">
-        <f>$B40+$Y40*Paramètres!$B$13</f>
-        <v/>
-      </c>
-      <c r="D40" s="26">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>2 boosters Pokémon MEGA Storm Emeralda M6 — 5 cartes chacun — set sorti le 31/07/2026, publier vite</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>12.74</v>
+      </c>
+      <c r="C40" s="6">
+        <f>$B40</f>
+        <v/>
+      </c>
+      <c r="D40" s="7">
         <f>$C40/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E40" s="25">
+      <c r="E40" s="6">
         <f>CEILING($D40*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F40" s="27" t="n">
-        <v>49</v>
-      </c>
-      <c r="G40" s="27">
+      <c r="F40" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="G40" s="8">
         <f>IF($F40="","",$F40-$C40-$M40-$N40)</f>
         <v/>
       </c>
-      <c r="H40" s="28">
+      <c r="H40" s="9">
         <f>IF($G40="","",$G40/$C40)</f>
         <v/>
       </c>
-      <c r="I40" s="29" t="n">
-        <v>4</v>
-      </c>
-      <c r="J40" s="25">
+      <c r="I40" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="6">
         <f>$C40/$I40</f>
         <v/>
       </c>
-      <c r="K40" s="25">
+      <c r="K40" s="6">
         <f>IF($F40="","",$F40/$I40)</f>
         <v/>
       </c>
-      <c r="L40" s="25">
+      <c r="L40" s="6">
         <f>IF($G40="","",$G40/$I40)</f>
         <v/>
       </c>
-      <c r="M40" s="26">
+      <c r="M40" s="7">
         <f>IF($F40="","",$F40*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N40" s="25" t="n">
+      <c r="N40" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="O40" s="30" t="n">
-        <v>30</v>
-      </c>
-      <c r="P40" s="30" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="Q40" s="31" t="inlineStr">
-        <is>
-          <t>ADN Le Mans</t>
-        </is>
-      </c>
-      <c r="R40" s="31" t="inlineStr">
+      <c r="O40" s="22" t="n"/>
+      <c r="P40" s="22" t="n"/>
+      <c r="Q40" s="12" t="inlineStr">
+        <is>
+          <t>Meccha Japan</t>
+        </is>
+      </c>
+      <c r="R40" s="12" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="S40" s="31" t="inlineStr">
-        <is>
-          <t>FB2026-44192</t>
-        </is>
-      </c>
-      <c r="T40" s="31" t="inlineStr">
-        <is>
-          <t>299</t>
-        </is>
-      </c>
-      <c r="U40" s="23" t="inlineStr">
-        <is>
-          <t>Leboncoin + eBay, en lot</t>
-        </is>
-      </c>
-      <c r="V40" s="23" t="inlineStr"/>
-      <c r="W40" s="23" t="inlineStr">
-        <is>
-          <t>Marge faible</t>
-        </is>
-      </c>
-      <c r="X40" s="23" t="inlineStr"/>
-      <c r="Y40" s="23" t="n">
+      <c r="S40" s="12" t="inlineStr">
+        <is>
+          <t>#FA429713</t>
+        </is>
+      </c>
+      <c r="T40" s="12" t="inlineStr">
+        <is>
+          <t>4521329462226</t>
+        </is>
+      </c>
+      <c r="U40" s="4" t="inlineStr">
+        <is>
+          <t>Leboncoin, lot de 2</t>
+        </is>
+      </c>
+      <c r="V40" s="4" t="inlineStr"/>
+      <c r="W40" s="4" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="X40" s="4" t="inlineStr"/>
+      <c r="Y40" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Pompe immergée ROBBY VP550W noir/gris — comme neuf, SOCLE CASSÉ</t>
+          <t>1 booster Pokémon High Class Pack MEGA Dream ex M2a — 10 cartes dans le booster</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>28.29</v>
+        <v>12.95</v>
       </c>
       <c r="C41" s="6">
         <f>$B41</f>
@@ -4161,9 +4146,7 @@
         <f>CEILING($D41*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F41" s="8" t="n">
-        <v>35</v>
-      </c>
+      <c r="F41" s="22" t="n"/>
       <c r="G41" s="8">
         <f>IF($F41="","",$F41-$C41-$M41-$N41)</f>
         <v/>
@@ -4198,33 +4181,33 @@
       <c r="P41" s="22" t="n"/>
       <c r="Q41" s="12" t="inlineStr">
         <is>
-          <t>ERA Enchères Rhône-Alpes</t>
+          <t>Meccha Japan</t>
         </is>
       </c>
       <c r="R41" s="12" t="inlineStr">
         <is>
-          <t>26/07/2026</t>
+          <t>03/08/2026</t>
         </is>
       </c>
       <c r="S41" s="12" t="inlineStr">
         <is>
-          <t>507148</t>
+          <t>#FA429713</t>
         </is>
       </c>
       <c r="T41" s="12" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>4521329431925</t>
         </is>
       </c>
       <c r="U41" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin, main propre</t>
+          <t>Prélevé — usage personnel</t>
         </is>
       </c>
       <c r="V41" s="4" t="inlineStr"/>
       <c r="W41" s="4" t="inlineStr">
         <is>
-          <t>Marge faible</t>
+          <t>PRÉLEVÉ</t>
         </is>
       </c>
       <c r="X41" s="4" t="inlineStr"/>
@@ -4235,11 +4218,11 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>2 boosters Pokémon MEGA Storm Emeralda M6 — 5 cartes chacun — set sorti le 31/07/2026, publier vite</t>
+          <t>Pompe immergée ROBBY VP550W bleu et noir — occasion, NE MARCHE QU'EN MODE AUTO</t>
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>12.74</v>
+        <v>19.41</v>
       </c>
       <c r="C42" s="6">
         <f>$B42</f>
@@ -4253,9 +4236,7 @@
         <f>CEILING($D42*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F42" s="8" t="n">
-        <v>19</v>
-      </c>
+      <c r="F42" s="22" t="n"/>
       <c r="G42" s="8">
         <f>IF($F42="","",$F42-$C42-$M42-$N42)</f>
         <v/>
@@ -4290,33 +4271,33 @@
       <c r="P42" s="22" t="n"/>
       <c r="Q42" s="12" t="inlineStr">
         <is>
-          <t>Meccha Japan</t>
+          <t>ERA Enchères Rhône-Alpes</t>
         </is>
       </c>
       <c r="R42" s="12" t="inlineStr">
         <is>
-          <t>03/08/2026</t>
+          <t>26/07/2026</t>
         </is>
       </c>
       <c r="S42" s="12" t="inlineStr">
         <is>
-          <t>#FA429713</t>
+          <t>507148</t>
         </is>
       </c>
       <c r="T42" s="12" t="inlineStr">
         <is>
-          <t>4521329462226</t>
+          <t>131</t>
         </is>
       </c>
       <c r="U42" s="4" t="inlineStr">
         <is>
-          <t>Leboncoin, lot de 2</t>
+          <t>Prélevée — usage personnel</t>
         </is>
       </c>
       <c r="V42" s="4" t="inlineStr"/>
       <c r="W42" s="4" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>PRÉLEVÉE</t>
         </is>
       </c>
       <c r="X42" s="4" t="inlineStr"/>
@@ -4325,182 +4306,198 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>1 booster Pokémon High Class Pack MEGA Dream ex M2a — 10 cartes dans le booster</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="n">
-        <v>12.95</v>
-      </c>
-      <c r="C43" s="6">
-        <f>$B43</f>
-        <v/>
-      </c>
-      <c r="D43" s="7">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>Baskets NIKE Air Max Moto 2K P.44.5 — neuves</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="C43" s="15">
+        <f>$B43+$Y43*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D43" s="16">
         <f>$C43/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E43" s="6">
+      <c r="E43" s="15">
         <f>CEILING($D43*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F43" s="22" t="n"/>
-      <c r="G43" s="8">
+      <c r="F43" s="32" t="n"/>
+      <c r="G43" s="17">
         <f>IF($F43="","",$F43-$C43-$M43-$N43)</f>
         <v/>
       </c>
-      <c r="H43" s="9">
+      <c r="H43" s="18">
         <f>IF($G43="","",$G43/$C43)</f>
         <v/>
       </c>
-      <c r="I43" s="10" t="n">
+      <c r="I43" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J43" s="6">
+      <c r="J43" s="15">
         <f>$C43/$I43</f>
         <v/>
       </c>
-      <c r="K43" s="6">
+      <c r="K43" s="15">
         <f>IF($F43="","",$F43/$I43)</f>
         <v/>
       </c>
-      <c r="L43" s="6">
+      <c r="L43" s="15">
         <f>IF($G43="","",$G43/$I43)</f>
         <v/>
       </c>
-      <c r="M43" s="7">
+      <c r="M43" s="16">
         <f>IF($F43="","",$F43*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N43" s="6" t="n">
+      <c r="N43" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="O43" s="22" t="n"/>
-      <c r="P43" s="22" t="n"/>
-      <c r="Q43" s="12" t="inlineStr">
-        <is>
-          <t>Meccha Japan</t>
-        </is>
-      </c>
-      <c r="R43" s="12" t="inlineStr">
-        <is>
-          <t>03/08/2026</t>
-        </is>
-      </c>
-      <c r="S43" s="12" t="inlineStr">
-        <is>
-          <t>#FA429713</t>
-        </is>
-      </c>
-      <c r="T43" s="12" t="inlineStr">
-        <is>
-          <t>4521329431925</t>
-        </is>
-      </c>
-      <c r="U43" s="4" t="inlineStr">
-        <is>
-          <t>Prélevé — usage personnel</t>
-        </is>
-      </c>
-      <c r="V43" s="4" t="inlineStr"/>
-      <c r="W43" s="4" t="inlineStr">
-        <is>
-          <t>PRÉLEVÉ</t>
-        </is>
-      </c>
-      <c r="X43" s="4" t="inlineStr"/>
-      <c r="Y43" s="4" t="n">
+      <c r="O43" s="20" t="n">
+        <v>40</v>
+      </c>
+      <c r="P43" s="20" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="Q43" s="21" t="inlineStr">
+        <is>
+          <t>ADN Le Mans</t>
+        </is>
+      </c>
+      <c r="R43" s="21" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="S43" s="21" t="inlineStr">
+        <is>
+          <t>FB2026-43716</t>
+        </is>
+      </c>
+      <c r="T43" s="21" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="U43" s="13" t="inlineStr">
+        <is>
+          <t>Prélevées — usage personnel</t>
+        </is>
+      </c>
+      <c r="V43" s="13" t="inlineStr"/>
+      <c r="W43" s="13" t="inlineStr">
+        <is>
+          <t>PRÉLEVÉES</t>
+        </is>
+      </c>
+      <c r="X43" s="13" t="inlineStr">
+        <is>
+          <t>PRÉLEVÉES 09/08</t>
+        </is>
+      </c>
+      <c r="Y43" s="13" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Pompe immergée ROBBY VP550W bleu et noir — occasion, NE MARCHE QU'EN MODE AUTO</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="n">
-        <v>19.41</v>
-      </c>
-      <c r="C44" s="6">
-        <f>$B44</f>
-        <v/>
-      </c>
-      <c r="D44" s="7">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>Baskets HOKA P.37 1/3 — neuves</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="n">
+        <v>63</v>
+      </c>
+      <c r="C44" s="15">
+        <f>$B44+$Y44*Paramètres!$B$13</f>
+        <v/>
+      </c>
+      <c r="D44" s="16">
         <f>$C44/(1-Paramètres!$B$5-Paramètres!$B$6)</f>
         <v/>
       </c>
-      <c r="E44" s="6">
+      <c r="E44" s="15">
         <f>CEILING($D44*Paramètres!$B$24,1)</f>
         <v/>
       </c>
-      <c r="F44" s="22" t="n"/>
-      <c r="G44" s="8">
+      <c r="F44" s="32" t="n"/>
+      <c r="G44" s="17">
         <f>IF($F44="","",$F44-$C44-$M44-$N44)</f>
         <v/>
       </c>
-      <c r="H44" s="9">
+      <c r="H44" s="18">
         <f>IF($G44="","",$G44/$C44)</f>
         <v/>
       </c>
-      <c r="I44" s="10" t="n">
+      <c r="I44" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="J44" s="6">
+      <c r="J44" s="15">
         <f>$C44/$I44</f>
         <v/>
       </c>
-      <c r="K44" s="6">
+      <c r="K44" s="15">
         <f>IF($F44="","",$F44/$I44)</f>
         <v/>
       </c>
-      <c r="L44" s="6">
+      <c r="L44" s="15">
         <f>IF($G44="","",$G44/$I44)</f>
         <v/>
       </c>
-      <c r="M44" s="7">
+      <c r="M44" s="16">
         <f>IF($F44="","",$F44*(Paramètres!$B$5+Paramètres!$B$6))</f>
         <v/>
       </c>
-      <c r="N44" s="6" t="n">
+      <c r="N44" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="O44" s="22" t="n"/>
-      <c r="P44" s="22" t="n"/>
-      <c r="Q44" s="12" t="inlineStr">
-        <is>
-          <t>ERA Enchères Rhône-Alpes</t>
-        </is>
-      </c>
-      <c r="R44" s="12" t="inlineStr">
-        <is>
-          <t>26/07/2026</t>
-        </is>
-      </c>
-      <c r="S44" s="12" t="inlineStr">
-        <is>
-          <t>507148</t>
-        </is>
-      </c>
-      <c r="T44" s="12" t="inlineStr">
-        <is>
-          <t>131</t>
-        </is>
-      </c>
-      <c r="U44" s="4" t="inlineStr">
-        <is>
-          <t>Prélevée — usage personnel</t>
-        </is>
-      </c>
-      <c r="V44" s="4" t="inlineStr"/>
-      <c r="W44" s="4" t="inlineStr">
-        <is>
-          <t>PRÉLEVÉE</t>
-        </is>
-      </c>
-      <c r="X44" s="4" t="inlineStr"/>
-      <c r="Y44" s="4" t="n">
+      <c r="O44" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="P44" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q44" s="21" t="inlineStr">
+        <is>
+          <t>ADN Le Mans</t>
+        </is>
+      </c>
+      <c r="R44" s="21" t="inlineStr">
+        <is>
+          <t>28/07/2026</t>
+        </is>
+      </c>
+      <c r="S44" s="21" t="inlineStr">
+        <is>
+          <t>FB2026-43716</t>
+        </is>
+      </c>
+      <c r="T44" s="21" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="U44" s="13" t="inlineStr">
+        <is>
+          <t>Prélevées — usage personnel</t>
+        </is>
+      </c>
+      <c r="V44" s="13" t="inlineStr"/>
+      <c r="W44" s="13" t="inlineStr">
+        <is>
+          <t>PRÉLEVÉES</t>
+        </is>
+      </c>
+      <c r="X44" s="13" t="inlineStr">
+        <is>
+          <t>PRÉLEVÉES 09/08</t>
+        </is>
+      </c>
+      <c r="Y44" s="13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4599,59 +4596,59 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="32" t="inlineStr">
+      <c r="A46" s="33" t="inlineStr">
         <is>
           <t>TOTAL — 40 lots</t>
         </is>
       </c>
-      <c r="B46" s="33">
+      <c r="B46" s="34">
         <f>SUM(B6:B45)</f>
         <v/>
       </c>
-      <c r="C46" s="33">
+      <c r="C46" s="34">
         <f>SUM(C6:C45)</f>
         <v/>
       </c>
-      <c r="D46" s="34" t="n"/>
-      <c r="E46" s="34" t="n"/>
-      <c r="F46" s="33">
+      <c r="D46" s="35" t="n"/>
+      <c r="E46" s="35" t="n"/>
+      <c r="F46" s="34">
         <f>SUM(F6:F45)</f>
         <v/>
       </c>
-      <c r="G46" s="33">
+      <c r="G46" s="34">
         <f>SUM(G6:G45)</f>
         <v/>
       </c>
-      <c r="H46" s="35">
+      <c r="H46" s="36">
         <f>G46/C46</f>
         <v/>
       </c>
-      <c r="I46" s="36">
+      <c r="I46" s="37">
         <f>SUM(I6:I45)</f>
         <v/>
       </c>
-      <c r="J46" s="34" t="n"/>
-      <c r="K46" s="34" t="n"/>
-      <c r="L46" s="34" t="n"/>
-      <c r="M46" s="33">
+      <c r="J46" s="35" t="n"/>
+      <c r="K46" s="35" t="n"/>
+      <c r="L46" s="35" t="n"/>
+      <c r="M46" s="34">
         <f>SUM(M6:M45)</f>
         <v/>
       </c>
-      <c r="N46" s="33">
+      <c r="N46" s="34">
         <f>SUM(N6:N45)</f>
         <v/>
       </c>
-      <c r="O46" s="34" t="n"/>
-      <c r="P46" s="34" t="n"/>
-      <c r="Q46" s="34" t="n"/>
-      <c r="R46" s="34" t="n"/>
-      <c r="S46" s="34" t="n"/>
-      <c r="T46" s="34" t="n"/>
-      <c r="U46" s="34" t="n"/>
-      <c r="V46" s="34" t="n"/>
-      <c r="W46" s="34" t="n"/>
-      <c r="X46" s="34" t="n"/>
-      <c r="Y46" s="34" t="n"/>
+      <c r="O46" s="35" t="n"/>
+      <c r="P46" s="35" t="n"/>
+      <c r="Q46" s="35" t="n"/>
+      <c r="R46" s="35" t="n"/>
+      <c r="S46" s="35" t="n"/>
+      <c r="T46" s="35" t="n"/>
+      <c r="U46" s="35" t="n"/>
+      <c r="V46" s="35" t="n"/>
+      <c r="W46" s="35" t="n"/>
+      <c r="X46" s="35" t="n"/>
+      <c r="Y46" s="35" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:Y45"/>
@@ -4686,14 +4683,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="37" t="inlineStr">
+      <c r="A3" s="38" t="inlineStr">
         <is>
           <t>CAPITAL ENGAGÉ</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="38" t="inlineStr">
+      <c r="A4" s="39" t="inlineStr">
         <is>
           <t>Marchandise ADN</t>
         </is>
@@ -4703,7 +4700,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="39" t="inlineStr">
         <is>
           <t>Livraison ADN</t>
         </is>
@@ -4714,7 +4711,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="39" t="inlineStr">
         <is>
           <t>Achats hors ADN (pompes, Pokémon)</t>
         </is>
@@ -4724,25 +4721,25 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="40" t="inlineStr">
         <is>
           <t>TOTAL ENGAGÉ</t>
         </is>
       </c>
-      <c r="B7" s="33">
+      <c r="B7" s="34">
         <f>'Stock complet'!C46</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="37" t="inlineStr">
+      <c r="A9" s="38" t="inlineStr">
         <is>
           <t>CHIFFRE D'AFFAIRES ET MARGE</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="39" t="inlineStr">
+      <c r="A10" s="40" t="inlineStr">
         <is>
           <t>Chiffre d'affaires attendu</t>
         </is>
@@ -4758,7 +4755,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="38" t="inlineStr">
+      <c r="A11" s="39" t="inlineStr">
         <is>
           <t>− URSSAF + CFP</t>
         </is>
@@ -4769,7 +4766,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="38" t="inlineStr">
+      <c r="A12" s="39" t="inlineStr">
         <is>
           <t>− Commission carte</t>
         </is>
@@ -4780,17 +4777,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="39">
+      <c r="A13" s="40">
         <f> Marge brute</f>
         <v/>
       </c>
-      <c r="B13" s="33">
+      <c r="B13" s="34">
         <f>'Stock complet'!G46</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="38" t="inlineStr">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>− Emballage</t>
         </is>
@@ -4801,7 +4798,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="38" t="inlineStr">
+      <c r="A15" s="39" t="inlineStr">
         <is>
           <t>− Frais fixe carte</t>
         </is>
@@ -4812,17 +4809,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="39">
+      <c r="A16" s="40">
         <f> Marge avant impôt</f>
         <v/>
       </c>
-      <c r="B16" s="33">
+      <c r="B16" s="34">
         <f>B13+B14+B15</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="38" t="inlineStr">
+      <c r="A17" s="39" t="inlineStr">
         <is>
           <t>Base imposable</t>
         </is>
@@ -4833,7 +4830,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="38" t="inlineStr">
+      <c r="A18" s="39" t="inlineStr">
         <is>
           <t>− Impôt estimé</t>
         </is>
@@ -4844,81 +4841,81 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="39">
+      <c r="A19" s="40">
         <f> CE QUI RESTE</f>
         <v/>
       </c>
-      <c r="B19" s="40">
+      <c r="B19" s="41">
         <f>B16+B18</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="37" t="inlineStr">
+      <c r="A21" s="38" t="inlineStr">
         <is>
           <t>RENDEMENT</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="38" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>Marge nette / capital engagé</t>
         </is>
       </c>
-      <c r="B22" s="41">
+      <c r="B22" s="42">
         <f>B19/B7</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="38" t="inlineStr">
+      <c r="A23" s="39" t="inlineStr">
         <is>
           <t>Articles physiques</t>
         </is>
       </c>
-      <c r="B23" s="42">
+      <c r="B23" s="43">
         <f>'Stock complet'!I46</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="37" t="inlineStr">
+      <c r="A25" s="38" t="inlineStr">
         <is>
           <t>À FAIRE</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="38" t="inlineStr">
+      <c r="A26" s="39" t="inlineStr">
         <is>
           <t>1 lot sans prix : Yeezy 700 V3, en attente d'authentification.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="38" t="inlineStr">
-        <is>
-          <t>Ventes du 09/08 et du 10/08/2026 : espèces, main propre. Nom de l'acheteur à noter.</t>
+      <c r="A27" s="44" t="inlineStr">
+        <is>
+          <t>CA encaissé : 343 €, pas 493 €. Les Hoka et les Nike sont des prélèvements, pas des ventes.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="38" t="inlineStr">
-        <is>
-          <t>Factures annoncées : lot n°84 (3 pompes Robby) et boîte de 30 boosters Pokémon.</t>
+      <c r="A28" s="39" t="inlineStr">
+        <is>
+          <t>Toutes les factures sont reçues. 150,50 € de stock prélevé pour usage personnel.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="43" t="inlineStr">
+      <c r="A29" s="44" t="inlineStr">
         <is>
           <t>SEUIL D'ÉQUILIBRE : ne jamais vendre en dessous, la vente coûterait de l'argent.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="38" t="inlineStr">
+      <c r="A30" s="39" t="inlineStr">
         <is>
           <t>PRIX PLANCHER : 30 % au-dessus du seuil. Le plus bas acceptable, famille comprise.</t>
         </is>
@@ -4965,19 +4962,19 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="37" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
         <is>
           <t>CHARGES SUR LE CHIFFRE D'AFFAIRES</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="38" t="inlineStr">
+      <c r="A5" s="39" t="inlineStr">
         <is>
           <t>Cotisations URSSAF (achat-revente BIC)</t>
         </is>
       </c>
-      <c r="B5" s="44" t="n">
+      <c r="B5" s="45" t="n">
         <v>0.123</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -4987,22 +4984,22 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="38" t="inlineStr">
+      <c r="A6" s="39" t="inlineStr">
         <is>
           <t>CFP — formation professionnelle</t>
         </is>
       </c>
-      <c r="B6" s="44" t="n">
+      <c r="B6" s="45" t="n">
         <v>0.001</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="38" t="inlineStr">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>Commission carte Shopify Payments</t>
         </is>
       </c>
-      <c r="B7" s="44" t="n">
+      <c r="B7" s="45" t="n">
         <v>0.015</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -5012,24 +5009,24 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="38" t="inlineStr">
+      <c r="A8" s="39" t="inlineStr">
         <is>
           <t>Frais fixe par transaction carte</t>
         </is>
       </c>
-      <c r="B8" s="45" t="n">
+      <c r="B8" s="46" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="37" t="inlineStr">
+      <c r="A10" s="38" t="inlineStr">
         <is>
           <t>LIVRAISON DES LOTS</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="38" t="inlineStr">
+      <c r="A11" s="39" t="inlineStr">
         <is>
           <t>Total des factures de livraison ADN</t>
         </is>
@@ -5044,7 +5041,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="38" t="inlineStr">
+      <c r="A12" s="39" t="inlineStr">
         <is>
           <t>Unités de vente reçues d'ADN</t>
         </is>
@@ -5059,7 +5056,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="38" t="inlineStr">
+      <c r="A13" s="39" t="inlineStr">
         <is>
           <t>Livraison par unité de vente</t>
         </is>
@@ -5075,19 +5072,19 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="37" t="inlineStr">
+      <c r="A15" s="38" t="inlineStr">
         <is>
           <t>IMPÔT SUR LE REVENU — MICRO-BIC</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="38" t="inlineStr">
+      <c r="A16" s="39" t="inlineStr">
         <is>
           <t>Abattement forfaitaire</t>
         </is>
       </c>
-      <c r="B16" s="44" t="n">
+      <c r="B16" s="45" t="n">
         <v>0.71</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -5097,12 +5094,12 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="38" t="inlineStr">
+      <c r="A17" s="39" t="inlineStr">
         <is>
           <t>Tranche marginale du foyer</t>
         </is>
       </c>
-      <c r="B17" s="44" t="n">
+      <c r="B17" s="45" t="n">
         <v>0.11</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -5112,46 +5109,46 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="37" t="inlineStr">
+      <c r="A19" s="38" t="inlineStr">
         <is>
           <t>FRAIS DE VENTE</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="38" t="inlineStr">
+      <c r="A20" s="39" t="inlineStr">
         <is>
           <t>Emballage par colis</t>
         </is>
       </c>
-      <c r="B20" s="45" t="n">
+      <c r="B20" s="46" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="38" t="inlineStr">
+      <c r="A21" s="39" t="inlineStr">
         <is>
           <t>Nombre d'annonces prévues</t>
         </is>
       </c>
-      <c r="B21" s="46" t="n">
+      <c r="B21" s="47" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="37" t="inlineStr">
+      <c r="A23" s="38" t="inlineStr">
         <is>
           <t>PLANCHER DE NÉGOCIATION</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="38" t="inlineStr">
+      <c r="A24" s="39" t="inlineStr">
         <is>
           <t>Coefficient sur le seuil d'équilibre</t>
         </is>
       </c>
-      <c r="B24" s="47" t="n">
+      <c r="B24" s="48" t="n">
         <v>1.3</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -6749,67 +6746,67 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="34" t="n"/>
-      <c r="B39" s="34" t="n"/>
-      <c r="C39" s="34" t="n"/>
-      <c r="D39" s="34" t="n"/>
-      <c r="E39" s="34" t="n"/>
-      <c r="F39" s="32" t="inlineStr">
+      <c r="A39" s="35" t="n"/>
+      <c r="B39" s="35" t="n"/>
+      <c r="C39" s="35" t="n"/>
+      <c r="D39" s="35" t="n"/>
+      <c r="E39" s="35" t="n"/>
+      <c r="F39" s="33" t="inlineStr">
         <is>
           <t>TOTAL MARCHANDISE</t>
         </is>
       </c>
-      <c r="G39" s="33">
+      <c r="G39" s="34">
         <f>SUM(G5:G38)</f>
         <v/>
       </c>
-      <c r="H39" s="33">
+      <c r="H39" s="34">
         <f>SUM(H5:H38)</f>
         <v/>
       </c>
-      <c r="I39" s="33">
+      <c r="I39" s="34">
         <f>SUM(I5:I38)</f>
         <v/>
       </c>
-      <c r="J39" s="33">
+      <c r="J39" s="34">
         <f>SUM(J5:J38)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="37" t="inlineStr">
+      <c r="A41" s="38" t="inlineStr">
         <is>
           <t>FACTURES DE LIVRAISON</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="48" t="inlineStr">
+      <c r="A42" s="49" t="inlineStr">
         <is>
           <t>Facture</t>
         </is>
       </c>
-      <c r="B42" s="48" t="inlineStr">
+      <c r="B42" s="49" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C42" s="48" t="inlineStr">
+      <c r="C42" s="49" t="inlineStr">
         <is>
           <t>Maison</t>
         </is>
       </c>
-      <c r="D42" s="48" t="inlineStr">
+      <c r="D42" s="49" t="inlineStr">
         <is>
           <t>Commande</t>
         </is>
       </c>
-      <c r="E42" s="48" t="inlineStr">
+      <c r="E42" s="49" t="inlineStr">
         <is>
           <t>Désignation</t>
         </is>
       </c>
-      <c r="F42" s="48" t="inlineStr">
+      <c r="F42" s="49" t="inlineStr">
         <is>
           <t>Total TTC</t>
         </is>
@@ -6966,16 +6963,16 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="34" t="n"/>
-      <c r="B48" s="34" t="n"/>
-      <c r="C48" s="34" t="n"/>
-      <c r="D48" s="34" t="n"/>
-      <c r="E48" s="32" t="inlineStr">
+      <c r="A48" s="35" t="n"/>
+      <c r="B48" s="35" t="n"/>
+      <c r="C48" s="35" t="n"/>
+      <c r="D48" s="35" t="n"/>
+      <c r="E48" s="33" t="inlineStr">
         <is>
           <t>TOTAL LIVRAISON</t>
         </is>
       </c>
-      <c r="F48" s="33">
+      <c r="F48" s="34">
         <f>SUM(F43:F47)</f>
         <v/>
       </c>

</xml_diff>